<commit_message>
Wave 14 v3: add consolidated up-and-coming tab
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TE8a9ptd2NGPUtY6iZfzkb
</commit_message>
<xml_diff>
--- a/reports/F1-Wave14-V3-Broad-2026-10.xlsx
+++ b/reports/F1-Wave14-V3-Broad-2026-10.xlsx
@@ -8,34 +8,36 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 READ ME" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Food &amp; Beverage" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="42 Health &amp; Wellness" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="53 Consumer &amp; Lifestyle" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X02 Real Estate &amp; Building Prod" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X04 Mining, Metals &amp; Commoditie" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X05 Agriculture &amp; AgTech" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X06 Retail &amp; E-commerce" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X09 Maritime, Shipping &amp; Ports" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X10 Batteries, EV, Waste &amp; Wate" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X14 Intralogistics &amp; Warehouse " sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X16 Specialty Chemicals &amp; Coati" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X17 Private 5G &amp; Telecom Equipm" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="98 PENDING" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="99 REJECTS" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 UP-AND-COMING (all)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Food &amp; Beverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="42 Health &amp; Wellness" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="53 Consumer &amp; Lifestyle" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X02 Real Estate &amp; Building Prod" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X04 Mining, Metals &amp; Commoditie" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X05 Agriculture &amp; AgTech" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X06 Retail &amp; E-commerce" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X09 Maritime, Shipping &amp; Ports" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X10 Batteries, EV, Waste &amp; Wate" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X14 Intralogistics &amp; Warehouse " sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X16 Specialty Chemicals &amp; Coati" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X17 Private 5G &amp; Telecom Equipm" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="98 PENDING" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="99 REJECTS" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'04 Food &amp; Beverage'!$A$3:$T$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'42 Health &amp; Wellness'!$A$3:$T$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'53 Consumer &amp; Lifestyle'!$A$3:$T$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'X02 Real Estate &amp; Building Prod'!$A$3:$T$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'X04 Mining, Metals &amp; Commoditie'!$A$3:$T$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'X05 Agriculture &amp; AgTech'!$A$3:$T$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'X06 Retail &amp; E-commerce'!$A$3:$T$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'X09 Maritime, Shipping &amp; Ports'!$A$3:$T$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'X10 Batteries, EV, Waste &amp; Wate'!$A$3:$T$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'X14 Intralogistics &amp; Warehouse '!$A$3:$T$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'X16 Specialty Chemicals &amp; Coati'!$A$3:$T$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'X17 Private 5G &amp; Telecom Equipm'!$A$3:$T$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01 UP-AND-COMING (all)'!$A$3:$T$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'04 Food &amp; Beverage'!$A$3:$T$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'42 Health &amp; Wellness'!$A$3:$T$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'53 Consumer &amp; Lifestyle'!$A$3:$T$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'X02 Real Estate &amp; Building Prod'!$A$3:$T$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'X04 Mining, Metals &amp; Commoditie'!$A$3:$T$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'X05 Agriculture &amp; AgTech'!$A$3:$T$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'X06 Retail &amp; E-commerce'!$A$3:$T$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'X09 Maritime, Shipping &amp; Ports'!$A$3:$T$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'X10 Batteries, EV, Waste &amp; Wate'!$A$3:$T$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'X14 Intralogistics &amp; Warehouse '!$A$3:$T$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'X16 Specialty Chemicals &amp; Coati'!$A$3:$T$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'X17 Private 5G &amp; Telecom Equipm'!$A$3:$T$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -893,7 +895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:T5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -921,7 +923,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>X10 Batteries, EV, Waste &amp; Water — Wave 14 (v3) — 1 new brands: 0 Yes / 1 Stretch / 0 Low-value</t>
+          <t>X09 Maritime, Shipping &amp; Ports — Wave 14 (v3) — 2 new brands: 0 Yes / 0 Stretch / 2 Low-value</t>
         </is>
       </c>
     </row>
@@ -1035,103 +1037,199 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="n">
+      <c r="A4" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="9" t="n">
-        <v>64</v>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>Envision AESC</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>X10 Batteries, EV, Waste &amp; Water</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="B4" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Frontline plc</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>X09 Maritime, Shipping &amp; Ports</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>aesc-group.com</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>Yokohama, Japan (global ops: UK, France, Spain, US, China)</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>Private; Envision Group majority; investors GIC, Primavera/HongShan, HSG, Nissan, NEC; HK IPO under consideration</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="inlineStr">
-        <is>
-          <t>EV and energy-storage lithium-ion batteries for Nissan, Renault, BMW, Mercedes-Benz, GM; 14 production bases planned or operating</t>
-        </is>
-      </c>
-      <c r="J4" s="9" t="inlineStr">
-        <is>
-          <t>1k-5k</t>
-        </is>
-      </c>
-      <c r="K4" s="9" t="inlineStr">
-        <is>
-          <t>Not found in searches (revenue unknown)</t>
-        </is>
-      </c>
-      <c r="L4" s="9" t="inlineStr">
-        <is>
-          <t>Reported target ~$10B in Series C (Bloomberg, 24 Nov 2023, target not confirmed closed); total funding $2.38B (Tracxn/PitchBook, 2026); considering HK IPO raising $1-2B (Bloomberg, 17 Apr 2026)</t>
-        </is>
-      </c>
-      <c r="M4" s="9" t="inlineStr">
-        <is>
-          <t>$1.38B project financing, May 2025 (PitchBook/Tracxn); IPO of $1-2B being considered, 2026</t>
-        </is>
-      </c>
-      <c r="N4" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="O4" s="9" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>frontline.bm</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Limassol, Cyprus</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>Public (NYSE/Oslo: FRO); controlled by John Fredriksen</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>Crude and product tanker transportation, 77-vessel fleet (40 VLCC, 19 Suezmax, 18 Aframax/LR2) chartered to oil majors and traders</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>51-200</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>Q2 2026 profit $659.2M, best-ever quarter, record TCE rates (Q2 2026 call, 28 Aug 2026)</t>
+        </is>
+      </c>
+      <c r="L4" s="10" t="inlineStr">
+        <is>
+          <t>Market cap ~USD 11.45B per StockAnalysis Q2 2026 listing; NOK 76.9B (~USD 7.5B est) at 30 Jun 2026; 85 employees</t>
+        </is>
+      </c>
+      <c r="M4" s="10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N4" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="O4" s="10" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="P4" s="9" t="inlineStr">
-        <is>
-          <t>Stretch</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Passes hard filters (reported ~$10B valuation target, ~1,870 employees Mar 2026, well funded, no F1 team or global partner tie; Envision Racing is Formula E only, not F1). Reservation: no published, confirmed valuation and the US plant pause. Marketing motive (pre-IPO awareness, parent already in motorsport) is credible. Prior concentration rejection is now a flag only.</t>
-        </is>
-      </c>
-      <c r="R4" s="9" t="inlineStr">
-        <is>
-          <t>Pre-IPO global brand-building: technology partnership around F1 2026 hybrid and electrification narrative, leveraging Envision Group's existing motorsport appetite (est); Silverstone or Suzuka GP for OEM and investor hospitality.</t>
-        </is>
-      </c>
-      <c r="S4" s="9" t="inlineStr">
-        <is>
-          <t>valuation is a reported 2023 target, unconfirmed; customer concentration (few OEMs); US plant paused Jun 2025 (Florence SC, $1.6B project); revenue unknown; Chinese-linked parent (Envision Group), US political risk; pre-IPO</t>
-        </is>
-      </c>
-      <c r="T4" s="9" t="inlineStr">
-        <is>
-          <t>Markets 1 (Japan, UK, France, Spain, US, China). Buyers 1 (OEM senior decision makers). Story 1 (high-performance battery technology, global ambition). Category 1 (batteries not on grid; sister team Envision Racing is in Formula E, not F1).</t>
+      <c r="P4" s="10" t="inlineStr">
+        <is>
+          <t>Low-value</t>
+        </is>
+      </c>
+      <c r="Q4" s="10" t="inlineStr">
+        <is>
+          <t>Passes hard filters (large market cap, 85 staff within 51+, record profit, no F1 tie found, not sanctioned per search). But it is a pure B2B tanker owner with concentrated counterparties, minimal marketing function and no brand ambition; fit 2.</t>
+        </is>
+      </c>
+      <c r="R4" s="10" t="inlineStr">
+        <is>
+          <t>Monaco or Abu Dhabi GP entertainment for charterer executives (est); very low odds as Frontline does not advertise.</t>
+        </is>
+      </c>
+      <c r="S4" s="10" t="inlineStr">
+        <is>
+          <t>concentrated customers (oil majors and trading houses); cyclical earnings at record high; pure B2B; controlled by single billionaire</t>
+        </is>
+      </c>
+      <c r="T4" s="10" t="inlineStr">
+        <is>
+          <t>Markets 0 (B2B shipping, not sold to consumers). Buyers 1 (oil major executives). Story 0. Category 1 (tankers not on grid).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Seaspan (Atlas Corp.)</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>X09 Maritime, Shipping &amp; Ports</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>seaspancorp.com</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Hong Kong / Vancouver, Canada (Atlas, Poseidon-owned)</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>Private since 2023: Poseidon consortium (Washington family, Fairfax, Ocean Network Express, David Sokol); Fairfax sold 23.2% of Poseidon for $1.91B in Mar 2026</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>Container ships on long-term charter (180+ vessels, ~9 liner customers) and marine services through Seaspan ULC</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>5k-10k</t>
+        </is>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>Atlas 2024 revenue $2,300.1M (Atlas 20-F, Mar 2025)</t>
+        </is>
+      </c>
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>Take-private EV ~$10.9B (2023, Seatrade); Poseidon equity ~USD 8.2B est (Fairfax sale at $28.30/sh for 23.2%, Mar 2026)</t>
+        </is>
+      </c>
+      <c r="M5" s="10" t="inlineStr">
+        <is>
+          <t>Mar 2026 secondary: Fairfax sold 67.6M Poseidon shares for $1.91B (The Insurer)</t>
+        </is>
+      </c>
+      <c r="N5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" s="10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="P5" s="10" t="inlineStr">
+        <is>
+          <t>Low-value</t>
+        </is>
+      </c>
+      <c r="Q5" s="10" t="inlineStr">
+        <is>
+          <t>Passes hard filters (EV $10.9B, ~6,200 staff, $2.3B revenue, no F1 tie found for Seaspan, Atlas, Poseidon or ONE). But it is a pure B2B ship-lessor with nine customers and no brand ambition; fit 1. Prior concentration rejection is now a flag only.</t>
+        </is>
+      </c>
+      <c r="R5" s="10" t="inlineStr">
+        <is>
+          <t>None credible; at most Canadian GP (Montreal) charterer hospitality (est). Not worth outreach effort.</t>
+        </is>
+      </c>
+      <c r="S5" s="10" t="inlineStr">
+        <is>
+          <t>concentrated customers (nine liner companies); pure B2B; partial ownership change Mar 2026 (secondary stake sale)</t>
+        </is>
+      </c>
+      <c r="T5" s="10" t="inlineStr">
+        <is>
+          <t>Markets 0 (B2B charter). Buyers 0. Story 0-1. Category 1. Scored 1.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:T4"/>
+  <autoFilter ref="A3:T5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1170,7 +1268,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>X14 Intralogistics &amp; Warehouse A — Wave 14 (v3) — 1 new brands: 0 Yes / 1 Stretch / 0 Low-value</t>
+          <t>X10 Batteries, EV, Waste &amp; Water — Wave 14 (v3) — 1 new brands: 0 Yes / 1 Stretch / 0 Low-value</t>
         </is>
       </c>
     </row>
@@ -1292,12 +1390,12 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>ContiTech (Continental)</t>
+          <t>Envision AESC</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>X14 Intralogistics &amp; Warehouse A</t>
+          <t>X10 Batteries, EV, Waste &amp; Water</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -1307,42 +1405,42 @@
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>continental.com/contitech</t>
+          <t>aesc-group.com</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>Hanover, Germany</t>
+          <t>Yokohama, Japan (global ops: UK, France, Spain, US, China)</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>Subsidiary of Continental AG (listed); sale to Lone Star Funds signed 2026, closing expected by end 2026 (PE incoming)</t>
+          <t>Private; Envision Group majority; investors GIC, Primavera/HongShan, HSG, Nissan, NEC; HK IPO under consideration</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>Industrial rubber and plastics technology: hoses, conveyor belts, surface materials, air springs, industrial fluid solutions; global B2B/OEM and aftermarket</t>
+          <t>EV and energy-storage lithium-ion batteries for Nissan, Renault, BMW, Mercedes-Benz, GM; 14 production bases planned or operating</t>
         </is>
       </c>
       <c r="J4" s="9" t="inlineStr">
         <is>
-          <t>10k+</t>
+          <t>1k-5k</t>
         </is>
       </c>
       <c r="K4" s="9" t="inlineStr">
         <is>
-          <t>FY2025 sales EUR 4.4B (Continental press release / Yahoo Finance, 2026)</t>
+          <t>Not found in searches (revenue unknown)</t>
         </is>
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>EUR 4.0B enterprise value agreed in sale to Lone Star plus up to EUR 250M earn-out (Continental ad-hoc release, 2026); ~0.9x FY2025 sales</t>
+          <t>Reported target ~$10B in Series C (Bloomberg, 24 Nov 2023, target not confirmed closed); total funding $2.38B (Tracxn/PitchBook, 2026); considering HK IPO raising $1-2B (Bloomberg, 17 Apr 2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>None; carve-out sale to Lone Star Funds 2026 (~EUR 3.1B cash proceeds to Continental)</t>
+          <t>$1.38B project financing, May 2025 (PitchBook/Tracxn); IPO of $1-2B being considered, 2026</t>
         </is>
       </c>
       <c r="N4" s="9" t="n">
@@ -1360,22 +1458,22 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Passes all hard filters: EV EUR 4.0B (2026), ~22,000 staff, FY2025 sales EUR 4.4B; divestiture is a portfolio decision, not distress (Continental Q2 2026 margins up per Investing.com). No F1 tie: Continental left F1 in 1955; Pirelli is sole tyre supplier; Continental only in Extreme E and a Rosberg ambassador deal (search 5 Oct 2026). Single reservation: ownership is changing now (Lone Star), so sponsorship budget authority and brand identity are unsettled until close.</t>
+          <t>Passes hard filters (reported ~$10B valuation target, ~1,870 employees Mar 2026, well funded, no F1 team or global partner tie; Envision Racing is Formula E only, not F1). Reservation: no published, confirmed valuation and the US plant pause. Marketing motive (pre-IPO awareness, parent already in motorsport) is credible. Prior concentration rejection is now a flag only.</t>
         </is>
       </c>
       <c r="R4" s="9" t="inlineStr">
         <is>
-          <t>Approach after Lone Star close (est Q4 2026-Q1 2027) with a global brand-launch platform: F1 technical-precision story (hoses/fluid systems in motorsport) for a new standalone ContiTech brand.</t>
+          <t>Pre-IPO global brand-building: technology partnership around F1 2026 hybrid and electrification narrative, leveraging Envision Group's existing motorsport appetite (est); Silverstone or Suzuka GP for OEM and investor hospitality.</t>
         </is>
       </c>
       <c r="S4" s="9" t="inlineStr">
         <is>
-          <t>recent ownership change (sale signed 2026, pending close); PE ownership incoming; brand may be separated from Continental parent; pure B2B</t>
+          <t>valuation is a reported 2023 target, unconfirmed; customer concentration (few OEMs); US plant paused Jun 2025 (Florence SC, $1.6B project); revenue unknown; Chinese-linked parent (Envision Group), US political risk; pre-IPO</t>
         </is>
       </c>
       <c r="T4" s="9" t="inlineStr">
         <is>
-          <t>Markets 1 (global, incl. Germany, Italy, Spain, UK, US, Japan, China); buyers 1 (B2B decision makers); story 1 (engineering/precision materials); category free 1 (industrial rubber not on grid; tyres are Pirelli's, not ContiTech)</t>
+          <t>Markets 1 (Japan, UK, France, Spain, US, China). Buyers 1 (OEM senior decision makers). Story 1 (high-performance battery technology, global ambition). Category 1 (batteries not on grid; sister team Envision Racing is in Formula E, not F1).</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1517,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>X16 Specialty Chemicals &amp; Coatin — Wave 14 (v3) — 1 new brands: 0 Yes / 1 Stretch / 0 Low-value</t>
+          <t>X14 Intralogistics &amp; Warehouse A — Wave 14 (v3) — 1 new brands: 0 Yes / 1 Stretch / 0 Low-value</t>
         </is>
       </c>
     </row>
@@ -1537,16 +1635,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="9" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Ingevity Corporation</t>
+          <t>ContiTech (Continental)</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>X16 Specialty Chemicals &amp; Coatin</t>
+          <t>X14 Intralogistics &amp; Warehouse A</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -1556,46 +1654,46 @@
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>ingevity.com</t>
+          <t>continental.com/contitech</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>North Charleston, South Carolina, USA</t>
+          <t>Hanover, Germany</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>Publicly listed (NYSE: NGVT); no controlling holder</t>
+          <t>Subsidiary of Continental AG (listed); sale to Lone Star Funds signed 2026, closing expected by end 2026 (PE incoming)</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>Performance Materials (activated carbon for automotive emissions) and Pavement Technologies (asphalt additives); customers automakers/Tier 1s and road builders; global, incl. US, Europe, Asia</t>
+          <t>Industrial rubber and plastics technology: hoses, conveyor belts, surface materials, air springs, industrial fluid solutions; global B2B/OEM and aftermarket</t>
         </is>
       </c>
       <c r="J4" s="9" t="inlineStr">
         <is>
-          <t>1k-5k</t>
+          <t>10k+</t>
         </is>
       </c>
       <c r="K4" s="9" t="inlineStr">
         <is>
-          <t>FY2025 net sales ~$1.3B total, $1.2B continuing; FY2026 guidance $1.05-1.15B (Q2 2026 release); adj EBITDA guidance $380-400M</t>
+          <t>FY2025 sales EUR 4.4B (Continental press release / Yahoo Finance, 2026)</t>
         </is>
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Market cap ~$2.63B (Q1 2026, Simply Wall St / SEC-linked data)</t>
+          <t>EUR 4.0B enterprise value agreed in sale to Lone Star plus up to EUR 250M earn-out (Continental ad-hoc release, 2026); ~0.9x FY2025 sales</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>None (listed; net leverage 2.5x per Q2 2026 call)</t>
+          <t>None; carve-out sale to Lone Star Funds 2026 (~EUR 3.1B cash proceeds to Continental)</t>
         </is>
       </c>
       <c r="N4" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O4" s="9" t="inlineStr">
         <is>
@@ -1609,22 +1707,22 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Passes hard filters: market cap ~$2.63B (Q1 2026), ~1,400 staff, no F1 tie found (search 5 Oct 2026). Capacity holds: FY2025 loss of $167.1M was non-cash impairment ($183.8M goodwill) while adj EBITDA was $397.5M, Q2 2026 adj EBITDA up 14% at 36.6% margin, FCF guide $220-245M. Divestitures (Industrial Specialties Jan 2026, Road Markings Apr 2026) are portfolio pruning, not distress. Reservation: low-profile B2B with weak marketing motive, fit 3 with category partly taken.</t>
+          <t>Passes all hard filters: EV EUR 4.0B (2026), ~22,000 staff, FY2025 sales EUR 4.4B; divestiture is a portfolio decision, not distress (Continental Q2 2026 margins up per Investing.com). No F1 tie: Continental left F1 in 1955; Pirelli is sole tyre supplier; Continental only in Extreme E and a Rosberg ambassador deal (search 5 Oct 2026). Single reservation: ownership is changing now (Lone Star), so sponsorship budget authority and brand identity are unsettled until close.</t>
         </is>
       </c>
       <c r="R4" s="9" t="inlineStr">
         <is>
-          <t>B2B hospitality for automotive-OEM and Tier 1 buyers: position carbon-canister emissions technology around F1 hybrid/sustainable-fuel narrative at a European or US race.</t>
+          <t>Approach after Lone Star close (est Q4 2026-Q1 2027) with a global brand-launch platform: F1 technical-precision story (hoses/fluid systems in motorsport) for a new standalone ContiTech brand.</t>
         </is>
       </c>
       <c r="S4" s="9" t="inlineStr">
         <is>
-          <t>customers likely concentrated (automotive Tier 1s; not verified at &lt;=20); pure B2B low consumer profile; FY2025 net loss $167M driven by $293M non-cash impairments; portfolio divestitures 2026</t>
+          <t>recent ownership change (sale signed 2026, pending close); PE ownership incoming; brand may be separated from Continental parent; pure B2B</t>
         </is>
       </c>
       <c r="T4" s="9" t="inlineStr">
         <is>
-          <t>Markets 1; buyers 1 (B2B decision makers); story 1 (materials technology/emissions performance); category free 0 (energy/chemicals/lubricants heavily represented on grid)</t>
+          <t>Markets 1 (global, incl. Germany, Italy, Spain, UK, US, Japan, China); buyers 1 (B2B decision makers); story 1 (engineering/precision materials); category free 1 (industrial rubber not on grid; tyres are Pirelli's, not ContiTech)</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1766,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>X17 Private 5G &amp; Telecom Equipme — Wave 14 (v3) — 1 new brands: 0 Yes / 0 Stretch / 1 Low-value</t>
+          <t>X16 Specialty Chemicals &amp; Coatin — Wave 14 (v3) — 1 new brands: 0 Yes / 1 Stretch / 0 Low-value</t>
         </is>
       </c>
     </row>
@@ -1782,98 +1880,98 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="n">
+      <c r="A4" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="10" t="n">
-        <v>32</v>
-      </c>
-      <c r="C4" s="10" t="inlineStr">
-        <is>
-          <t>Vantage Towers</t>
-        </is>
-      </c>
-      <c r="D4" s="10" t="inlineStr">
-        <is>
-          <t>X17 Private 5G &amp; Telecom Equipme</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="B4" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Ingevity Corporation</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>X16 Specialty Chemicals &amp; Coatin</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>vantagetowers.com</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="inlineStr">
-        <is>
-          <t>Dusseldorf, Germany</t>
-        </is>
-      </c>
-      <c r="H4" s="10" t="inlineStr">
-        <is>
-          <t>Oak Holdings (50:50 Vodafone and KKR/GIP) holds ~89%; remainder free float (OTC)</t>
-        </is>
-      </c>
-      <c r="I4" s="10" t="inlineStr">
-        <is>
-          <t>Wireless tower infrastructure leased to mobile network operators across 10 European countries (87,824 sites, Mar 2025); no consumer sales</t>
-        </is>
-      </c>
-      <c r="J4" s="10" t="inlineStr">
-        <is>
-          <t>201-1k</t>
-        </is>
-      </c>
-      <c r="K4" s="10" t="inlineStr">
-        <is>
-          <t>FY2024/25 revenue EUR 665.9M (company filings, Mar 2025)</t>
-        </is>
-      </c>
-      <c r="L4" s="10" t="inlineStr">
-        <is>
-          <t>Equity value EUR 16.2B in the KKR/GIP transaction (announced Nov 2022, EUR 32/share, stale; same price for Vodafone's 10% sale at EUR 1.3B)</t>
-        </is>
-      </c>
-      <c r="M4" s="10" t="inlineStr">
-        <is>
-          <t>None; Vodafone sold further 10% for EUR 1.3B (2026 report, DCD) completing 50:50 JV</t>
-        </is>
-      </c>
-      <c r="N4" s="10" t="n">
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>ingevity.com</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>North Charleston, South Carolina, USA</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>Publicly listed (NYSE: NGVT); no controlling holder</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>Performance Materials (activated carbon for automotive emissions) and Pavement Technologies (asphalt additives); customers automakers/Tier 1s and road builders; global, incl. US, Europe, Asia</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>FY2025 net sales ~$1.3B total, $1.2B continuing; FY2026 guidance $1.05-1.15B (Q2 2026 release); adj EBITDA guidance $380-400M</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>Market cap ~$2.63B (Q1 2026, Simply Wall St / SEC-linked data)</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>None (listed; net leverage 2.5x per Q2 2026 call)</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="10" t="inlineStr">
+      <c r="O4" s="9" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="P4" s="10" t="inlineStr">
-        <is>
-          <t>Low-value</t>
-        </is>
-      </c>
-      <c r="Q4" s="10" t="inlineStr">
-        <is>
-          <t>Passes hard filters: EV/equity EUR 16.2B (Nov 2022 deal, dated), ~883 avg staff (Oak Group, Mar 2025), healthy infrastructure cash flows, no F1 tie (Vodafone's McLaren deal ended 2013; no current Vodafone/KKR F1 team tie found, search 5 Oct 2026; note Vantage Markets, the Ferrari partner, is an unrelated broker). But pure B2B tower supplier with a handful of MNO customers (Vodafone alone ~83-90%) and no brand-building need, so unlikely to convert.</t>
-        </is>
-      </c>
-      <c r="R4" s="10" t="inlineStr">
-        <is>
-          <t>Only via parent: Vodafone/KKR hospitality angle is weak; park unless Vodafone Group re-enters F1.</t>
-        </is>
-      </c>
-      <c r="S4" s="10" t="inlineStr">
-        <is>
-          <t>customer concentration: Vodafone ~83-90% of revenue plus a handful of MNOs; pure B2B, no consumer brand; ownership change 2023 (infrastructure funds); valuation figure stale (2022); infrastructure-fund owned</t>
-        </is>
-      </c>
-      <c r="T4" s="10" t="inlineStr">
-        <is>
-          <t>Markets 1 (Germany, Spain, Italy, Portugal, Hungary, Netherlands etc.); buyers 1 (MNO senior executives); story 1 (network technology); category free 0 (telecom/infrastructure presence on grid via T-Mobile/Vodafone-type partners; unverified)</t>
+      <c r="P4" s="9" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>Passes hard filters: market cap ~$2.63B (Q1 2026), ~1,400 staff, no F1 tie found (search 5 Oct 2026). Capacity holds: FY2025 loss of $167.1M was non-cash impairment ($183.8M goodwill) while adj EBITDA was $397.5M, Q2 2026 adj EBITDA up 14% at 36.6% margin, FCF guide $220-245M. Divestitures (Industrial Specialties Jan 2026, Road Markings Apr 2026) are portfolio pruning, not distress. Reservation: low-profile B2B with weak marketing motive, fit 3 with category partly taken.</t>
+        </is>
+      </c>
+      <c r="R4" s="9" t="inlineStr">
+        <is>
+          <t>B2B hospitality for automotive-OEM and Tier 1 buyers: position carbon-canister emissions technology around F1 hybrid/sustainable-fuel narrative at a European or US race.</t>
+        </is>
+      </c>
+      <c r="S4" s="9" t="inlineStr">
+        <is>
+          <t>customers likely concentrated (automotive Tier 1s; not verified at &lt;=20); pure B2B low consumer profile; FY2025 net loss $167M driven by $293M non-cash impairments; portfolio divestitures 2026</t>
+        </is>
+      </c>
+      <c r="T4" s="9" t="inlineStr">
+        <is>
+          <t>Markets 1; buyers 1 (B2B decision makers); story 1 (materials technology/emissions performance); category free 0 (energy/chemicals/lubricants heavily represented on grid)</t>
         </is>
       </c>
     </row>
@@ -1884,6 +1982,255 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="70" customWidth="1" min="17" max="17"/>
+    <col width="60" customWidth="1" min="18" max="18"/>
+    <col width="40" customWidth="1" min="19" max="19"/>
+    <col width="50" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>X17 Private 5G &amp; Telecom Equipme — Wave 14 (v3) — 1 new brands: 0 Yes / 0 Stretch / 1 Low-value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Fresh names only (nothing here is in the master or expansion book). Blue = Yes, amber = Stretch, RED = passes the v3 gates but judged low-value / waste of time. Ranked best first. Source_pool: G = broad discovery, A = recovered v2 reject, B = unicorn register.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>priority_score</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>sector_tab</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>source_pool</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>domain</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>hq</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>ownership</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>what_it_sells</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>headcount_band</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>revenue (dated, sourced)</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>valuation (dated, sourced)</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>latest_raise</t>
+        </is>
+      </c>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>fit_score</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="inlineStr">
+        <is>
+          <t>up_and_coming</t>
+        </is>
+      </c>
+      <c r="P3" s="7" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="Q3" s="7" t="inlineStr">
+        <is>
+          <t>verdict_reason</t>
+        </is>
+      </c>
+      <c r="R3" s="7" t="inlineStr">
+        <is>
+          <t>best_angle</t>
+        </is>
+      </c>
+      <c r="S3" s="7" t="inlineStr">
+        <is>
+          <t>flags</t>
+        </is>
+      </c>
+      <c r="T3" s="7" t="inlineStr">
+        <is>
+          <t>fit_detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Vantage Towers</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>X17 Private 5G &amp; Telecom Equipme</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>vantagetowers.com</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Dusseldorf, Germany</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>Oak Holdings (50:50 Vodafone and KKR/GIP) holds ~89%; remainder free float (OTC)</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>Wireless tower infrastructure leased to mobile network operators across 10 European countries (87,824 sites, Mar 2025); no consumer sales</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>201-1k</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>FY2024/25 revenue EUR 665.9M (company filings, Mar 2025)</t>
+        </is>
+      </c>
+      <c r="L4" s="10" t="inlineStr">
+        <is>
+          <t>Equity value EUR 16.2B in the KKR/GIP transaction (announced Nov 2022, EUR 32/share, stale; same price for Vodafone's 10% sale at EUR 1.3B)</t>
+        </is>
+      </c>
+      <c r="M4" s="10" t="inlineStr">
+        <is>
+          <t>None; Vodafone sold further 10% for EUR 1.3B (2026 report, DCD) completing 50:50 JV</t>
+        </is>
+      </c>
+      <c r="N4" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="O4" s="10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="P4" s="10" t="inlineStr">
+        <is>
+          <t>Low-value</t>
+        </is>
+      </c>
+      <c r="Q4" s="10" t="inlineStr">
+        <is>
+          <t>Passes hard filters: EV/equity EUR 16.2B (Nov 2022 deal, dated), ~883 avg staff (Oak Group, Mar 2025), healthy infrastructure cash flows, no F1 tie (Vodafone's McLaren deal ended 2013; no current Vodafone/KKR F1 team tie found, search 5 Oct 2026; note Vantage Markets, the Ferrari partner, is an unrelated broker). But pure B2B tower supplier with a handful of MNO customers (Vodafone alone ~83-90%) and no brand-building need, so unlikely to convert.</t>
+        </is>
+      </c>
+      <c r="R4" s="10" t="inlineStr">
+        <is>
+          <t>Only via parent: Vodafone/KKR hospitality angle is weak; park unless Vodafone Group re-enters F1.</t>
+        </is>
+      </c>
+      <c r="S4" s="10" t="inlineStr">
+        <is>
+          <t>customer concentration: Vodafone ~83-90% of revenue plus a handful of MNOs; pure B2B, no consumer brand; ownership change 2023 (infrastructure funds); valuation figure stale (2022); infrastructure-fund owned</t>
+        </is>
+      </c>
+      <c r="T4" s="10" t="inlineStr">
+        <is>
+          <t>Markets 1 (Germany, Spain, Italy, Portugal, Hungary, Netherlands etc.); buyers 1 (MNO senior executives); story 1 (network technology); category free 0 (telecom/infrastructure presence on grid via T-Mobile/Vodafone-type partners; unverified)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:T4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22071,7 +22418,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22451,6 +22798,351 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="70" customWidth="1" min="17" max="17"/>
+    <col width="60" customWidth="1" min="18" max="18"/>
+    <col width="40" customWidth="1" min="19" max="19"/>
+    <col width="50" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>UP-AND-COMING BRANDS, ALL SECTORS — 2 names: crossed $1B within 24 months, growing &gt;40%/yr, 2025-26 IPO, or visible challenger</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Consolidated view of every up_and_coming=yes brand across all tabs, ranked best first. The same rows also sit on their sector tabs. Blue = Yes, amber = Stretch, RED = low-value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>priority_score</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>sector_tab</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>source_pool</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>domain</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>hq</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>ownership</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>what_it_sells</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>headcount_band</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>revenue (dated, sourced)</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>valuation (dated, sourced)</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>latest_raise</t>
+        </is>
+      </c>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>fit_score</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="inlineStr">
+        <is>
+          <t>up_and_coming</t>
+        </is>
+      </c>
+      <c r="P3" s="7" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="Q3" s="7" t="inlineStr">
+        <is>
+          <t>verdict_reason</t>
+        </is>
+      </c>
+      <c r="R3" s="7" t="inlineStr">
+        <is>
+          <t>best_angle</t>
+        </is>
+      </c>
+      <c r="S3" s="7" t="inlineStr">
+        <is>
+          <t>flags</t>
+        </is>
+      </c>
+      <c r="T3" s="7" t="inlineStr">
+        <is>
+          <t>fit_detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Bayut (EMPG)</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>X02 Real Estate &amp; Building Produ</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>dubizzlegroup.com</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Dubai, UAE</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Private; Dubizzle Group (ex-EMPG, merged with OLX Group MENA 2022); IPO on Dubai market planned 2026 (est). Prosus/OLX and General Atlantic among holders (not re-verified)</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Online property and classifieds marketplaces: Bayut, dubizzle (UAE, GCC, Egypt), plus Zameen (Pakistan), OLX, Lamudi (Indonesia, Philippines)</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>Group revenue USD 222M in 2024 (up from 220.8M 2023); H1 2025 USD 133M vs 105M H1 2024 (Dubizzle Group IPO coverage, 2025-26)</t>
+        </is>
+      </c>
+      <c r="L4" s="8" t="inlineStr">
+        <is>
+          <t>Over USD 1B at 2021 USD 150M round (MENAbytes, 2021); Bloomberg-reported IPO value around USD 2B (2026, via capex.com/Gulf News coverage). Analyst peer-multiple estimate USD 0.6-0.9B (est, lower-confidence)</t>
+        </is>
+      </c>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>USD 200M round, Oct 2022 (Entrepreneur ME/Arabian Business); IPO of about 30% (1.25B shares) targeted for Dubai listing around Nov 2026 (Gulf News, 2026)</t>
+        </is>
+      </c>
+      <c r="N4" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="O4" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t>All v3 hard filters pass: valuation over USD 1B (2021 round, IPO talk ~USD 2B), about 2,400-3,500 employees, revenue USD 222M 2024 with H1 2025 growth ~27% and EBITDA-positive per CEO, no F1/motorsport tie found in search, not sanctioned. Fit 3, consumer brand with IPO-driven awareness motive.</t>
+        </is>
+      </c>
+      <c r="R4" s="8" t="inlineStr">
+        <is>
+          <t>Pre-IPO awareness play in the Gulf races (Abu Dhabi, Jeddah, Qatar): hospitality and regional digital-activation package positioning Bayut/dubizzle as the Gulf's property and marketplace leader, sold to the CMO ahead of the Nov 2026 listing (est).</t>
+        </is>
+      </c>
+      <c r="S4" s="8" t="inlineStr">
+        <is>
+          <t>IPO pending (planned Nov 2026); valuation sources mixed (2021 USD 1B+ confirmed; USD 2B IPO figure is press-reported); revenue figure is group-level, not Bayut alone; PE/strategic holder structure</t>
+        </is>
+      </c>
+      <c r="T4" s="8" t="inlineStr">
+        <is>
+          <t>Sells in 3+ F1 markets: yes (UAE, Saudi/Qatar/Bahrain GCC, Egypt, Indonesia, Philippines). Affluent 25-54 property buyers/sellers: yes. Brand story tech marketplace with listing ambition: yes. Category not on grid: unconfirmed, marked 0 pending check (property portals not seen among 2026 team partner lists). No F1 tie found in search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>MP Materials</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>X04 Mining, Metals &amp; Commodities</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>mpmaterials.com</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Las Vegas, Nevada, USA</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>Public (NYSE: MP); US Dept of Defense is a large minority holder (not majority, est ~15%)</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>NdPr oxide, rare-earth magnets and precursors to US defense primes, automakers (GM) and Apple supply deal; customers few and strategic</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>Q2 2026 revenue $108.5M, +89% YoY; revenue plus PPA income $126.1M; Q2 net loss $20.3M, adj. EBITDA +$28.5M (Q2 2026 call, Aug 2026)</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>Market cap $8.6B (182.74M sh x $46.98, Oct 2026 per search aggregator)</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>Not re-verified this run (2025 DoD/Apple/bank financing recalled from prior knowledge, est); Q2 2026 EBITDA now positive</t>
+        </is>
+      </c>
+      <c r="N5" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="O5" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>Passes hard filters (market cap $8.6B Oct 2026, ~1,071 employees Dec 2025, no distress or F1 tie found; revenue +89% YoY). Prior concentration rejection no longer applies. Reservation: no visible consumer or sports marketing function, so marketing motive is unproven; still loss-making at net level.</t>
+        </is>
+      </c>
+      <c r="R5" s="9" t="inlineStr">
+        <is>
+          <t>Position as the American rare-earth magnet supplier for hybrid/electric powertrains and precision motors (F1 2026 hybrid theme); US GP Austin/Miami hospitality for OEM and defense buyers (est).</t>
+        </is>
+      </c>
+      <c r="S5" s="9" t="inlineStr">
+        <is>
+          <t>concentrated customers (DoD, defense primes, automakers, Apple); US government large shareholder (not majority); net loss, approaching breakeven; revenue small relative to valuation (~20-25x TTM est); stock-price driven valuation</t>
+        </is>
+      </c>
+      <c r="T5" s="9" t="inlineStr">
+        <is>
+          <t>Markets 0 (US-centred sales, est). Buyers 1 (senior defense/auto procurement). Story 1 (precision tech, strategic supply, ambition). Category 1 (rare earths not on grid).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:T5"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23755,7 +24447,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -24484,7 +25176,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -24729,351 +25421,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A3:T4"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:T5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="38" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
-    <col width="50" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
-    <col width="7" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="70" customWidth="1" min="17" max="17"/>
-    <col width="60" customWidth="1" min="18" max="18"/>
-    <col width="40" customWidth="1" min="19" max="19"/>
-    <col width="50" customWidth="1" min="20" max="20"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>X02 Real Estate &amp; Building Produ — Wave 14 (v3) — 2 new brands: 1 Yes / 0 Stretch / 1 Low-value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Fresh names only (nothing here is in the master or expansion book). Blue = Yes, amber = Stretch, RED = passes the v3 gates but judged low-value / waste of time. Ranked best first. Source_pool: G = broad discovery, A = recovered v2 reject, B = unicorn register.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>rank</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>priority_score</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>company</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>sector_tab</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>source_pool</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>domain</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
-        <is>
-          <t>hq</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>ownership</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr">
-        <is>
-          <t>what_it_sells</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>headcount_band</t>
-        </is>
-      </c>
-      <c r="K3" s="7" t="inlineStr">
-        <is>
-          <t>revenue (dated, sourced)</t>
-        </is>
-      </c>
-      <c r="L3" s="7" t="inlineStr">
-        <is>
-          <t>valuation (dated, sourced)</t>
-        </is>
-      </c>
-      <c r="M3" s="7" t="inlineStr">
-        <is>
-          <t>latest_raise</t>
-        </is>
-      </c>
-      <c r="N3" s="7" t="inlineStr">
-        <is>
-          <t>fit_score</t>
-        </is>
-      </c>
-      <c r="O3" s="7" t="inlineStr">
-        <is>
-          <t>up_and_coming</t>
-        </is>
-      </c>
-      <c r="P3" s="7" t="inlineStr">
-        <is>
-          <t>verdict</t>
-        </is>
-      </c>
-      <c r="Q3" s="7" t="inlineStr">
-        <is>
-          <t>verdict_reason</t>
-        </is>
-      </c>
-      <c r="R3" s="7" t="inlineStr">
-        <is>
-          <t>best_angle</t>
-        </is>
-      </c>
-      <c r="S3" s="7" t="inlineStr">
-        <is>
-          <t>flags</t>
-        </is>
-      </c>
-      <c r="T3" s="7" t="inlineStr">
-        <is>
-          <t>fit_detail</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Bayut (EMPG)</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>X02 Real Estate &amp; Building Produ</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>dubizzlegroup.com</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>Dubai, UAE</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>Private; Dubizzle Group (ex-EMPG, merged with OLX Group MENA 2022); IPO on Dubai market planned 2026 (est). Prosus/OLX and General Atlantic among holders (not re-verified)</t>
-        </is>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>Online property and classifieds marketplaces: Bayut, dubizzle (UAE, GCC, Egypt), plus Zameen (Pakistan), OLX, Lamudi (Indonesia, Philippines)</t>
-        </is>
-      </c>
-      <c r="J4" s="8" t="inlineStr">
-        <is>
-          <t>1k-5k</t>
-        </is>
-      </c>
-      <c r="K4" s="8" t="inlineStr">
-        <is>
-          <t>Group revenue USD 222M in 2024 (up from 220.8M 2023); H1 2025 USD 133M vs 105M H1 2024 (Dubizzle Group IPO coverage, 2025-26)</t>
-        </is>
-      </c>
-      <c r="L4" s="8" t="inlineStr">
-        <is>
-          <t>Over USD 1B at 2021 USD 150M round (MENAbytes, 2021); Bloomberg-reported IPO value around USD 2B (2026, via capex.com/Gulf News coverage). Analyst peer-multiple estimate USD 0.6-0.9B (est, lower-confidence)</t>
-        </is>
-      </c>
-      <c r="M4" s="8" t="inlineStr">
-        <is>
-          <t>USD 200M round, Oct 2022 (Entrepreneur ME/Arabian Business); IPO of about 30% (1.25B shares) targeted for Dubai listing around Nov 2026 (Gulf News, 2026)</t>
-        </is>
-      </c>
-      <c r="N4" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="O4" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q4" s="8" t="inlineStr">
-        <is>
-          <t>All v3 hard filters pass: valuation over USD 1B (2021 round, IPO talk ~USD 2B), about 2,400-3,500 employees, revenue USD 222M 2024 with H1 2025 growth ~27% and EBITDA-positive per CEO, no F1/motorsport tie found in search, not sanctioned. Fit 3, consumer brand with IPO-driven awareness motive.</t>
-        </is>
-      </c>
-      <c r="R4" s="8" t="inlineStr">
-        <is>
-          <t>Pre-IPO awareness play in the Gulf races (Abu Dhabi, Jeddah, Qatar): hospitality and regional digital-activation package positioning Bayut/dubizzle as the Gulf's property and marketplace leader, sold to the CMO ahead of the Nov 2026 listing (est).</t>
-        </is>
-      </c>
-      <c r="S4" s="8" t="inlineStr">
-        <is>
-          <t>IPO pending (planned Nov 2026); valuation sources mixed (2021 USD 1B+ confirmed; USD 2B IPO figure is press-reported); revenue figure is group-level, not Bayut alone; PE/strategic holder structure</t>
-        </is>
-      </c>
-      <c r="T4" s="8" t="inlineStr">
-        <is>
-          <t>Sells in 3+ F1 markets: yes (UAE, Saudi/Qatar/Bahrain GCC, Egypt, Indonesia, Philippines). Affluent 25-54 property buyers/sellers: yes. Brand story tech marketplace with listing ambition: yes. Category not on grid: unconfirmed, marked 0 pending check (property portals not seen among 2026 team partner lists). No F1 tie found in search.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="10" t="n">
-        <v>24</v>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>LGI Homes Inc</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>X02 Real Estate &amp; Building Produ</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>lgihomes.com</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>The Woodlands, Texas, USA</t>
-        </is>
-      </c>
-      <c r="H5" s="10" t="inlineStr">
-        <is>
-          <t>Public (NASDAQ: LGIH)</t>
-        </is>
-      </c>
-      <c r="I5" s="10" t="inlineStr">
-        <is>
-          <t>Entry-level single-family homes in US only (~30+ US markets)</t>
-        </is>
-      </c>
-      <c r="J5" s="10" t="inlineStr">
-        <is>
-          <t>1k-5k</t>
-        </is>
-      </c>
-      <c r="K5" s="10" t="inlineStr">
-        <is>
-          <t>TTM revenue ~$1.67-1.71B, down ~22.6% YoY (StockAnalysis/Fool, Jul-Aug 2026); H1 2026 net income $29.1M, TTM net income $66.2M (10-Q 30 Jun 2026)</t>
-        </is>
-      </c>
-      <c r="L5" s="10" t="inlineStr">
-        <is>
-          <t>Market cap $1.34B (StockAnalysis, 23 Jul 2026); 1,056 employees (same source)</t>
-        </is>
-      </c>
-      <c r="M5" s="10" t="inlineStr">
-        <is>
-          <t>none (public; reduced debt by $128.6M in Q2 2026, ~$1.6B debt outstanding, debt/capital 42.6% - Q2 2026 call, Aug 2026)</t>
-        </is>
-      </c>
-      <c r="N5" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="O5" s="10" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="P5" s="10" t="inlineStr">
-        <is>
-          <t>Low-value</t>
-        </is>
-      </c>
-      <c r="Q5" s="10" t="inlineStr">
-        <is>
-          <t>Passes hard filters (mkt cap $1.34B Jul 2026, 1,056 staff, profitable and deleveraging with no layoffs or going-concern doubt found, no F1 tie found in search) but fit is 1 and the brand is entry-level, US-only; unlikely to convert. Prior capacity rejection not upheld under v3: profit is down but positive and no restructuring found.</t>
-        </is>
-      </c>
-      <c r="R5" s="10" t="inlineStr">
-        <is>
-          <t>US-only: Austin/Miami GP hospitality for builder and land-partner entertaining (est); low odds given $66M TTM profit and deleveraging priority.</t>
-        </is>
-      </c>
-      <c r="S5" s="10" t="inlineStr">
-        <is>
-          <t>revenue down ~22% YoY; net income falling, still profitable; deleveraging phase, ~$1.6B debt; market cap only ~34% above $1B bar; US-only sales</t>
-        </is>
-      </c>
-      <c r="T5" s="10" t="inlineStr">
-        <is>
-          <t>Markets 0 (US only). Buyers 0 (entry-level first-time buyers, not affluent). Story 0 (no performance/tech narrative). Category 1 (homebuilding not on grid).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A3:T5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -25112,7 +25459,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>X04 Mining, Metals &amp; Commodities — Wave 14 (v3) — 2 new brands: 0 Yes / 1 Stretch / 1 Low-value</t>
+          <t>X02 Real Estate &amp; Building Produ — Wave 14 (v3) — 2 new brands: 1 Yes / 0 Stretch / 1 Low-value</t>
         </is>
       </c>
     </row>
@@ -25226,98 +25573,98 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="n">
+      <c r="A4" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="9" t="n">
-        <v>58</v>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>MP Materials</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>X04 Mining, Metals &amp; Commodities</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="B4" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Bayut (EMPG)</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>X02 Real Estate &amp; Building Produ</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>mpmaterials.com</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>Las Vegas, Nevada, USA</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>Public (NYSE: MP); US Dept of Defense is a large minority holder (not majority, est ~15%)</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="inlineStr">
-        <is>
-          <t>NdPr oxide, rare-earth magnets and precursors to US defense primes, automakers (GM) and Apple supply deal; customers few and strategic</t>
-        </is>
-      </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>dubizzlegroup.com</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Dubai, UAE</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Private; Dubizzle Group (ex-EMPG, merged with OLX Group MENA 2022); IPO on Dubai market planned 2026 (est). Prosus/OLX and General Atlantic among holders (not re-verified)</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Online property and classifieds marketplaces: Bayut, dubizzle (UAE, GCC, Egypt), plus Zameen (Pakistan), OLX, Lamudi (Indonesia, Philippines)</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
         <is>
           <t>1k-5k</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr">
-        <is>
-          <t>Q2 2026 revenue $108.5M, +89% YoY; revenue plus PPA income $126.1M; Q2 net loss $20.3M, adj. EBITDA +$28.5M (Q2 2026 call, Aug 2026)</t>
-        </is>
-      </c>
-      <c r="L4" s="9" t="inlineStr">
-        <is>
-          <t>Market cap $8.6B (182.74M sh x $46.98, Oct 2026 per search aggregator)</t>
-        </is>
-      </c>
-      <c r="M4" s="9" t="inlineStr">
-        <is>
-          <t>Not re-verified this run (2025 DoD/Apple/bank financing recalled from prior knowledge, est); Q2 2026 EBITDA now positive</t>
-        </is>
-      </c>
-      <c r="N4" s="9" t="n">
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>Group revenue USD 222M in 2024 (up from 220.8M 2023); H1 2025 USD 133M vs 105M H1 2024 (Dubizzle Group IPO coverage, 2025-26)</t>
+        </is>
+      </c>
+      <c r="L4" s="8" t="inlineStr">
+        <is>
+          <t>Over USD 1B at 2021 USD 150M round (MENAbytes, 2021); Bloomberg-reported IPO value around USD 2B (2026, via capex.com/Gulf News coverage). Analyst peer-multiple estimate USD 0.6-0.9B (est, lower-confidence)</t>
+        </is>
+      </c>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>USD 200M round, Oct 2022 (Entrepreneur ME/Arabian Business); IPO of about 30% (1.25B shares) targeted for Dubai listing around Nov 2026 (Gulf News, 2026)</t>
+        </is>
+      </c>
+      <c r="N4" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="9" t="inlineStr">
+      <c r="O4" s="8" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="P4" s="9" t="inlineStr">
-        <is>
-          <t>Stretch</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Passes hard filters (market cap $8.6B Oct 2026, ~1,071 employees Dec 2025, no distress or F1 tie found; revenue +89% YoY). Prior concentration rejection no longer applies. Reservation: no visible consumer or sports marketing function, so marketing motive is unproven; still loss-making at net level.</t>
-        </is>
-      </c>
-      <c r="R4" s="9" t="inlineStr">
-        <is>
-          <t>Position as the American rare-earth magnet supplier for hybrid/electric powertrains and precision motors (F1 2026 hybrid theme); US GP Austin/Miami hospitality for OEM and defense buyers (est).</t>
-        </is>
-      </c>
-      <c r="S4" s="9" t="inlineStr">
-        <is>
-          <t>concentrated customers (DoD, defense primes, automakers, Apple); US government large shareholder (not majority); net loss, approaching breakeven; revenue small relative to valuation (~20-25x TTM est); stock-price driven valuation</t>
-        </is>
-      </c>
-      <c r="T4" s="9" t="inlineStr">
-        <is>
-          <t>Markets 0 (US-centred sales, est). Buyers 1 (senior defense/auto procurement). Story 1 (precision tech, strategic supply, ambition). Category 1 (rare earths not on grid).</t>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t>All v3 hard filters pass: valuation over USD 1B (2021 round, IPO talk ~USD 2B), about 2,400-3,500 employees, revenue USD 222M 2024 with H1 2025 growth ~27% and EBITDA-positive per CEO, no F1/motorsport tie found in search, not sanctioned. Fit 3, consumer brand with IPO-driven awareness motive.</t>
+        </is>
+      </c>
+      <c r="R4" s="8" t="inlineStr">
+        <is>
+          <t>Pre-IPO awareness play in the Gulf races (Abu Dhabi, Jeddah, Qatar): hospitality and regional digital-activation package positioning Bayut/dubizzle as the Gulf's property and marketplace leader, sold to the CMO ahead of the Nov 2026 listing (est).</t>
+        </is>
+      </c>
+      <c r="S4" s="8" t="inlineStr">
+        <is>
+          <t>IPO pending (planned Nov 2026); valuation sources mixed (2021 USD 1B+ confirmed; USD 2B IPO figure is press-reported); revenue figure is group-level, not Bayut alone; PE/strategic holder structure</t>
+        </is>
+      </c>
+      <c r="T4" s="8" t="inlineStr">
+        <is>
+          <t>Sells in 3+ F1 markets: yes (UAE, Saudi/Qatar/Bahrain GCC, Egypt, Indonesia, Philippines). Affluent 25-54 property buyers/sellers: yes. Brand story tech marketplace with listing ambition: yes. Category not on grid: unconfirmed, marked 0 pending check (property portals not seen among 2026 team partner lists). No F1 tie found in search.</t>
         </is>
       </c>
     </row>
@@ -25326,16 +25673,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>NRW Holdings</t>
+          <t>LGI Homes Inc</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>X04 Mining, Metals &amp; Commodities</t>
+          <t>X02 Real Estate &amp; Building Produ</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
@@ -25345,46 +25692,46 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>nrw.com.au</t>
+          <t>lgihomes.com</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>Perth, Australia</t>
+          <t>The Woodlands, Texas, USA</t>
         </is>
       </c>
       <c r="H5" s="10" t="inlineStr">
         <is>
-          <t>Public (ASX: NWH)</t>
+          <t>Public (NASDAQ: LGIH)</t>
         </is>
       </c>
       <c r="I5" s="10" t="inlineStr">
         <is>
-          <t>Civil, mining contracting and drill-and-blast / mining services (Fredon acquired Oct 2025); customers are mining, energy and infrastructure clients in Australia</t>
+          <t>Entry-level single-family homes in US only (~30+ US markets)</t>
         </is>
       </c>
       <c r="J5" s="10" t="inlineStr">
         <is>
-          <t>10k+</t>
+          <t>1k-5k</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>FY26 (to Jun 2026) revenue A$4.3B, +31.4% YoY; underlying EBITA A$288.6M, NPAT A$182.7M (Investing.com/Kalkine, Aug 2026)</t>
+          <t>TTM revenue ~$1.67-1.71B, down ~22.6% YoY (StockAnalysis/Fool, Jul-Aug 2026); H1 2026 net income $29.1M, TTM net income $66.2M (10-Q 30 Jun 2026)</t>
         </is>
       </c>
       <c r="L5" s="10" t="inlineStr">
         <is>
-          <t>Market cap 3.68B (currency AUD/NZD per source; roughly USD 2.1-2.4B est) as of 2 Oct 2026 (companiesmarketcap/StockAnalysis); ~14,000 employees (Kalkine, 2026)</t>
+          <t>Market cap $1.34B (StockAnalysis, 23 Jul 2026); 1,056 employees (same source)</t>
         </is>
       </c>
       <c r="M5" s="10" t="inlineStr">
         <is>
-          <t>none; Fredon acquisition completed Oct 2025</t>
+          <t>none (public; reduced debt by $128.6M in Q2 2026, ~$1.6B debt outstanding, debt/capital 42.6% - Q2 2026 call, Aug 2026)</t>
         </is>
       </c>
       <c r="N5" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O5" s="10" t="inlineStr">
         <is>
@@ -25398,22 +25745,22 @@
       </c>
       <c r="Q5" s="10" t="inlineStr">
         <is>
-          <t>All hard filters pass (market cap ~USD 2B+ est, ~14,000 staff, record profit, no F1 tie found). But it is a pure B2B contractor with concentrated customers, no consumer brand and no sign of brand ambition; fit 2 at best with no credible marketing motive.</t>
+          <t>Passes hard filters (mkt cap $1.34B Jul 2026, 1,056 staff, profitable and deleveraging with no layoffs or going-concern doubt found, no F1 tie found in search) but fit is 1 and the brand is entry-level, US-only; unlikely to convert. Prior capacity rejection not upheld under v3: profit is down but positive and no restructuring found.</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
-          <t>Australian GP (Melbourne) client hospitality for mining and energy executives (est), pitched as precision-engineering safety/reliability story; low conversion odds.</t>
+          <t>US-only: Austin/Miami GP hospitality for builder and land-partner entertaining (est); low odds given $66M TTM profit and deleveraging priority.</t>
         </is>
       </c>
       <c r="S5" s="10" t="inlineStr">
         <is>
-          <t>concentrated customers (small number of large mining clients); pure B2B contractor; recent acquisition (Fredon, Oct 2025); single-country revenue</t>
+          <t>revenue down ~22% YoY; net income falling, still profitable; deleveraging phase, ~$1.6B debt; market cap only ~34% above $1B bar; US-only sales</t>
         </is>
       </c>
       <c r="T5" s="10" t="inlineStr">
         <is>
-          <t>Markets 0 (Australia-centred). Buyers 1 (senior mining/energy decision makers). Story 0-1 engineering reliability, scored 0. Category 1 (mining services not on grid).</t>
+          <t>Markets 0 (US only). Buyers 0 (entry-level first-time buyers, not affluent). Story 0 (no performance/tech narrative). Category 1 (homebuilding not on grid).</t>
         </is>
       </c>
     </row>
@@ -25429,7 +25776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:T5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -25457,7 +25804,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>X05 Agriculture &amp; AgTech — Wave 14 (v3) — 3 new brands: 0 Yes / 2 Stretch / 1 Low-value</t>
+          <t>X04 Mining, Metals &amp; Commodities — Wave 14 (v3) — 2 new brands: 0 Yes / 1 Stretch / 1 Low-value</t>
         </is>
       </c>
     </row>
@@ -25579,12 +25926,12 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Netafim (Orbia)</t>
+          <t>MP Materials</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>X05 Agriculture &amp; AgTech</t>
+          <t>X04 Mining, Metals &amp; Commodities</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -25594,22 +25941,22 @@
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>netafim.com</t>
+          <t>mpmaterials.com</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>Tel Aviv, Israel (Kibbutz Hatzerim origin)</t>
+          <t>Las Vegas, Nevada, USA</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>Orbia (Mexico, NYSE-listed parent) 80%, Kibbutz Hatzerim 20%; controlling stake under sale, no deal closed</t>
+          <t>Public (NYSE: MP); US Dept of Defense is a large minority holder (not majority, est ~15%)</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>Drip and precision-irrigation systems and digital agronomy in 110+ countries</t>
+          <t>NdPr oxide, rare-earth magnets and precursors to US defense primes, automakers (GM) and Apple supply deal; customers few and strategic</t>
         </is>
       </c>
       <c r="J4" s="9" t="inlineStr">
@@ -25619,17 +25966,17 @@
       </c>
       <c r="K4" s="9" t="inlineStr">
         <is>
-          <t>Annual revenue &gt;$1B, ~$250M (about 25%) in US (Calcalist/ynet, Feb 2026); segment revenue reportedly down 3 consecutive years (prior hint)</t>
+          <t>Q2 2026 revenue $108.5M, +89% YoY; revenue plus PPA income $126.1M; Q2 net loss $20.3M, adj. EBITDA +$28.5M (Q2 2026 call, Aug 2026)</t>
         </is>
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Reported EV ~$1.2B (asking ~$1.4B), vs $1.8B paid by Orbia in 2017 (Calcalist, Aug 2026)</t>
+          <t>Market cap $8.6B (182.74M sh x $46.98, Oct 2026 per search aggregator)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>none; 2026 sale process: Chinese (Dayu/Hopu) bid hit regulatory hurdles, Fortissimo talks froze, Spanish bidder at ~$1.4B (Calcalist, Aug 2026)</t>
+          <t>Not re-verified this run (2025 DoD/Apple/bank financing recalled from prior knowledge, est); Q2 2026 EBITDA now positive</t>
         </is>
       </c>
       <c r="N4" s="9" t="n">
@@ -25637,229 +25984,133 @@
       </c>
       <c r="O4" s="9" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="P4" s="9" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>Passes hard filters (market cap $8.6B Oct 2026, ~1,071 employees Dec 2025, no distress or F1 tie found; revenue +89% YoY). Prior concentration rejection no longer applies. Reservation: no visible consumer or sports marketing function, so marketing motive is unproven; still loss-making at net level.</t>
+        </is>
+      </c>
+      <c r="R4" s="9" t="inlineStr">
+        <is>
+          <t>Position as the American rare-earth magnet supplier for hybrid/electric powertrains and precision motors (F1 2026 hybrid theme); US GP Austin/Miami hospitality for OEM and defense buyers (est).</t>
+        </is>
+      </c>
+      <c r="S4" s="9" t="inlineStr">
+        <is>
+          <t>concentrated customers (DoD, defense primes, automakers, Apple); US government large shareholder (not majority); net loss, approaching breakeven; revenue small relative to valuation (~20-25x TTM est); stock-price driven valuation</t>
+        </is>
+      </c>
+      <c r="T4" s="9" t="inlineStr">
+        <is>
+          <t>Markets 0 (US-centred sales, est). Buyers 1 (senior defense/auto procurement). Story 1 (precision tech, strategic supply, ambition). Category 1 (rare earths not on grid).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>NRW Holdings</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>X04 Mining, Metals &amp; Commodities</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>nrw.com.au</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Perth, Australia</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>Public (ASX: NWH)</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>Civil, mining contracting and drill-and-blast / mining services (Fredon acquired Oct 2025); customers are mining, energy and infrastructure clients in Australia</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>FY26 (to Jun 2026) revenue A$4.3B, +31.4% YoY; underlying EBITA A$288.6M, NPAT A$182.7M (Investing.com/Kalkine, Aug 2026)</t>
+        </is>
+      </c>
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>Market cap 3.68B (currency AUD/NZD per source; roughly USD 2.1-2.4B est) as of 2 Oct 2026 (companiesmarketcap/StockAnalysis); ~14,000 employees (Kalkine, 2026)</t>
+        </is>
+      </c>
+      <c r="M5" s="10" t="inlineStr">
+        <is>
+          <t>none; Fredon acquisition completed Oct 2025</t>
+        </is>
+      </c>
+      <c r="N5" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="O5" s="10" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
-      <c r="P4" s="9" t="inlineStr">
-        <is>
-          <t>Stretch</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Passes hard filters (EV ~$1.2-1.4B reported 2026, ~4,500 staff, revenue &gt;$1B, no F1 tie found for Netafim or Orbia). Real reservation: control is being sold by a financially stressed parent, so budget authority and marketing priority are uncertain. Parent distress is not Netafim distress, so not hardened to No.</t>
-        </is>
-      </c>
-      <c r="R4" s="9" t="inlineStr">
-        <is>
-          <t>Wait for new owner; then pitch precision-irrigation 'water-efficiency engineering' sustainability partnership at US/Miami or Spanish GP hospitality (est).</t>
-        </is>
-      </c>
-      <c r="S4" s="9" t="inlineStr">
-        <is>
-          <t>ownership change pending (sale of control in progress); parent Orbia under financial pressure; valuation only modestly above $1B and falling; declining revenue (prior hint); possible Chinese buyer, regulatory risk</t>
-        </is>
-      </c>
-      <c r="T4" s="9" t="inlineStr">
-        <is>
-          <t>Markets 1 (110+ countries, US, India, Europe). Buyers 0 (growers, not affluent urban 25-54; B2B decision makers weak). Story 1 (precision, technology, water). Category 1 (irrigation not on grid). Scored 3 incl. B2B senior buyers loosely.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="9" t="n">
-        <v>58</v>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>Pivot Bio</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>X05 Agriculture &amp; AgTech</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>pivotbio.com</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>Minnetonka, Minnesota, USA (HQ moved from Berkeley)</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>Private, venture-backed</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="inlineStr">
-        <is>
-          <t>Microbial nitrogen products for corn, wheat and sorghum farmers (PROVEN 40 etc.)</t>
-        </is>
-      </c>
-      <c r="J5" s="9" t="inlineStr">
-        <is>
-          <t>201-1k</t>
-        </is>
-      </c>
-      <c r="K5" s="9" t="inlineStr">
-        <is>
-          <t>Surpassed USD 100M revenue by 2023 (AgFunderNews, 2023); current revenue not confirmed</t>
-        </is>
-      </c>
-      <c r="L5" s="9" t="inlineStr">
-        <is>
-          <t>USD 1.66B post-money at Series F-2 (Forge/Pivot Bio, 11 Mar 2026); USD 2.0B at Series D (Aug 2023)</t>
-        </is>
-      </c>
-      <c r="M5" s="9" t="inlineStr">
-        <is>
-          <t>USD 100M Series F-2, 11 Mar 2026 at USD 5.71/share, investors undisclosed (Forge, Pivot Bio press release, 2026)</t>
-        </is>
-      </c>
-      <c r="N5" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="O5" s="9" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="P5" s="9" t="inlineStr">
-        <is>
-          <t>Stretch</t>
-        </is>
-      </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Hard filters pass: valuation USD 1.66B (Mar 2026), about 310 staff, USD 100M raised Mar 2026 (within 24 months), no F1 tie, not sanctioned. One real reservation: capacity doubt, since 2025 layoffs and a down round suggest cost discipline and the farmer audience limits F1 relevance.</t>
-        </is>
-      </c>
-      <c r="R5" s="9" t="inlineStr">
-        <is>
-          <t>Sustainability-and-technology story for US/Canada/Brazil/Mexico race weekends: a hospitality and content package aimed at ag retailers, co-ops and grain-company decision makers, positioned as precision biology (est).</t>
-        </is>
-      </c>
-      <c r="S5" s="9" t="inlineStr">
-        <is>
-          <t>valuation down round: USD 2.0B (2023) to USD 1.66B (2026); 62 layoffs (about 20%) and Berkeley R&amp;D relocation, May-Jun 2025; B2B ag brand with farmer audience; 310 employees (ZoomInfo/Trueup, 2026)</t>
-        </is>
-      </c>
-      <c r="T5" s="9" t="inlineStr">
-        <is>
-          <t>Sells in 3+ F1 markets: US, Canada, Brazil (1, est, not re-verified). Buyers are farm owners/ag retailers, mostly not affluent 25-54 consumers (0). Biology and machine-learning technology story (1). Category not on grid (1). No F1 or motorsport tie found.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>PI Industries</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>X05 Agriculture &amp; AgTech</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>piindustries.com</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>Udaipur, Rajasthan, India</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>Public (NSE/BSE: PIIND); promoter-led (Mehra family)</t>
-        </is>
-      </c>
-      <c r="I6" s="10" t="inlineStr">
-        <is>
-          <t>Custom synthesis and manufacturing (CSM, ~76% of revenue) for global agrochemical innovators plus domestic agrochemicals and Plant Health brands</t>
-        </is>
-      </c>
-      <c r="J6" s="10" t="inlineStr">
-        <is>
-          <t>5k-10k</t>
-        </is>
-      </c>
-      <c r="K6" s="10" t="inlineStr">
-        <is>
-          <t>FY26 (to Mar 2026) revenue INR 6,714-7,024 crore (~USD 770-800M est), down from INR 8,322 crore FY25; net profit INR 1,321 crore vs 1,660 crore (Axis/StockAnalysis, Oct 2026)</t>
-        </is>
-      </c>
-      <c r="L6" s="10" t="inlineStr">
-        <is>
-          <t>Market cap INR 34,061 crore (~USD 3.9B est at ~87.5 INR/USD) as of 5 Oct 2026 (companiesmarketcap); 6,353 employees (same)</t>
-        </is>
-      </c>
-      <c r="M6" s="10" t="inlineStr">
-        <is>
-          <t>none (public)</t>
-        </is>
-      </c>
-      <c r="N6" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="O6" s="10" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="P6" s="10" t="inlineStr">
+      <c r="P5" s="10" t="inlineStr">
         <is>
           <t>Low-value</t>
         </is>
       </c>
-      <c r="Q6" s="10" t="inlineStr">
-        <is>
-          <t>All hard filters pass (market cap ~USD 3.9B, 6,353 staff, profitable, no F1 tie found). But the core is B2B contract manufacturing for ~20 innovators with no brand ambition, revenue and profit are falling, and fit is only 2; domestic Plant Health brands target farmers, not an F1 audience.</t>
-        </is>
-      </c>
-      <c r="R6" s="10" t="inlineStr">
-        <is>
-          <t>Singapore or Abu Dhabi GP client hospitality for global agrochemical innovator executives (est); India-focused brand play has no F1 race to anchor.</t>
-        </is>
-      </c>
-      <c r="S6" s="10" t="inlineStr">
-        <is>
-          <t>concentrated customers (~20 global innovators, 18 of top 20); revenue down ~16% in FY26; profit down 20%; pure B2B CSM core</t>
-        </is>
-      </c>
-      <c r="T6" s="10" t="inlineStr">
-        <is>
-          <t>Markets 1 (exports to US, Europe, Japan, plus India; est). Buyers 0 (farmers; innovator procurement). Story 0-1. Category 1. Scored 2.</t>
+      <c r="Q5" s="10" t="inlineStr">
+        <is>
+          <t>All hard filters pass (market cap ~USD 2B+ est, ~14,000 staff, record profit, no F1 tie found). But it is a pure B2B contractor with concentrated customers, no consumer brand and no sign of brand ambition; fit 2 at best with no credible marketing motive.</t>
+        </is>
+      </c>
+      <c r="R5" s="10" t="inlineStr">
+        <is>
+          <t>Australian GP (Melbourne) client hospitality for mining and energy executives (est), pitched as precision-engineering safety/reliability story; low conversion odds.</t>
+        </is>
+      </c>
+      <c r="S5" s="10" t="inlineStr">
+        <is>
+          <t>concentrated customers (small number of large mining clients); pure B2B contractor; recent acquisition (Fredon, Oct 2025); single-country revenue</t>
+        </is>
+      </c>
+      <c r="T5" s="10" t="inlineStr">
+        <is>
+          <t>Markets 0 (Australia-centred). Buyers 1 (senior mining/energy decision makers). Story 0-1 engineering reliability, scored 0. Category 1 (mining services not on grid).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:T6"/>
+  <autoFilter ref="A3:T5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -25898,7 +26149,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce — Wave 14 (v3) — 3 new brands: 0 Yes / 2 Stretch / 1 Low-value</t>
+          <t>X05 Agriculture &amp; AgTech — Wave 14 (v3) — 3 new brands: 0 Yes / 2 Stretch / 1 Low-value</t>
         </is>
       </c>
     </row>
@@ -26016,16 +26267,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="9" t="n">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>ESW (eShopWorld)</t>
+          <t>Netafim (Orbia)</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>X05 Agriculture &amp; AgTech</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -26035,46 +26286,46 @@
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>esw.com</t>
+          <t>netafim.com</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>Dublin, Ireland</t>
+          <t>Tel Aviv, Israel (Kibbutz Hatzerim origin)</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>Wholly owned by Asendia (JV of Swiss Post and La Poste Groupe) since 2021</t>
+          <t>Orbia (Mexico, NYSE-listed parent) 80%, Kibbutz Hatzerim 20%; controlling stake under sale, no deal closed</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>Cross-border e-commerce platform and logistics for global brands (200+ markets)</t>
+          <t>Drip and precision-irrigation systems and digital agronomy in 110+ countries</t>
         </is>
       </c>
       <c r="J4" s="9" t="inlineStr">
         <is>
-          <t>201-1k</t>
+          <t>1k-5k</t>
         </is>
       </c>
       <c r="K4" s="9" t="inlineStr">
         <is>
-          <t>About EUR 1B annualised revenue (Silicon Republic, Oct 2020/2021); more recent revenue not confirmed</t>
+          <t>Annual revenue &gt;$1B, ~$250M (about 25%) in US (Calcalist/ynet, Feb 2026); segment revenue reportedly down 3 consecutive years (prior hint)</t>
         </is>
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Industry sources valued it above EUR 1B at the 2021 Asendia buy-out (Silicon Republic/Business &amp; Finance, 2021); no current valuation</t>
+          <t>Reported EV ~$1.2B (asking ~$1.4B), vs $1.8B paid by Orbia in 2017 (Calcalist, Aug 2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>None; Asendia bought remaining stake from founder Thomas Kelly in 2021 (WWD, 2021)</t>
+          <t>none; 2026 sale process: Chinese (Dayu/Hopu) bid hit regulatory hurdles, Fortissimo talks froze, Spanish bidder at ~$1.4B (Calcalist, Aug 2026)</t>
         </is>
       </c>
       <c r="N4" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O4" s="9" t="inlineStr">
         <is>
@@ -26088,22 +26339,22 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Hard filters pass: dated valuation estimate above EUR 1B (2021), about 900 staff, around EUR 1B revenue, no F1 tie, not sanctioned. One reservation: the valuation is stale and ESW is a subsidiary of a state-owned JV, so spend authority and current financial health are unconfirmed.</t>
+          <t>Passes hard filters (EV ~$1.2-1.4B reported 2026, ~4,500 staff, revenue &gt;$1B, no F1 tie found for Netafim or Orbia). Real reservation: control is being sold by a financially stressed parent, so budget authority and marketing priority are uncertain. Parent distress is not Netafim distress, so not hardened to No.</t>
         </is>
       </c>
       <c r="R4" s="9" t="inlineStr">
         <is>
-          <t>B2B brand play: trackside hospitality at European and North American races for the brands ESW wants as clients (fashion, consumer electronics), pitched as a 'global ambition' partner in cross-border commerce (est).</t>
+          <t>Wait for new owner; then pitch precision-irrigation 'water-efficiency engineering' sustainability partnership at US/Miami or Spanish GP hospitality (est).</t>
         </is>
       </c>
       <c r="S4" s="9" t="inlineStr">
         <is>
-          <t>state-linked parent (Asendia owned by Swiss Post and La Poste Groupe); valuation is a 2021 press estimate; up to 45 Dublin roles cut Apr 2025 (Irish Times); subsidiary: budget approval may sit with Asendia; 906 staff (Apr 2025)</t>
+          <t>ownership change pending (sale of control in progress); parent Orbia under financial pressure; valuation only modestly above $1B and falling; declining revenue (prior hint); possible Chinese buyer, regulatory risk</t>
         </is>
       </c>
       <c r="T4" s="9" t="inlineStr">
         <is>
-          <t>Sells across 200+ markets (1); buyers are senior retail/brand decision makers (1); global ambition and technology story (1); category (cross-border e-commerce) not on grid (1). No F1 tie found for ESW, Asendia, Swiss Post or La Poste.</t>
+          <t>Markets 1 (110+ countries, US, India, Europe). Buyers 0 (growers, not affluent urban 25-54; B2B decision makers weak). Story 1 (precision, technology, water). Category 1 (irrigation not on grid). Scored 3 incl. B2B senior buyers loosely.</t>
         </is>
       </c>
     </row>
@@ -26112,16 +26363,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="9" t="n">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Pivot Bio</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>X05 Agriculture &amp; AgTech</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -26131,46 +26382,46 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>target.com</t>
+          <t>pivotbio.com</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>Minneapolis, Minnesota, USA</t>
+          <t>Minnetonka, Minnesota, USA (HQ moved from Berkeley)</t>
         </is>
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>Public (NYSE: TGT)</t>
+          <t>Private, venture-backed</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
-          <t>General merchandise and grocery through ~1,900 US stores and digital; US only</t>
+          <t>Microbial nitrogen products for corn, wheat and sorghum farmers (PROVEN 40 etc.)</t>
         </is>
       </c>
       <c r="J5" s="9" t="inlineStr">
         <is>
-          <t>10k+</t>
+          <t>201-1k</t>
         </is>
       </c>
       <c r="K5" s="9" t="inlineStr">
         <is>
-          <t>Q2 FY2026 net sales $26.5B (+5.3% YoY), comp sales +3.8%, operating margin 9.6% (Target 8-K/CNBC, 19 Aug 2026)</t>
+          <t>Surpassed USD 100M revenue by 2023 (AgFunderNews, 2023); current revenue not confirmed</t>
         </is>
       </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
-          <t>Market cap $71.1B (30 Sep 2026)</t>
+          <t>USD 1.66B post-money at Series F-2 (Forge/Pivot Bio, 11 Mar 2026); USD 2.0B at Series D (Aug 2023)</t>
         </is>
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
-          <t>none (public)</t>
+          <t>USD 100M Series F-2, 11 Mar 2026 at USD 5.71/share, investors undisclosed (Forge, Pivot Bio press release, 2026)</t>
         </is>
       </c>
       <c r="N5" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O5" s="9" t="inlineStr">
         <is>
@@ -26184,22 +26435,22 @@
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>Passes hard filters: $71.1B market cap, 10k+ staff, Q2 2026 sales and margin both improving, no F1 tie found. Capacity gate judged as passed because cuts are modest reallocation, not distress, but this is the reservation, plus fit 2 with weak angles. Prior capacity rejection not upheld.</t>
+          <t>Hard filters pass: valuation USD 1.66B (Mar 2026), about 310 staff, USD 100M raised Mar 2026 (within 24 months), no F1 tie, not sanctioned. One real reservation: capacity doubt, since 2025 layoffs and a down round suggest cost discipline and the farmer audience limits F1 relevance.</t>
         </is>
       </c>
       <c r="R5" s="9" t="inlineStr">
         <is>
-          <t>US-only Miami or Austin GP: licensed collaboration capsule or family fan-zone retail presence (est); needs a US-market-only rights package.</t>
+          <t>Sustainability-and-technology story for US/Canada/Brazil/Mexico race weekends: a hospitality and content package aimed at ag retailers, co-ops and grain-company decision makers, positioned as precision biology (est).</t>
         </is>
       </c>
       <c r="S5" s="9" t="inlineStr">
         <is>
-          <t>corporate job cuts: ~1,800 roles Oct 2025, ~500 roles Feb 2026 (Fast Company); turnaround in progress, upgraded by HSBC 3 Oct 2026; US-only</t>
+          <t>valuation down round: USD 2.0B (2023) to USD 1.66B (2026); 62 layoffs (about 20%) and Berkeley R&amp;D relocation, May-Jun 2025; B2B ag brand with farmer audience; 310 employees (ZoomInfo/Trueup, 2026)</t>
         </is>
       </c>
       <c r="T5" s="9" t="inlineStr">
         <is>
-          <t>Markets 0 (US only). Buyers 1 (core shoppers 25-54 with above-average household income vs mass retail, est). Story 0. Category 1 (mass retail not on grid). Weak angles.</t>
+          <t>Sells in 3+ F1 markets: US, Canada, Brazil (1, est, not re-verified). Buyers are farm owners/ag retailers, mostly not affluent 25-54 consumers (0). Biology and machine-learning technology story (1). Category not on grid (1). No F1 or motorsport tie found.</t>
         </is>
       </c>
     </row>
@@ -26208,65 +26459,65 @@
         <v>3</v>
       </c>
       <c r="B6" s="10" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Kobe Bussan</t>
+          <t>PI Industries</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>X05 Agriculture &amp; AgTech</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>kobebussan.co.jp</t>
+          <t>piindustries.com</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>Kakogawa, Japan</t>
+          <t>Udaipur, Rajasthan, India</t>
         </is>
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>Listed (TSE 3038)</t>
+          <t>Public (NSE/BSE: PIIND); promoter-led (Mehra family)</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr">
         <is>
-          <t>Gyomu Super discount supermarket franchise (~1,144 stores), private-label foods</t>
+          <t>Custom synthesis and manufacturing (CSM, ~76% of revenue) for global agrochemical innovators plus domestic agrochemicals and Plant Health brands</t>
         </is>
       </c>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>1k-5k</t>
+          <t>5k-10k</t>
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>~USD 3.72B TTM to 30-Apr-2026 (companiesmarketcap); FY Oct-2026 net sales forecast JPY 566.5B (+2.7%)</t>
+          <t>FY26 (to Mar 2026) revenue INR 6,714-7,024 crore (~USD 770-800M est), down from INR 8,322 crore FY25; net profit INR 1,321 crore vs 1,660 crore (Axis/StockAnalysis, Oct 2026)</t>
         </is>
       </c>
       <c r="L6" s="10" t="inlineStr">
         <is>
-          <t>Market cap ~USD 3.90B (Aug 2026, companiesmarketcap); JPY 670B (30-Sep-2026, stockanalysis)</t>
+          <t>Market cap INR 34,061 crore (~USD 3.9B est at ~87.5 INR/USD) as of 5 Oct 2026 (companiesmarketcap); 6,353 employees (same)</t>
         </is>
       </c>
       <c r="M6" s="10" t="inlineStr">
         <is>
-          <t>n/a (listed, no raise)</t>
+          <t>none (public)</t>
         </is>
       </c>
       <c r="N6" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O6" s="10" t="inlineStr">
         <is>
@@ -26280,22 +26531,22 @@
       </c>
       <c r="Q6" s="10" t="inlineStr">
         <is>
-          <t>Passes hard filters (~USD 3.9B cap, no F1 tie) but fit 1: domestic discount grocery with no overseas market overlap or F1-type brand story.</t>
+          <t>All hard filters pass (market cap ~USD 3.9B, 6,353 staff, profitable, no F1 tie found). But the core is B2B contract manufacturing for ~20 innovators with no brand ambition, revenue and profit are falling, and fit is only 2; domestic Plant Health brands target farmers, not an F1 audience.</t>
         </is>
       </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
-          <t>Little credible angle; at most a Japan GP local-market promotion (est).</t>
+          <t>Singapore or Abu Dhabi GP client hospitality for global agrochemical innovator executives (est); India-focused brand play has no F1 race to anchor.</t>
         </is>
       </c>
       <c r="S6" s="10" t="inlineStr">
         <is>
-          <t>no F1 tie found; sales growth ~5% H1 FY2026, not a growth spurt; employees 2,955 (some sources 1,600-1,700)</t>
+          <t>concentrated customers (~20 global innovators, 18 of top 20); revenue down ~16% in FY26; profit down 20%; pure B2B CSM core</t>
         </is>
       </c>
       <c r="T6" s="10" t="inlineStr">
         <is>
-          <t>Markets 0 (essentially Japan-only retail); affluent 0 (value shoppers); story 0; category 1 (discount grocery not on grid).</t>
+          <t>Markets 1 (exports to US, Europe, Japan, plus India; est). Buyers 0 (farmers; innovator procurement). Story 0-1. Category 1. Scored 2.</t>
         </is>
       </c>
     </row>
@@ -26311,7 +26562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T5"/>
+  <dimension ref="A1:T6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -26339,7 +26590,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>X09 Maritime, Shipping &amp; Ports — Wave 14 (v3) — 2 new brands: 0 Yes / 0 Stretch / 2 Low-value</t>
+          <t>X06 Retail &amp; E-commerce — Wave 14 (v3) — 3 new brands: 0 Yes / 2 Stretch / 1 Low-value</t>
         </is>
       </c>
     </row>
@@ -26453,199 +26704,295 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="n">
+      <c r="A4" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="C4" s="10" t="inlineStr">
-        <is>
-          <t>Frontline plc</t>
-        </is>
-      </c>
-      <c r="D4" s="10" t="inlineStr">
-        <is>
-          <t>X09 Maritime, Shipping &amp; Ports</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="B4" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>ESW (eShopWorld)</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>X06 Retail &amp; E-commerce</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>frontline.bm</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="inlineStr">
-        <is>
-          <t>Limassol, Cyprus</t>
-        </is>
-      </c>
-      <c r="H4" s="10" t="inlineStr">
-        <is>
-          <t>Public (NYSE/Oslo: FRO); controlled by John Fredriksen</t>
-        </is>
-      </c>
-      <c r="I4" s="10" t="inlineStr">
-        <is>
-          <t>Crude and product tanker transportation, 77-vessel fleet (40 VLCC, 19 Suezmax, 18 Aframax/LR2) chartered to oil majors and traders</t>
-        </is>
-      </c>
-      <c r="J4" s="10" t="inlineStr">
-        <is>
-          <t>51-200</t>
-        </is>
-      </c>
-      <c r="K4" s="10" t="inlineStr">
-        <is>
-          <t>Q2 2026 profit $659.2M, best-ever quarter, record TCE rates (Q2 2026 call, 28 Aug 2026)</t>
-        </is>
-      </c>
-      <c r="L4" s="10" t="inlineStr">
-        <is>
-          <t>Market cap ~USD 11.45B per StockAnalysis Q2 2026 listing; NOK 76.9B (~USD 7.5B est) at 30 Jun 2026; 85 employees</t>
-        </is>
-      </c>
-      <c r="M4" s="10" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="N4" s="10" t="n">
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>esw.com</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>Dublin, Ireland</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>Wholly owned by Asendia (JV of Swiss Post and La Poste Groupe) since 2021</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>Cross-border e-commerce platform and logistics for global brands (200+ markets)</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>201-1k</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>About EUR 1B annualised revenue (Silicon Republic, Oct 2020/2021); more recent revenue not confirmed</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>Industry sources valued it above EUR 1B at the 2021 Asendia buy-out (Silicon Republic/Business &amp; Finance, 2021); no current valuation</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>None; Asendia bought remaining stake from founder Thomas Kelly in 2021 (WWD, 2021)</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="P4" s="9" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>Hard filters pass: dated valuation estimate above EUR 1B (2021), about 900 staff, around EUR 1B revenue, no F1 tie, not sanctioned. One reservation: the valuation is stale and ESW is a subsidiary of a state-owned JV, so spend authority and current financial health are unconfirmed.</t>
+        </is>
+      </c>
+      <c r="R4" s="9" t="inlineStr">
+        <is>
+          <t>B2B brand play: trackside hospitality at European and North American races for the brands ESW wants as clients (fashion, consumer electronics), pitched as a 'global ambition' partner in cross-border commerce (est).</t>
+        </is>
+      </c>
+      <c r="S4" s="9" t="inlineStr">
+        <is>
+          <t>state-linked parent (Asendia owned by Swiss Post and La Poste Groupe); valuation is a 2021 press estimate; up to 45 Dublin roles cut Apr 2025 (Irish Times); subsidiary: budget approval may sit with Asendia; 906 staff (Apr 2025)</t>
+        </is>
+      </c>
+      <c r="T4" s="9" t="inlineStr">
+        <is>
+          <t>Sells across 200+ markets (1); buyers are senior retail/brand decision makers (1); global ambition and technology story (1); category (cross-border e-commerce) not on grid (1). No F1 tie found for ESW, Asendia, Swiss Post or La Poste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="O4" s="10" t="inlineStr">
+      <c r="B5" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>X06 Retail &amp; E-commerce</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>target.com</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Minneapolis, Minnesota, USA</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>Public (NYSE: TGT)</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>General merchandise and grocery through ~1,900 US stores and digital; US only</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>Q2 FY2026 net sales $26.5B (+5.3% YoY), comp sales +3.8%, operating margin 9.6% (Target 8-K/CNBC, 19 Aug 2026)</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>Market cap $71.1B (30 Sep 2026)</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>none (public)</t>
+        </is>
+      </c>
+      <c r="N5" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="O5" s="9" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="P4" s="10" t="inlineStr">
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>Passes hard filters: $71.1B market cap, 10k+ staff, Q2 2026 sales and margin both improving, no F1 tie found. Capacity gate judged as passed because cuts are modest reallocation, not distress, but this is the reservation, plus fit 2 with weak angles. Prior capacity rejection not upheld.</t>
+        </is>
+      </c>
+      <c r="R5" s="9" t="inlineStr">
+        <is>
+          <t>US-only Miami or Austin GP: licensed collaboration capsule or family fan-zone retail presence (est); needs a US-market-only rights package.</t>
+        </is>
+      </c>
+      <c r="S5" s="9" t="inlineStr">
+        <is>
+          <t>corporate job cuts: ~1,800 roles Oct 2025, ~500 roles Feb 2026 (Fast Company); turnaround in progress, upgraded by HSBC 3 Oct 2026; US-only</t>
+        </is>
+      </c>
+      <c r="T5" s="9" t="inlineStr">
+        <is>
+          <t>Markets 0 (US only). Buyers 1 (core shoppers 25-54 with above-average household income vs mass retail, est). Story 0. Category 1 (mass retail not on grid). Weak angles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Kobe Bussan</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>X06 Retail &amp; E-commerce</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>kobebussan.co.jp</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>Kakogawa, Japan</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>Listed (TSE 3038)</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>Gyomu Super discount supermarket franchise (~1,144 stores), private-label foods</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>~USD 3.72B TTM to 30-Apr-2026 (companiesmarketcap); FY Oct-2026 net sales forecast JPY 566.5B (+2.7%)</t>
+        </is>
+      </c>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>Market cap ~USD 3.90B (Aug 2026, companiesmarketcap); JPY 670B (30-Sep-2026, stockanalysis)</t>
+        </is>
+      </c>
+      <c r="M6" s="10" t="inlineStr">
+        <is>
+          <t>n/a (listed, no raise)</t>
+        </is>
+      </c>
+      <c r="N6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" s="10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="P6" s="10" t="inlineStr">
         <is>
           <t>Low-value</t>
         </is>
       </c>
-      <c r="Q4" s="10" t="inlineStr">
-        <is>
-          <t>Passes hard filters (large market cap, 85 staff within 51+, record profit, no F1 tie found, not sanctioned per search). But it is a pure B2B tanker owner with concentrated counterparties, minimal marketing function and no brand ambition; fit 2.</t>
-        </is>
-      </c>
-      <c r="R4" s="10" t="inlineStr">
-        <is>
-          <t>Monaco or Abu Dhabi GP entertainment for charterer executives (est); very low odds as Frontline does not advertise.</t>
-        </is>
-      </c>
-      <c r="S4" s="10" t="inlineStr">
-        <is>
-          <t>concentrated customers (oil majors and trading houses); cyclical earnings at record high; pure B2B; controlled by single billionaire</t>
-        </is>
-      </c>
-      <c r="T4" s="10" t="inlineStr">
-        <is>
-          <t>Markets 0 (B2B shipping, not sold to consumers). Buyers 1 (oil major executives). Story 0. Category 1 (tankers not on grid).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="10" t="n">
-        <v>24</v>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>Seaspan (Atlas Corp.)</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>X09 Maritime, Shipping &amp; Ports</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>seaspancorp.com</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>Hong Kong / Vancouver, Canada (Atlas, Poseidon-owned)</t>
-        </is>
-      </c>
-      <c r="H5" s="10" t="inlineStr">
-        <is>
-          <t>Private since 2023: Poseidon consortium (Washington family, Fairfax, Ocean Network Express, David Sokol); Fairfax sold 23.2% of Poseidon for $1.91B in Mar 2026</t>
-        </is>
-      </c>
-      <c r="I5" s="10" t="inlineStr">
-        <is>
-          <t>Container ships on long-term charter (180+ vessels, ~9 liner customers) and marine services through Seaspan ULC</t>
-        </is>
-      </c>
-      <c r="J5" s="10" t="inlineStr">
-        <is>
-          <t>5k-10k</t>
-        </is>
-      </c>
-      <c r="K5" s="10" t="inlineStr">
-        <is>
-          <t>Atlas 2024 revenue $2,300.1M (Atlas 20-F, Mar 2025)</t>
-        </is>
-      </c>
-      <c r="L5" s="10" t="inlineStr">
-        <is>
-          <t>Take-private EV ~$10.9B (2023, Seatrade); Poseidon equity ~USD 8.2B est (Fairfax sale at $28.30/sh for 23.2%, Mar 2026)</t>
-        </is>
-      </c>
-      <c r="M5" s="10" t="inlineStr">
-        <is>
-          <t>Mar 2026 secondary: Fairfax sold 67.6M Poseidon shares for $1.91B (The Insurer)</t>
-        </is>
-      </c>
-      <c r="N5" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="O5" s="10" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="P5" s="10" t="inlineStr">
-        <is>
-          <t>Low-value</t>
-        </is>
-      </c>
-      <c r="Q5" s="10" t="inlineStr">
-        <is>
-          <t>Passes hard filters (EV $10.9B, ~6,200 staff, $2.3B revenue, no F1 tie found for Seaspan, Atlas, Poseidon or ONE). But it is a pure B2B ship-lessor with nine customers and no brand ambition; fit 1. Prior concentration rejection is now a flag only.</t>
-        </is>
-      </c>
-      <c r="R5" s="10" t="inlineStr">
-        <is>
-          <t>None credible; at most Canadian GP (Montreal) charterer hospitality (est). Not worth outreach effort.</t>
-        </is>
-      </c>
-      <c r="S5" s="10" t="inlineStr">
-        <is>
-          <t>concentrated customers (nine liner companies); pure B2B; partial ownership change Mar 2026 (secondary stake sale)</t>
-        </is>
-      </c>
-      <c r="T5" s="10" t="inlineStr">
-        <is>
-          <t>Markets 0 (B2B charter). Buyers 0. Story 0-1. Category 1. Scored 1.</t>
+      <c r="Q6" s="10" t="inlineStr">
+        <is>
+          <t>Passes hard filters (~USD 3.9B cap, no F1 tie) but fit 1: domestic discount grocery with no overseas market overlap or F1-type brand story.</t>
+        </is>
+      </c>
+      <c r="R6" s="10" t="inlineStr">
+        <is>
+          <t>Little credible angle; at most a Japan GP local-market promotion (est).</t>
+        </is>
+      </c>
+      <c r="S6" s="10" t="inlineStr">
+        <is>
+          <t>no F1 tie found; sales growth ~5% H1 FY2026, not a growth spurt; employees 2,955 (some sources 1,600-1,700)</t>
+        </is>
+      </c>
+      <c r="T6" s="10" t="inlineStr">
+        <is>
+          <t>Markets 0 (essentially Japan-only retail); affluent 0 (value shoppers); story 0; category 1 (discount grocery not on grid).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:T5"/>
+  <autoFilter ref="A3:T6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Wave 14 v3: cycle rebuild (241 verified)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TE8a9ptd2NGPUtY6iZfzkb
</commit_message>
<xml_diff>
--- a/reports/F1-Wave14-V3-Broad-2026-10.xlsx
+++ b/reports/F1-Wave14-V3-Broad-2026-10.xlsx
@@ -46175,12 +46175,12 @@
     <row r="925">
       <c r="A925" s="4" t="inlineStr">
         <is>
-          <t>Motive (formerly KeepTruckin)</t>
+          <t>Nominal</t>
         </is>
       </c>
       <c r="B925" s="4" t="inlineStr">
         <is>
-          <t>24 Logistics</t>
+          <t>X07 Aviation &amp; Aerospace Suppliers</t>
         </is>
       </c>
       <c r="C925" s="4" t="inlineStr">
@@ -46192,12 +46192,12 @@
     <row r="926">
       <c r="A926" s="4" t="inlineStr">
         <is>
-          <t>Nominal</t>
+          <t>Fruitist</t>
         </is>
       </c>
       <c r="B926" s="4" t="inlineStr">
         <is>
-          <t>X07 Aviation &amp; Aerospace Suppliers</t>
+          <t>43 Mobility &amp; Automotive</t>
         </is>
       </c>
       <c r="C926" s="4" t="inlineStr">
@@ -46209,12 +46209,12 @@
     <row r="927">
       <c r="A927" s="4" t="inlineStr">
         <is>
-          <t>Fruitist</t>
+          <t>Zaxby's</t>
         </is>
       </c>
       <c r="B927" s="4" t="inlineStr">
         <is>
-          <t>43 Mobility &amp; Automotive</t>
+          <t>53 Consumer &amp; Lifestyle</t>
         </is>
       </c>
       <c r="C927" s="4" t="inlineStr">
@@ -46226,12 +46226,12 @@
     <row r="928">
       <c r="A928" s="4" t="inlineStr">
         <is>
-          <t>Zaxby's</t>
+          <t>Ziff Davis</t>
         </is>
       </c>
       <c r="B928" s="4" t="inlineStr">
         <is>
-          <t>53 Consumer &amp; Lifestyle</t>
+          <t>29 Tech Media &amp; Gaming</t>
         </is>
       </c>
       <c r="C928" s="4" t="inlineStr">
@@ -46243,12 +46243,12 @@
     <row r="929">
       <c r="A929" s="4" t="inlineStr">
         <is>
-          <t>Ziff Davis</t>
+          <t>Ninja</t>
         </is>
       </c>
       <c r="B929" s="4" t="inlineStr">
         <is>
-          <t>29 Tech Media &amp; Gaming</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C929" s="4" t="inlineStr">
@@ -46260,12 +46260,12 @@
     <row r="930">
       <c r="A930" s="4" t="inlineStr">
         <is>
-          <t>Ninja</t>
+          <t>Grindr</t>
         </is>
       </c>
       <c r="B930" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>29 Tech Media &amp; Gaming</t>
         </is>
       </c>
       <c r="C930" s="4" t="inlineStr">
@@ -46277,12 +46277,12 @@
     <row r="931">
       <c r="A931" s="4" t="inlineStr">
         <is>
-          <t>Grindr</t>
+          <t>Kitopi</t>
         </is>
       </c>
       <c r="B931" s="4" t="inlineStr">
         <is>
-          <t>29 Tech Media &amp; Gaming</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C931" s="4" t="inlineStr">
@@ -46294,12 +46294,12 @@
     <row r="932">
       <c r="A932" s="4" t="inlineStr">
         <is>
-          <t>Kitopi</t>
+          <t>MoonActive</t>
         </is>
       </c>
       <c r="B932" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>29 Tech Media &amp; Gaming</t>
         </is>
       </c>
       <c r="C932" s="4" t="inlineStr">
@@ -46311,12 +46311,12 @@
     <row r="933">
       <c r="A933" s="4" t="inlineStr">
         <is>
-          <t>MoonActive</t>
+          <t>Too Good To Go</t>
         </is>
       </c>
       <c r="B933" s="4" t="inlineStr">
         <is>
-          <t>29 Tech Media &amp; Gaming</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C933" s="4" t="inlineStr">
@@ -46328,12 +46328,12 @@
     <row r="934">
       <c r="A934" s="4" t="inlineStr">
         <is>
-          <t>Too Good To Go</t>
+          <t>Asmodee Group</t>
         </is>
       </c>
       <c r="B934" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>29 Tech Media &amp; Gaming</t>
         </is>
       </c>
       <c r="C934" s="4" t="inlineStr">
@@ -46345,12 +46345,12 @@
     <row r="935">
       <c r="A935" s="4" t="inlineStr">
         <is>
-          <t>Asmodee Group</t>
+          <t>Glossier</t>
         </is>
       </c>
       <c r="B935" s="4" t="inlineStr">
         <is>
-          <t>29 Tech Media &amp; Gaming</t>
+          <t>03 Luxury &amp; Beauty</t>
         </is>
       </c>
       <c r="C935" s="4" t="inlineStr">
@@ -46362,12 +46362,12 @@
     <row r="936">
       <c r="A936" s="4" t="inlineStr">
         <is>
-          <t>Glossier</t>
+          <t>Outdoorsy</t>
         </is>
       </c>
       <c r="B936" s="4" t="inlineStr">
         <is>
-          <t>03 Luxury &amp; Beauty</t>
+          <t>16 Travel &amp; Hospitality</t>
         </is>
       </c>
       <c r="C936" s="4" t="inlineStr">
@@ -46379,29 +46379,29 @@
     <row r="937">
       <c r="A937" s="4" t="inlineStr">
         <is>
-          <t>Outdoorsy</t>
+          <t>Banamex (Citibanamex)</t>
         </is>
       </c>
       <c r="B937" s="4" t="inlineStr">
         <is>
-          <t>16 Travel &amp; Hospitality</t>
+          <t>01 Banking &amp; Insurance</t>
         </is>
       </c>
       <c r="C937" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
     </row>
     <row r="938">
       <c r="A938" s="4" t="inlineStr">
         <is>
-          <t>Banamex (Citibanamex)</t>
+          <t>Aeromexico</t>
         </is>
       </c>
       <c r="B938" s="4" t="inlineStr">
         <is>
-          <t>01 Banking &amp; Insurance</t>
+          <t>16 Travel &amp; Hospitality</t>
         </is>
       </c>
       <c r="C938" s="4" t="inlineStr">
@@ -46413,7 +46413,7 @@
     <row r="939">
       <c r="A939" s="4" t="inlineStr">
         <is>
-          <t>Aeromexico</t>
+          <t>Grupo Aeroportuario del Pacifico</t>
         </is>
       </c>
       <c r="B939" s="4" t="inlineStr">
@@ -46430,12 +46430,12 @@
     <row r="940">
       <c r="A940" s="4" t="inlineStr">
         <is>
-          <t>Grupo Aeroportuario del Pacifico</t>
+          <t>Cemex</t>
         </is>
       </c>
       <c r="B940" s="4" t="inlineStr">
         <is>
-          <t>16 Travel &amp; Hospitality</t>
+          <t>X02 Real Estate &amp; Building Produ</t>
         </is>
       </c>
       <c r="C940" s="4" t="inlineStr">
@@ -46447,12 +46447,12 @@
     <row r="941">
       <c r="A941" s="4" t="inlineStr">
         <is>
-          <t>Cemex</t>
+          <t>Liverpool (El Puerto de Liverpool)</t>
         </is>
       </c>
       <c r="B941" s="4" t="inlineStr">
         <is>
-          <t>X02 Real Estate &amp; Building Produ</t>
+          <t>X41 LatAm Consumer &amp; Retail Champions</t>
         </is>
       </c>
       <c r="C941" s="4" t="inlineStr">
@@ -46464,7 +46464,7 @@
     <row r="942">
       <c r="A942" s="4" t="inlineStr">
         <is>
-          <t>Liverpool (El Puerto de Liverpool)</t>
+          <t>Coppel</t>
         </is>
       </c>
       <c r="B942" s="4" t="inlineStr">
@@ -46481,7 +46481,7 @@
     <row r="943">
       <c r="A943" s="4" t="inlineStr">
         <is>
-          <t>Coppel</t>
+          <t>Grupo Salinas</t>
         </is>
       </c>
       <c r="B943" s="4" t="inlineStr">
@@ -46498,12 +46498,12 @@
     <row r="944">
       <c r="A944" s="4" t="inlineStr">
         <is>
-          <t>Grupo Salinas</t>
+          <t>Cinepolis</t>
         </is>
       </c>
       <c r="B944" s="4" t="inlineStr">
         <is>
-          <t>X41 LatAm Consumer &amp; Retail Champions</t>
+          <t>X24 Ticketing, Live Events &amp; Experiences</t>
         </is>
       </c>
       <c r="C944" s="4" t="inlineStr">
@@ -46515,12 +46515,12 @@
     <row r="945">
       <c r="A945" s="4" t="inlineStr">
         <is>
-          <t>Cinepolis</t>
+          <t>Kimberly-Clark de Mexico</t>
         </is>
       </c>
       <c r="B945" s="4" t="inlineStr">
         <is>
-          <t>X24 Ticketing, Live Events &amp; Experiences</t>
+          <t>53 Consumer &amp; Lifestyle</t>
         </is>
       </c>
       <c r="C945" s="4" t="inlineStr">
@@ -46532,12 +46532,12 @@
     <row r="946">
       <c r="A946" s="4" t="inlineStr">
         <is>
-          <t>Kimberly-Clark de Mexico</t>
+          <t>Empresas Copec</t>
         </is>
       </c>
       <c r="B946" s="4" t="inlineStr">
         <is>
-          <t>53 Consumer &amp; Lifestyle</t>
+          <t>02 Energy &amp; Industrial</t>
         </is>
       </c>
       <c r="C946" s="4" t="inlineStr">
@@ -46549,12 +46549,12 @@
     <row r="947">
       <c r="A947" s="4" t="inlineStr">
         <is>
-          <t>Empresas Copec</t>
+          <t>easyJet</t>
         </is>
       </c>
       <c r="B947" s="4" t="inlineStr">
         <is>
-          <t>02 Energy &amp; Industrial</t>
+          <t>16 Travel &amp; Hospitality</t>
         </is>
       </c>
       <c r="C947" s="4" t="inlineStr">
@@ -46566,7 +46566,7 @@
     <row r="948">
       <c r="A948" s="4" t="inlineStr">
         <is>
-          <t>easyJet</t>
+          <t>Ryanair</t>
         </is>
       </c>
       <c r="B948" s="4" t="inlineStr">
@@ -46583,7 +46583,7 @@
     <row r="949">
       <c r="A949" s="4" t="inlineStr">
         <is>
-          <t>Ryanair</t>
+          <t>Aena</t>
         </is>
       </c>
       <c r="B949" s="4" t="inlineStr">
@@ -46600,7 +46600,7 @@
     <row r="950">
       <c r="A950" s="4" t="inlineStr">
         <is>
-          <t>Aena</t>
+          <t>IHG Hotels and Resorts</t>
         </is>
       </c>
       <c r="B950" s="4" t="inlineStr">
@@ -46617,12 +46617,12 @@
     <row r="951">
       <c r="A951" s="4" t="inlineStr">
         <is>
-          <t>IHG Hotels and Resorts</t>
+          <t>Elis</t>
         </is>
       </c>
       <c r="B951" s="4" t="inlineStr">
         <is>
-          <t>16 Travel &amp; Hospitality</t>
+          <t>18 Services &amp; Other</t>
         </is>
       </c>
       <c r="C951" s="4" t="inlineStr">
@@ -46634,12 +46634,12 @@
     <row r="952">
       <c r="A952" s="4" t="inlineStr">
         <is>
-          <t>Elis</t>
+          <t>Publicis Groupe</t>
         </is>
       </c>
       <c r="B952" s="4" t="inlineStr">
         <is>
-          <t>18 Services &amp; Other</t>
+          <t>07 Marketing &amp; Sales</t>
         </is>
       </c>
       <c r="C952" s="4" t="inlineStr">
@@ -46651,12 +46651,12 @@
     <row r="953">
       <c r="A953" s="4" t="inlineStr">
         <is>
-          <t>Publicis Groupe</t>
+          <t>Deutsche Telekom</t>
         </is>
       </c>
       <c r="B953" s="4" t="inlineStr">
         <is>
-          <t>07 Marketing &amp; Sales</t>
+          <t>48 Telecom &amp; Space</t>
         </is>
       </c>
       <c r="C953" s="4" t="inlineStr">
@@ -46668,7 +46668,7 @@
     <row r="954">
       <c r="A954" s="4" t="inlineStr">
         <is>
-          <t>Deutsche Telekom</t>
+          <t>Cellnex</t>
         </is>
       </c>
       <c r="B954" s="4" t="inlineStr">
@@ -46685,12 +46685,12 @@
     <row r="955">
       <c r="A955" s="4" t="inlineStr">
         <is>
-          <t>Cellnex</t>
+          <t>Compagnie Financiere Richemont</t>
         </is>
       </c>
       <c r="B955" s="4" t="inlineStr">
         <is>
-          <t>48 Telecom &amp; Space</t>
+          <t>X21 Watches &amp; Jewellery</t>
         </is>
       </c>
       <c r="C955" s="4" t="inlineStr">
@@ -46702,12 +46702,12 @@
     <row r="956">
       <c r="A956" s="4" t="inlineStr">
         <is>
-          <t>Compagnie Financiere Richemont</t>
+          <t>Tulip Retail</t>
         </is>
       </c>
       <c r="B956" s="4" t="inlineStr">
         <is>
-          <t>X21 Watches &amp; Jewellery</t>
+          <t>47 Vertical SaaS</t>
         </is>
       </c>
       <c r="C956" s="4" t="inlineStr">
@@ -46719,7 +46719,7 @@
     <row r="957">
       <c r="A957" s="4" t="inlineStr">
         <is>
-          <t>Tulip Retail</t>
+          <t>Visier</t>
         </is>
       </c>
       <c r="B957" s="4" t="inlineStr">
@@ -46736,7 +46736,7 @@
     <row r="958">
       <c r="A958" s="4" t="inlineStr">
         <is>
-          <t>Visier</t>
+          <t>Jane App</t>
         </is>
       </c>
       <c r="B958" s="4" t="inlineStr">
@@ -46753,12 +46753,12 @@
     <row r="959">
       <c r="A959" s="4" t="inlineStr">
         <is>
-          <t>Jane App</t>
+          <t>Benevity</t>
         </is>
       </c>
       <c r="B959" s="4" t="inlineStr">
         <is>
-          <t>47 Vertical SaaS</t>
+          <t>22 SaaS</t>
         </is>
       </c>
       <c r="C959" s="4" t="inlineStr">
@@ -46770,12 +46770,12 @@
     <row r="960">
       <c r="A960" s="4" t="inlineStr">
         <is>
-          <t>Benevity</t>
+          <t>GeoComply</t>
         </is>
       </c>
       <c r="B960" s="4" t="inlineStr">
         <is>
-          <t>22 SaaS</t>
+          <t>31 GRC &amp; Risk SW</t>
         </is>
       </c>
       <c r="C960" s="4" t="inlineStr">
@@ -46787,12 +46787,12 @@
     <row r="961">
       <c r="A961" s="4" t="inlineStr">
         <is>
-          <t>GeoComply</t>
+          <t>Juniper Square</t>
         </is>
       </c>
       <c r="B961" s="4" t="inlineStr">
         <is>
-          <t>31 GRC &amp; Risk SW</t>
+          <t>47 Vertical SaaS</t>
         </is>
       </c>
       <c r="C961" s="4" t="inlineStr">
@@ -46804,12 +46804,12 @@
     <row r="962">
       <c r="A962" s="4" t="inlineStr">
         <is>
-          <t>Juniper Square</t>
+          <t>MX Technologies</t>
         </is>
       </c>
       <c r="B962" s="4" t="inlineStr">
         <is>
-          <t>47 Vertical SaaS</t>
+          <t>09 Fintech</t>
         </is>
       </c>
       <c r="C962" s="4" t="inlineStr">
@@ -46821,12 +46821,12 @@
     <row r="963">
       <c r="A963" s="4" t="inlineStr">
         <is>
-          <t>MX Technologies</t>
+          <t>Iterative Health</t>
         </is>
       </c>
       <c r="B963" s="4" t="inlineStr">
         <is>
-          <t>09 Fintech</t>
+          <t>42 Health &amp; Wellness</t>
         </is>
       </c>
       <c r="C963" s="4" t="inlineStr">
@@ -46838,12 +46838,12 @@
     <row r="964">
       <c r="A964" s="4" t="inlineStr">
         <is>
-          <t>Iterative Health</t>
+          <t>ezCater</t>
         </is>
       </c>
       <c r="B964" s="4" t="inlineStr">
         <is>
-          <t>42 Health &amp; Wellness</t>
+          <t>18 Services &amp; Other</t>
         </is>
       </c>
       <c r="C964" s="4" t="inlineStr">
@@ -46855,12 +46855,12 @@
     <row r="965">
       <c r="A965" s="4" t="inlineStr">
         <is>
-          <t>ezCater</t>
+          <t>Weee! (Sayweee)</t>
         </is>
       </c>
       <c r="B965" s="4" t="inlineStr">
         <is>
-          <t>18 Services &amp; Other</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C965" s="4" t="inlineStr">
@@ -46872,12 +46872,12 @@
     <row r="966">
       <c r="A966" s="4" t="inlineStr">
         <is>
-          <t>Weee! (Sayweee)</t>
+          <t>Bharat Coking Coal</t>
         </is>
       </c>
       <c r="B966" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>X04 Mining, Metals &amp; Commodities</t>
         </is>
       </c>
       <c r="C966" s="4" t="inlineStr">
@@ -46889,12 +46889,12 @@
     <row r="967">
       <c r="A967" s="4" t="inlineStr">
         <is>
-          <t>Bharat Coking Coal</t>
+          <t>WeWork India Management</t>
         </is>
       </c>
       <c r="B967" s="4" t="inlineStr">
         <is>
-          <t>X04 Mining, Metals &amp; Commodities</t>
+          <t>X02 Real Estate &amp; Building Produ</t>
         </is>
       </c>
       <c r="C967" s="4" t="inlineStr">
@@ -46906,12 +46906,12 @@
     <row r="968">
       <c r="A968" s="4" t="inlineStr">
         <is>
-          <t>WeWork India Management</t>
+          <t>SBI Funds Management</t>
         </is>
       </c>
       <c r="B968" s="4" t="inlineStr">
         <is>
-          <t>X02 Real Estate &amp; Building Produ</t>
+          <t>X01 Asset Mgmt, PE &amp; Trading Fir</t>
         </is>
       </c>
       <c r="C968" s="4" t="inlineStr">
@@ -46923,12 +46923,12 @@
     <row r="969">
       <c r="A969" s="4" t="inlineStr">
         <is>
-          <t>SBI Funds Management</t>
+          <t>HDFC Credila Financial Services</t>
         </is>
       </c>
       <c r="B969" s="4" t="inlineStr">
         <is>
-          <t>X01 Asset Mgmt, PE &amp; Trading Fir</t>
+          <t>09 Fintech</t>
         </is>
       </c>
       <c r="C969" s="4" t="inlineStr">
@@ -46940,7 +46940,7 @@
     <row r="970">
       <c r="A970" s="4" t="inlineStr">
         <is>
-          <t>HDFC Credila Financial Services</t>
+          <t>Hero FinCorp</t>
         </is>
       </c>
       <c r="B970" s="4" t="inlineStr">
@@ -46957,12 +46957,12 @@
     <row r="971">
       <c r="A971" s="4" t="inlineStr">
         <is>
-          <t>Hero FinCorp</t>
+          <t>Samsung Epis Holdings</t>
         </is>
       </c>
       <c r="B971" s="4" t="inlineStr">
         <is>
-          <t>09 Fintech</t>
+          <t>X03 CDMO, CRO &amp; Life-Science Too</t>
         </is>
       </c>
       <c r="C971" s="4" t="inlineStr">
@@ -46974,12 +46974,12 @@
     <row r="972">
       <c r="A972" s="4" t="inlineStr">
         <is>
-          <t>Samsung Epis Holdings</t>
+          <t>HD Hyundai Robotics</t>
         </is>
       </c>
       <c r="B972" s="4" t="inlineStr">
         <is>
-          <t>X03 CDMO, CRO &amp; Life-Science Too</t>
+          <t>33 Automation &amp; Robotics</t>
         </is>
       </c>
       <c r="C972" s="4" t="inlineStr">
@@ -46991,12 +46991,12 @@
     <row r="973">
       <c r="A973" s="4" t="inlineStr">
         <is>
-          <t>HD Hyundai Robotics</t>
+          <t>CXMT (ChangXin Memory Technologies)</t>
         </is>
       </c>
       <c r="B973" s="4" t="inlineStr">
         <is>
-          <t>33 Automation &amp; Robotics</t>
+          <t>27 Chip Makers</t>
         </is>
       </c>
       <c r="C973" s="4" t="inlineStr">
@@ -47008,12 +47008,12 @@
     <row r="974">
       <c r="A974" s="4" t="inlineStr">
         <is>
-          <t>CXMT (ChangXin Memory Technologies)</t>
+          <t>Haitian Flavouring and Food</t>
         </is>
       </c>
       <c r="B974" s="4" t="inlineStr">
         <is>
-          <t>27 Chip Makers</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C974" s="4" t="inlineStr">
@@ -47025,12 +47025,12 @@
     <row r="975">
       <c r="A975" s="4" t="inlineStr">
         <is>
-          <t>Haitian Flavouring and Food</t>
+          <t>Voyah Automobile</t>
         </is>
       </c>
       <c r="B975" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>43 Mobility &amp; Automotive</t>
         </is>
       </c>
       <c r="C975" s="4" t="inlineStr">
@@ -47042,12 +47042,12 @@
     <row r="976">
       <c r="A976" s="4" t="inlineStr">
         <is>
-          <t>Voyah Automobile</t>
+          <t>Dangote Petroleum Refinery</t>
         </is>
       </c>
       <c r="B976" s="4" t="inlineStr">
         <is>
-          <t>43 Mobility &amp; Automotive</t>
+          <t>02 Energy &amp; Industrial</t>
         </is>
       </c>
       <c r="C976" s="4" t="inlineStr">
@@ -47059,12 +47059,12 @@
     <row r="977">
       <c r="A977" s="4" t="inlineStr">
         <is>
-          <t>Dangote Petroleum Refinery</t>
+          <t>Agibank</t>
         </is>
       </c>
       <c r="B977" s="4" t="inlineStr">
         <is>
-          <t>02 Energy &amp; Industrial</t>
+          <t>X41 LatAm Consumer &amp; Retail Champions</t>
         </is>
       </c>
       <c r="C977" s="4" t="inlineStr">
@@ -47076,12 +47076,12 @@
     <row r="978">
       <c r="A978" s="4" t="inlineStr">
         <is>
-          <t>Agibank</t>
+          <t>Grupo Aeromexico</t>
         </is>
       </c>
       <c r="B978" s="4" t="inlineStr">
         <is>
-          <t>X41 LatAm Consumer &amp; Retail Champions</t>
+          <t>16 Travel &amp; Hospitality</t>
         </is>
       </c>
       <c r="C978" s="4" t="inlineStr">
@@ -47093,12 +47093,12 @@
     <row r="979">
       <c r="A979" s="4" t="inlineStr">
         <is>
-          <t>Grupo Aeromexico</t>
+          <t>Plenitude (Eni)</t>
         </is>
       </c>
       <c r="B979" s="4" t="inlineStr">
         <is>
-          <t>16 Travel &amp; Hospitality</t>
+          <t>02 Energy &amp; Industrial</t>
         </is>
       </c>
       <c r="C979" s="4" t="inlineStr">
@@ -47110,12 +47110,12 @@
     <row r="980">
       <c r="A980" s="4" t="inlineStr">
         <is>
-          <t>Plenitude (Eni)</t>
+          <t>DePuy Synthes (J&amp;J orthopaedics)</t>
         </is>
       </c>
       <c r="B980" s="4" t="inlineStr">
         <is>
-          <t>02 Energy &amp; Industrial</t>
+          <t>42 Health &amp; Wellness</t>
         </is>
       </c>
       <c r="C980" s="4" t="inlineStr">
@@ -47127,12 +47127,12 @@
     <row r="981">
       <c r="A981" s="4" t="inlineStr">
         <is>
-          <t>DePuy Synthes (J&amp;J orthopaedics)</t>
+          <t>Grupo Clarin</t>
         </is>
       </c>
       <c r="B981" s="4" t="inlineStr">
         <is>
-          <t>42 Health &amp; Wellness</t>
+          <t>29 Tech Media &amp; Gaming</t>
         </is>
       </c>
       <c r="C981" s="4" t="inlineStr">
@@ -47144,12 +47144,12 @@
     <row r="982">
       <c r="A982" s="4" t="inlineStr">
         <is>
-          <t>Grupo Clarin</t>
+          <t>Banco Mercantil del Norte (Banorte)</t>
         </is>
       </c>
       <c r="B982" s="4" t="inlineStr">
         <is>
-          <t>29 Tech Media &amp; Gaming</t>
+          <t>01 Banking &amp; Insurance</t>
         </is>
       </c>
       <c r="C982" s="4" t="inlineStr">
@@ -47161,12 +47161,12 @@
     <row r="983">
       <c r="A983" s="4" t="inlineStr">
         <is>
-          <t>Banco Mercantil del Norte (Banorte)</t>
+          <t>Grupo Soma</t>
         </is>
       </c>
       <c r="B983" s="4" t="inlineStr">
         <is>
-          <t>01 Banking &amp; Insurance</t>
+          <t>X41 LatAm Consumer &amp; Retail Champions</t>
         </is>
       </c>
       <c r="C983" s="4" t="inlineStr">
@@ -47178,7 +47178,7 @@
     <row r="984">
       <c r="A984" s="4" t="inlineStr">
         <is>
-          <t>Grupo Soma</t>
+          <t>Livelo</t>
         </is>
       </c>
       <c r="B984" s="4" t="inlineStr">
@@ -47195,12 +47195,12 @@
     <row r="985">
       <c r="A985" s="4" t="inlineStr">
         <is>
-          <t>Livelo</t>
+          <t>Grupo Silvio Santos</t>
         </is>
       </c>
       <c r="B985" s="4" t="inlineStr">
         <is>
-          <t>X41 LatAm Consumer &amp; Retail Champions</t>
+          <t>29 Tech Media &amp; Gaming</t>
         </is>
       </c>
       <c r="C985" s="4" t="inlineStr">
@@ -47212,12 +47212,12 @@
     <row r="986">
       <c r="A986" s="4" t="inlineStr">
         <is>
-          <t>Grupo Silvio Santos</t>
+          <t>Companhia Brasileira de Aluminio (CBA)</t>
         </is>
       </c>
       <c r="B986" s="4" t="inlineStr">
         <is>
-          <t>29 Tech Media &amp; Gaming</t>
+          <t>X04 Mining, Metals &amp; Commodities</t>
         </is>
       </c>
       <c r="C986" s="4" t="inlineStr">
@@ -47229,12 +47229,12 @@
     <row r="987">
       <c r="A987" s="4" t="inlineStr">
         <is>
-          <t>Companhia Brasileira de Aluminio (CBA)</t>
+          <t>Grupo Mateus</t>
         </is>
       </c>
       <c r="B987" s="4" t="inlineStr">
         <is>
-          <t>X04 Mining, Metals &amp; Commodities</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C987" s="4" t="inlineStr">
@@ -47246,12 +47246,12 @@
     <row r="988">
       <c r="A988" s="4" t="inlineStr">
         <is>
-          <t>Grupo Mateus</t>
+          <t>Rede D'Or Sao Luiz</t>
         </is>
       </c>
       <c r="B988" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>42 Health &amp; Wellness</t>
         </is>
       </c>
       <c r="C988" s="4" t="inlineStr">
@@ -47263,12 +47263,12 @@
     <row r="989">
       <c r="A989" s="4" t="inlineStr">
         <is>
-          <t>Rede D'Or Sao Luiz</t>
+          <t>Hapvida NotreDame Intermedica</t>
         </is>
       </c>
       <c r="B989" s="4" t="inlineStr">
         <is>
-          <t>42 Health &amp; Wellness</t>
+          <t>01 Banking &amp; Insurance</t>
         </is>
       </c>
       <c r="C989" s="4" t="inlineStr">
@@ -47280,12 +47280,12 @@
     <row r="990">
       <c r="A990" s="4" t="inlineStr">
         <is>
-          <t>Hapvida NotreDame Intermedica</t>
+          <t>WEG</t>
         </is>
       </c>
       <c r="B990" s="4" t="inlineStr">
         <is>
-          <t>01 Banking &amp; Insurance</t>
+          <t>02 Energy &amp; Industrial</t>
         </is>
       </c>
       <c r="C990" s="4" t="inlineStr">
@@ -47297,7 +47297,7 @@
     <row r="991">
       <c r="A991" s="4" t="inlineStr">
         <is>
-          <t>WEG</t>
+          <t>Cosan</t>
         </is>
       </c>
       <c r="B991" s="4" t="inlineStr">
@@ -47314,12 +47314,12 @@
     <row r="992">
       <c r="A992" s="4" t="inlineStr">
         <is>
-          <t>Cosan</t>
+          <t>Wal-Mart de Mexico (Walmex)</t>
         </is>
       </c>
       <c r="B992" s="4" t="inlineStr">
         <is>
-          <t>02 Energy &amp; Industrial</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C992" s="4" t="inlineStr">
@@ -47331,12 +47331,12 @@
     <row r="993">
       <c r="A993" s="4" t="inlineStr">
         <is>
-          <t>Wal-Mart de Mexico (Walmex)</t>
+          <t>Arca Continental</t>
         </is>
       </c>
       <c r="B993" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C993" s="4" t="inlineStr">
@@ -47348,7 +47348,7 @@
     <row r="994">
       <c r="A994" s="4" t="inlineStr">
         <is>
-          <t>Arca Continental</t>
+          <t>Gruma</t>
         </is>
       </c>
       <c r="B994" s="4" t="inlineStr">
@@ -47365,12 +47365,12 @@
     <row r="995">
       <c r="A995" s="4" t="inlineStr">
         <is>
-          <t>Gruma</t>
+          <t>Alsea</t>
         </is>
       </c>
       <c r="B995" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>X28 Franchise Groups</t>
         </is>
       </c>
       <c r="C995" s="4" t="inlineStr">
@@ -47382,24 +47382,24 @@
     <row r="996">
       <c r="A996" s="4" t="inlineStr">
         <is>
-          <t>Alsea</t>
+          <t>Redo</t>
         </is>
       </c>
       <c r="B996" s="4" t="inlineStr">
         <is>
-          <t>X28 Franchise Groups</t>
+          <t>13 AI Agents</t>
         </is>
       </c>
       <c r="C996" s="4" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="997">
       <c r="A997" s="4" t="inlineStr">
         <is>
-          <t>Redo</t>
+          <t>Insitro</t>
         </is>
       </c>
       <c r="B997" s="4" t="inlineStr">
@@ -47416,12 +47416,12 @@
     <row r="998">
       <c r="A998" s="4" t="inlineStr">
         <is>
-          <t>Insitro</t>
+          <t>Unconventional AI</t>
         </is>
       </c>
       <c r="B998" s="4" t="inlineStr">
         <is>
-          <t>13 AI Agents</t>
+          <t>17 AI Cloud &amp; Data</t>
         </is>
       </c>
       <c r="C998" s="4" t="inlineStr">
@@ -47433,7 +47433,7 @@
     <row r="999">
       <c r="A999" s="4" t="inlineStr">
         <is>
-          <t>Unconventional AI</t>
+          <t>Zama</t>
         </is>
       </c>
       <c r="B999" s="4" t="inlineStr">
@@ -47450,12 +47450,12 @@
     <row r="1000">
       <c r="A1000" s="4" t="inlineStr">
         <is>
-          <t>Zama</t>
+          <t>Immunai</t>
         </is>
       </c>
       <c r="B1000" s="4" t="inlineStr">
         <is>
-          <t>17 AI Cloud &amp; Data</t>
+          <t>13 AI Agents</t>
         </is>
       </c>
       <c r="C1000" s="4" t="inlineStr">
@@ -47467,7 +47467,7 @@
     <row r="1001">
       <c r="A1001" s="4" t="inlineStr">
         <is>
-          <t>Immunai</t>
+          <t>Riiid</t>
         </is>
       </c>
       <c r="B1001" s="4" t="inlineStr">
@@ -47484,12 +47484,12 @@
     <row r="1002">
       <c r="A1002" s="4" t="inlineStr">
         <is>
-          <t>Riiid</t>
+          <t>Manycore Tech (Kujiale)</t>
         </is>
       </c>
       <c r="B1002" s="4" t="inlineStr">
         <is>
-          <t>13 AI Agents</t>
+          <t>17 AI Cloud &amp; Data</t>
         </is>
       </c>
       <c r="C1002" s="4" t="inlineStr">
@@ -47501,7 +47501,7 @@
     <row r="1003">
       <c r="A1003" s="4" t="inlineStr">
         <is>
-          <t>Manycore Tech (Kujiale)</t>
+          <t>Terminus Group</t>
         </is>
       </c>
       <c r="B1003" s="4" t="inlineStr">
@@ -47518,7 +47518,7 @@
     <row r="1004">
       <c r="A1004" s="4" t="inlineStr">
         <is>
-          <t>Terminus Group</t>
+          <t>Clarifai</t>
         </is>
       </c>
       <c r="B1004" s="4" t="inlineStr">
@@ -47535,12 +47535,12 @@
     <row r="1005">
       <c r="A1005" s="4" t="inlineStr">
         <is>
-          <t>Clarifai</t>
+          <t>Paige AI</t>
         </is>
       </c>
       <c r="B1005" s="4" t="inlineStr">
         <is>
-          <t>17 AI Cloud &amp; Data</t>
+          <t>13 AI Agents</t>
         </is>
       </c>
       <c r="C1005" s="4" t="inlineStr">
@@ -47552,29 +47552,29 @@
     <row r="1006">
       <c r="A1006" s="4" t="inlineStr">
         <is>
-          <t>Paige AI</t>
+          <t>Synnex Technology International</t>
         </is>
       </c>
       <c r="B1006" s="4" t="inlineStr">
         <is>
-          <t>13 AI Agents</t>
+          <t>45 Electronic Parts</t>
         </is>
       </c>
       <c r="C1006" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
     </row>
     <row r="1007">
       <c r="A1007" s="4" t="inlineStr">
         <is>
-          <t>Synnex Technology International</t>
+          <t>Taiwan High Speed Rail</t>
         </is>
       </c>
       <c r="B1007" s="4" t="inlineStr">
         <is>
-          <t>45 Electronic Parts</t>
+          <t>X12 Rail, Transit &amp; Road Infra</t>
         </is>
       </c>
       <c r="C1007" s="4" t="inlineStr">
@@ -47586,12 +47586,12 @@
     <row r="1008">
       <c r="A1008" s="4" t="inlineStr">
         <is>
-          <t>Taiwan High Speed Rail</t>
+          <t>Chicony Electronics</t>
         </is>
       </c>
       <c r="B1008" s="4" t="inlineStr">
         <is>
-          <t>X12 Rail, Transit &amp; Road Infra</t>
+          <t>45 Electronic Parts</t>
         </is>
       </c>
       <c r="C1008" s="4" t="inlineStr">
@@ -47603,7 +47603,7 @@
     <row r="1009">
       <c r="A1009" s="4" t="inlineStr">
         <is>
-          <t>Chicony Electronics</t>
+          <t>Gold Circuit Electronics</t>
         </is>
       </c>
       <c r="B1009" s="4" t="inlineStr">
@@ -47620,12 +47620,12 @@
     <row r="1010">
       <c r="A1010" s="4" t="inlineStr">
         <is>
-          <t>Gold Circuit Electronics</t>
+          <t>ASMedia Technology</t>
         </is>
       </c>
       <c r="B1010" s="4" t="inlineStr">
         <is>
-          <t>45 Electronic Parts</t>
+          <t>27 Chip Makers</t>
         </is>
       </c>
       <c r="C1010" s="4" t="inlineStr">
@@ -47637,12 +47637,12 @@
     <row r="1011">
       <c r="A1011" s="4" t="inlineStr">
         <is>
-          <t>ASMedia Technology</t>
+          <t>Hotai Motor</t>
         </is>
       </c>
       <c r="B1011" s="4" t="inlineStr">
         <is>
-          <t>27 Chip Makers</t>
+          <t>43 Mobility &amp; Automotive</t>
         </is>
       </c>
       <c r="C1011" s="4" t="inlineStr">
@@ -47654,12 +47654,12 @@
     <row r="1012">
       <c r="A1012" s="4" t="inlineStr">
         <is>
-          <t>Hotai Motor</t>
+          <t>Ruentex Development</t>
         </is>
       </c>
       <c r="B1012" s="4" t="inlineStr">
         <is>
-          <t>43 Mobility &amp; Automotive</t>
+          <t>X02 Real Estate &amp; Building Produ</t>
         </is>
       </c>
       <c r="C1012" s="4" t="inlineStr">
@@ -47671,12 +47671,12 @@
     <row r="1013">
       <c r="A1013" s="4" t="inlineStr">
         <is>
-          <t>Ruentex Development</t>
+          <t>Far Eastern New Century</t>
         </is>
       </c>
       <c r="B1013" s="4" t="inlineStr">
         <is>
-          <t>X02 Real Estate &amp; Building Produ</t>
+          <t>21 Materials &amp; Mech Parts</t>
         </is>
       </c>
       <c r="C1013" s="4" t="inlineStr">
@@ -47688,12 +47688,12 @@
     <row r="1014">
       <c r="A1014" s="4" t="inlineStr">
         <is>
-          <t>Far Eastern New Century</t>
+          <t>Lotes</t>
         </is>
       </c>
       <c r="B1014" s="4" t="inlineStr">
         <is>
-          <t>21 Materials &amp; Mech Parts</t>
+          <t>45 Electronic Parts</t>
         </is>
       </c>
       <c r="C1014" s="4" t="inlineStr">
@@ -47705,7 +47705,7 @@
     <row r="1015">
       <c r="A1015" s="4" t="inlineStr">
         <is>
-          <t>Lotes</t>
+          <t>BizLink Holding</t>
         </is>
       </c>
       <c r="B1015" s="4" t="inlineStr">
@@ -47722,24 +47722,24 @@
     <row r="1016">
       <c r="A1016" s="4" t="inlineStr">
         <is>
-          <t>BizLink Holding</t>
+          <t>Global Jet Capital</t>
         </is>
       </c>
       <c r="B1016" s="4" t="inlineStr">
         <is>
-          <t>45 Electronic Parts</t>
+          <t>Private Aviation &amp; Business Jets</t>
         </is>
       </c>
       <c r="C1016" s="4" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="1017">
       <c r="A1017" s="4" t="inlineStr">
         <is>
-          <t>Global Jet Capital</t>
+          <t>Modern Aviation</t>
         </is>
       </c>
       <c r="B1017" s="4" t="inlineStr">
@@ -47756,7 +47756,7 @@
     <row r="1018">
       <c r="A1018" s="4" t="inlineStr">
         <is>
-          <t>Modern Aviation</t>
+          <t>Ross Aviation LLC</t>
         </is>
       </c>
       <c r="B1018" s="4" t="inlineStr">
@@ -47773,12 +47773,12 @@
     <row r="1019">
       <c r="A1019" s="4" t="inlineStr">
         <is>
-          <t>Ross Aviation LLC</t>
+          <t>Two Circles Ltd</t>
         </is>
       </c>
       <c r="B1019" s="4" t="inlineStr">
         <is>
-          <t>Private Aviation &amp; Business Jets</t>
+          <t>Sports Tech &amp; Fan Engagement</t>
         </is>
       </c>
       <c r="C1019" s="4" t="inlineStr">
@@ -47790,12 +47790,12 @@
     <row r="1020">
       <c r="A1020" s="4" t="inlineStr">
         <is>
-          <t>Two Circles Ltd</t>
+          <t>ShareChat (Mohalla Tech Pvt Ltd)</t>
         </is>
       </c>
       <c r="B1020" s="4" t="inlineStr">
         <is>
-          <t>Sports Tech &amp; Fan Engagement</t>
+          <t>Creator Economy &amp; Influencer Platforms</t>
         </is>
       </c>
       <c r="C1020" s="4" t="inlineStr">
@@ -47807,12 +47807,12 @@
     <row r="1021">
       <c r="A1021" s="4" t="inlineStr">
         <is>
-          <t>ShareChat (Mohalla Tech Pvt Ltd)</t>
+          <t>MultiChoice Group Limited</t>
         </is>
       </c>
       <c r="B1021" s="4" t="inlineStr">
         <is>
-          <t>Creator Economy &amp; Influencer Platforms</t>
+          <t>Africa Champions</t>
         </is>
       </c>
       <c r="C1021" s="4" t="inlineStr">
@@ -47824,7 +47824,7 @@
     <row r="1022">
       <c r="A1022" s="4" t="inlineStr">
         <is>
-          <t>MultiChoice Group Limited</t>
+          <t>Exxaro Resources Limited</t>
         </is>
       </c>
       <c r="B1022" s="4" t="inlineStr">
@@ -47841,7 +47841,7 @@
     <row r="1023">
       <c r="A1023" s="4" t="inlineStr">
         <is>
-          <t>Exxaro Resources Limited</t>
+          <t>Transnational Corporation of Nigeria Plc (Transcorp)</t>
         </is>
       </c>
       <c r="B1023" s="4" t="inlineStr">
@@ -47858,12 +47858,12 @@
     <row r="1024">
       <c r="A1024" s="4" t="inlineStr">
         <is>
-          <t>Transnational Corporation of Nigeria Plc (Transcorp)</t>
+          <t>Halyk Bank (Halyk Savings Bank of Kazakhstan JSC)</t>
         </is>
       </c>
       <c r="B1024" s="4" t="inlineStr">
         <is>
-          <t>Africa Champions</t>
+          <t>Central Asia &amp; Caucasus Champions</t>
         </is>
       </c>
       <c r="C1024" s="4" t="inlineStr">
@@ -47875,7 +47875,7 @@
     <row r="1025">
       <c r="A1025" s="4" t="inlineStr">
         <is>
-          <t>Halyk Bank (Halyk Savings Bank of Kazakhstan JSC)</t>
+          <t>Kazakhtelecom JSC</t>
         </is>
       </c>
       <c r="B1025" s="4" t="inlineStr">
@@ -47892,29 +47892,29 @@
     <row r="1026">
       <c r="A1026" s="4" t="inlineStr">
         <is>
-          <t>Kazakhtelecom JSC</t>
+          <t>Olive Young (CJ Olive Young)</t>
         </is>
       </c>
       <c r="B1026" s="4" t="inlineStr">
         <is>
-          <t>Central Asia &amp; Caucasus Champions</t>
+          <t>03 Luxury &amp; Beauty</t>
         </is>
       </c>
       <c r="C1026" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
     </row>
     <row r="1027">
       <c r="A1027" s="4" t="inlineStr">
         <is>
-          <t>Olive Young (CJ Olive Young)</t>
+          <t>HD Hyundai Heavy</t>
         </is>
       </c>
       <c r="B1027" s="4" t="inlineStr">
         <is>
-          <t>03 Luxury &amp; Beauty</t>
+          <t>X09 Maritime, Shipping &amp; Ports</t>
         </is>
       </c>
       <c r="C1027" s="4" t="inlineStr">
@@ -47926,12 +47926,12 @@
     <row r="1028">
       <c r="A1028" s="4" t="inlineStr">
         <is>
-          <t>HD Hyundai Heavy</t>
+          <t>Danal</t>
         </is>
       </c>
       <c r="B1028" s="4" t="inlineStr">
         <is>
-          <t>X09 Maritime, Shipping &amp; Ports</t>
+          <t>09 Fintech</t>
         </is>
       </c>
       <c r="C1028" s="4" t="inlineStr">
@@ -47943,12 +47943,12 @@
     <row r="1029">
       <c r="A1029" s="4" t="inlineStr">
         <is>
-          <t>Danal</t>
+          <t>Bucketplace (Today's House)</t>
         </is>
       </c>
       <c r="B1029" s="4" t="inlineStr">
         <is>
-          <t>09 Fintech</t>
+          <t>49 Home &amp; Living</t>
         </is>
       </c>
       <c r="C1029" s="4" t="inlineStr">
@@ -47960,12 +47960,12 @@
     <row r="1030">
       <c r="A1030" s="4" t="inlineStr">
         <is>
-          <t>Bucketplace (Today's House)</t>
+          <t>Zigbang</t>
         </is>
       </c>
       <c r="B1030" s="4" t="inlineStr">
         <is>
-          <t>49 Home &amp; Living</t>
+          <t>X02 Real Estate &amp; Building Produ</t>
         </is>
       </c>
       <c r="C1030" s="4" t="inlineStr">
@@ -47977,12 +47977,12 @@
     <row r="1031">
       <c r="A1031" s="4" t="inlineStr">
         <is>
-          <t>Zigbang</t>
+          <t>Woowa Brothers (Baemin)</t>
         </is>
       </c>
       <c r="B1031" s="4" t="inlineStr">
         <is>
-          <t>X02 Real Estate &amp; Building Produ</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1031" s="4" t="inlineStr">
@@ -47994,12 +47994,12 @@
     <row r="1032">
       <c r="A1032" s="4" t="inlineStr">
         <is>
-          <t>Woowa Brothers (Baemin)</t>
+          <t>Foxconn (Hon Hai)</t>
         </is>
       </c>
       <c r="B1032" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>45 Electronic Parts</t>
         </is>
       </c>
       <c r="C1032" s="4" t="inlineStr">
@@ -48011,12 +48011,12 @@
     <row r="1033">
       <c r="A1033" s="4" t="inlineStr">
         <is>
-          <t>Foxconn (Hon Hai)</t>
+          <t>AVC (Asia Vital Components)</t>
         </is>
       </c>
       <c r="B1033" s="4" t="inlineStr">
         <is>
-          <t>45 Electronic Parts</t>
+          <t>34 DC Power &amp; Cooling</t>
         </is>
       </c>
       <c r="C1033" s="4" t="inlineStr">
@@ -48028,12 +48028,12 @@
     <row r="1034">
       <c r="A1034" s="4" t="inlineStr">
         <is>
-          <t>AVC (Asia Vital Components)</t>
+          <t>Yang Ming Marine</t>
         </is>
       </c>
       <c r="B1034" s="4" t="inlineStr">
         <is>
-          <t>34 DC Power &amp; Cooling</t>
+          <t>X09 Maritime, Shipping &amp; Ports</t>
         </is>
       </c>
       <c r="C1034" s="4" t="inlineStr">
@@ -48045,12 +48045,12 @@
     <row r="1035">
       <c r="A1035" s="4" t="inlineStr">
         <is>
-          <t>Yang Ming Marine</t>
+          <t>OVO</t>
         </is>
       </c>
       <c r="B1035" s="4" t="inlineStr">
         <is>
-          <t>X09 Maritime, Shipping &amp; Ports</t>
+          <t>09 Fintech</t>
         </is>
       </c>
       <c r="C1035" s="4" t="inlineStr">
@@ -48062,29 +48062,29 @@
     <row r="1036">
       <c r="A1036" s="4" t="inlineStr">
         <is>
-          <t>OVO</t>
+          <t>Ominimo</t>
         </is>
       </c>
       <c r="B1036" s="4" t="inlineStr">
         <is>
-          <t>09 Fintech</t>
+          <t>01 Banking &amp; Insurance</t>
         </is>
       </c>
       <c r="C1036" s="4" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="1037">
       <c r="A1037" s="4" t="inlineStr">
         <is>
-          <t>Ominimo</t>
+          <t>Erebor Bank</t>
         </is>
       </c>
       <c r="B1037" s="4" t="inlineStr">
         <is>
-          <t>01 Banking &amp; Insurance</t>
+          <t>12 Trading &amp; Crypto</t>
         </is>
       </c>
       <c r="C1037" s="4" t="inlineStr">
@@ -48096,7 +48096,7 @@
     <row r="1038">
       <c r="A1038" s="4" t="inlineStr">
         <is>
-          <t>Erebor Bank</t>
+          <t>Whop</t>
         </is>
       </c>
       <c r="B1038" s="4" t="inlineStr">
@@ -48113,7 +48113,7 @@
     <row r="1039">
       <c r="A1039" s="4" t="inlineStr">
         <is>
-          <t>Whop</t>
+          <t>Ripple</t>
         </is>
       </c>
       <c r="B1039" s="4" t="inlineStr">
@@ -48130,7 +48130,7 @@
     <row r="1040">
       <c r="A1040" s="4" t="inlineStr">
         <is>
-          <t>Ripple</t>
+          <t>Mesh</t>
         </is>
       </c>
       <c r="B1040" s="4" t="inlineStr">
@@ -48147,12 +48147,12 @@
     <row r="1041">
       <c r="A1041" s="4" t="inlineStr">
         <is>
-          <t>Mesh</t>
+          <t>Moneybox</t>
         </is>
       </c>
       <c r="B1041" s="4" t="inlineStr">
         <is>
-          <t>12 Trading &amp; Crypto</t>
+          <t>X25 Wealth Mgmt &amp; Private Banking</t>
         </is>
       </c>
       <c r="C1041" s="4" t="inlineStr">
@@ -48164,12 +48164,12 @@
     <row r="1042">
       <c r="A1042" s="4" t="inlineStr">
         <is>
-          <t>Moneybox</t>
+          <t>Slash</t>
         </is>
       </c>
       <c r="B1042" s="4" t="inlineStr">
         <is>
-          <t>X25 Wealth Mgmt &amp; Private Banking</t>
+          <t>09 Fintech</t>
         </is>
       </c>
       <c r="C1042" s="4" t="inlineStr">
@@ -48181,7 +48181,7 @@
     <row r="1043">
       <c r="A1043" s="4" t="inlineStr">
         <is>
-          <t>Slash</t>
+          <t>Super.com</t>
         </is>
       </c>
       <c r="B1043" s="4" t="inlineStr">
@@ -48198,12 +48198,12 @@
     <row r="1044">
       <c r="A1044" s="4" t="inlineStr">
         <is>
-          <t>Super.com</t>
+          <t>Circle Internet Group</t>
         </is>
       </c>
       <c r="B1044" s="4" t="inlineStr">
         <is>
-          <t>09 Fintech</t>
+          <t>12 Trading &amp; Crypto</t>
         </is>
       </c>
       <c r="C1044" s="4" t="inlineStr">
@@ -48215,12 +48215,12 @@
     <row r="1045">
       <c r="A1045" s="4" t="inlineStr">
         <is>
-          <t>Circle Internet Group</t>
+          <t>Bank Jago</t>
         </is>
       </c>
       <c r="B1045" s="4" t="inlineStr">
         <is>
-          <t>12 Trading &amp; Crypto</t>
+          <t>09 Fintech</t>
         </is>
       </c>
       <c r="C1045" s="4" t="inlineStr">
@@ -48232,12 +48232,12 @@
     <row r="1046">
       <c r="A1046" s="4" t="inlineStr">
         <is>
-          <t>Bank Jago</t>
+          <t>Enovix Corporation</t>
         </is>
       </c>
       <c r="B1046" s="4" t="inlineStr">
         <is>
-          <t>09 Fintech</t>
+          <t>43 Mobility &amp; Automotive</t>
         </is>
       </c>
       <c r="C1046" s="4" t="inlineStr">
@@ -48249,12 +48249,12 @@
     <row r="1047">
       <c r="A1047" s="4" t="inlineStr">
         <is>
-          <t>Enovix Corporation</t>
+          <t>Xpressbees</t>
         </is>
       </c>
       <c r="B1047" s="4" t="inlineStr">
         <is>
-          <t>43 Mobility &amp; Automotive</t>
+          <t>24 Logistics</t>
         </is>
       </c>
       <c r="C1047" s="4" t="inlineStr">
@@ -48266,12 +48266,12 @@
     <row r="1048">
       <c r="A1048" s="4" t="inlineStr">
         <is>
-          <t>Xpressbees</t>
+          <t>Ola Consumer (ANI Technologies)</t>
         </is>
       </c>
       <c r="B1048" s="4" t="inlineStr">
         <is>
-          <t>24 Logistics</t>
+          <t>43 Mobility &amp; Automotive</t>
         </is>
       </c>
       <c r="C1048" s="4" t="inlineStr">
@@ -48283,7 +48283,7 @@
     <row r="1049">
       <c r="A1049" s="4" t="inlineStr">
         <is>
-          <t>Ola Consumer (ANI Technologies)</t>
+          <t>Apeel Sciences</t>
         </is>
       </c>
       <c r="B1049" s="4" t="inlineStr">
@@ -48300,7 +48300,7 @@
     <row r="1050">
       <c r="A1050" s="4" t="inlineStr">
         <is>
-          <t>Apeel Sciences</t>
+          <t>Eat Just / GOOD Meat</t>
         </is>
       </c>
       <c r="B1050" s="4" t="inlineStr">
@@ -48317,12 +48317,12 @@
     <row r="1051">
       <c r="A1051" s="4" t="inlineStr">
         <is>
-          <t>Eat Just / GOOD Meat</t>
+          <t>Forto</t>
         </is>
       </c>
       <c r="B1051" s="4" t="inlineStr">
         <is>
-          <t>43 Mobility &amp; Automotive</t>
+          <t>24 Logistics</t>
         </is>
       </c>
       <c r="C1051" s="4" t="inlineStr">
@@ -48334,7 +48334,7 @@
     <row r="1052">
       <c r="A1052" s="4" t="inlineStr">
         <is>
-          <t>Forto</t>
+          <t>Loggi</t>
         </is>
       </c>
       <c r="B1052" s="4" t="inlineStr">
@@ -48351,12 +48351,12 @@
     <row r="1053">
       <c r="A1053" s="4" t="inlineStr">
         <is>
-          <t>Loggi</t>
+          <t>Rimac Group</t>
         </is>
       </c>
       <c r="B1053" s="4" t="inlineStr">
         <is>
-          <t>24 Logistics</t>
+          <t>43 Mobility &amp; Automotive</t>
         </is>
       </c>
       <c r="C1053" s="4" t="inlineStr">
@@ -48368,7 +48368,7 @@
     <row r="1054">
       <c r="A1054" s="4" t="inlineStr">
         <is>
-          <t>Rimac Group</t>
+          <t>Captain Fresh</t>
         </is>
       </c>
       <c r="B1054" s="4" t="inlineStr">
@@ -48385,12 +48385,12 @@
     <row r="1055">
       <c r="A1055" s="4" t="inlineStr">
         <is>
-          <t>Captain Fresh</t>
+          <t>Flash Express (Flash Group)</t>
         </is>
       </c>
       <c r="B1055" s="4" t="inlineStr">
         <is>
-          <t>43 Mobility &amp; Automotive</t>
+          <t>24 Logistics</t>
         </is>
       </c>
       <c r="C1055" s="4" t="inlineStr">
@@ -48402,29 +48402,29 @@
     <row r="1056">
       <c r="A1056" s="4" t="inlineStr">
         <is>
-          <t>Flash Express (Flash Group)</t>
+          <t>Petrolimex</t>
         </is>
       </c>
       <c r="B1056" s="4" t="inlineStr">
         <is>
-          <t>24 Logistics</t>
+          <t>02 Energy &amp; Industrial</t>
         </is>
       </c>
       <c r="C1056" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
     </row>
     <row r="1057">
       <c r="A1057" s="4" t="inlineStr">
         <is>
-          <t>Petrolimex</t>
+          <t>Bank of the Philippine Islands</t>
         </is>
       </c>
       <c r="B1057" s="4" t="inlineStr">
         <is>
-          <t>02 Energy &amp; Industrial</t>
+          <t>01 Banking &amp; Insurance</t>
         </is>
       </c>
       <c r="C1057" s="4" t="inlineStr">
@@ -48436,12 +48436,12 @@
     <row r="1058">
       <c r="A1058" s="4" t="inlineStr">
         <is>
-          <t>Bank of the Philippine Islands</t>
+          <t>Manila Electric Company (Meralco)</t>
         </is>
       </c>
       <c r="B1058" s="4" t="inlineStr">
         <is>
-          <t>01 Banking &amp; Insurance</t>
+          <t>02 Energy &amp; Industrial</t>
         </is>
       </c>
       <c r="C1058" s="4" t="inlineStr">
@@ -48453,12 +48453,12 @@
     <row r="1059">
       <c r="A1059" s="4" t="inlineStr">
         <is>
-          <t>Manila Electric Company (Meralco)</t>
+          <t>Century Pacific Food</t>
         </is>
       </c>
       <c r="B1059" s="4" t="inlineStr">
         <is>
-          <t>02 Energy &amp; Industrial</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C1059" s="4" t="inlineStr">
@@ -48470,12 +48470,12 @@
     <row r="1060">
       <c r="A1060" s="4" t="inlineStr">
         <is>
-          <t>Century Pacific Food</t>
+          <t>Premier Investments</t>
         </is>
       </c>
       <c r="B1060" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1060" s="4" t="inlineStr">
@@ -48487,12 +48487,12 @@
     <row r="1061">
       <c r="A1061" s="4" t="inlineStr">
         <is>
-          <t>Premier Investments</t>
+          <t>The a2 Milk Company</t>
         </is>
       </c>
       <c r="B1061" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C1061" s="4" t="inlineStr">
@@ -48504,7 +48504,7 @@
     <row r="1062">
       <c r="A1062" s="4" t="inlineStr">
         <is>
-          <t>The a2 Milk Company</t>
+          <t>Bega Cheese</t>
         </is>
       </c>
       <c r="B1062" s="4" t="inlineStr">
@@ -48521,12 +48521,12 @@
     <row r="1063">
       <c r="A1063" s="4" t="inlineStr">
         <is>
-          <t>Bega Cheese</t>
+          <t>Australian Retirement Trust</t>
         </is>
       </c>
       <c r="B1063" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>X25 Wealth Mgmt &amp; Private Banking</t>
         </is>
       </c>
       <c r="C1063" s="4" t="inlineStr">
@@ -48538,12 +48538,12 @@
     <row r="1064">
       <c r="A1064" s="4" t="inlineStr">
         <is>
-          <t>Australian Retirement Trust</t>
+          <t>Future Fund Australia</t>
         </is>
       </c>
       <c r="B1064" s="4" t="inlineStr">
         <is>
-          <t>X25 Wealth Mgmt &amp; Private Banking</t>
+          <t>X01 Asset Mgmt, PE &amp; Trading Fir</t>
         </is>
       </c>
       <c r="C1064" s="4" t="inlineStr">
@@ -48555,12 +48555,12 @@
     <row r="1065">
       <c r="A1065" s="4" t="inlineStr">
         <is>
-          <t>Future Fund Australia</t>
+          <t>Saudi Awwal Bank (SAB)</t>
         </is>
       </c>
       <c r="B1065" s="4" t="inlineStr">
         <is>
-          <t>X01 Asset Mgmt, PE &amp; Trading Fir</t>
+          <t>01 Banking &amp; Insurance</t>
         </is>
       </c>
       <c r="C1065" s="4" t="inlineStr">
@@ -48572,12 +48572,12 @@
     <row r="1066">
       <c r="A1066" s="4" t="inlineStr">
         <is>
-          <t>Saudi Awwal Bank (SAB)</t>
+          <t>Theo Mueller (Mueller Group)</t>
         </is>
       </c>
       <c r="B1066" s="4" t="inlineStr">
         <is>
-          <t>01 Banking &amp; Insurance</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C1066" s="4" t="inlineStr">
@@ -48589,7 +48589,7 @@
     <row r="1067">
       <c r="A1067" s="4" t="inlineStr">
         <is>
-          <t>Theo Mueller (Mueller Group)</t>
+          <t>Toennies Group</t>
         </is>
       </c>
       <c r="B1067" s="4" t="inlineStr">
@@ -48606,7 +48606,7 @@
     <row r="1068">
       <c r="A1068" s="4" t="inlineStr">
         <is>
-          <t>Toennies Group</t>
+          <t>Hochland</t>
         </is>
       </c>
       <c r="B1068" s="4" t="inlineStr">
@@ -48623,12 +48623,12 @@
     <row r="1069">
       <c r="A1069" s="4" t="inlineStr">
         <is>
-          <t>Hochland</t>
+          <t>Peek &amp; Cloppenburg (Duesseldorf)</t>
         </is>
       </c>
       <c r="B1069" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1069" s="4" t="inlineStr">
@@ -48640,7 +48640,7 @@
     <row r="1070">
       <c r="A1070" s="4" t="inlineStr">
         <is>
-          <t>Peek &amp; Cloppenburg (Duesseldorf)</t>
+          <t>Action</t>
         </is>
       </c>
       <c r="B1070" s="4" t="inlineStr">
@@ -48657,7 +48657,7 @@
     <row r="1071">
       <c r="A1071" s="4" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Coolblue</t>
         </is>
       </c>
       <c r="B1071" s="4" t="inlineStr">
@@ -48674,12 +48674,12 @@
     <row r="1072">
       <c r="A1072" s="4" t="inlineStr">
         <is>
-          <t>Coolblue</t>
+          <t>FrieslandCampina</t>
         </is>
       </c>
       <c r="B1072" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C1072" s="4" t="inlineStr">
@@ -48691,12 +48691,12 @@
     <row r="1073">
       <c r="A1073" s="4" t="inlineStr">
         <is>
-          <t>FrieslandCampina</t>
+          <t>Jumbo Supermarkten</t>
         </is>
       </c>
       <c r="B1073" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1073" s="4" t="inlineStr">
@@ -48708,12 +48708,12 @@
     <row r="1074">
       <c r="A1074" s="4" t="inlineStr">
         <is>
-          <t>Jumbo Supermarkten</t>
+          <t>Notino</t>
         </is>
       </c>
       <c r="B1074" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>03 Luxury &amp; Beauty</t>
         </is>
       </c>
       <c r="C1074" s="4" t="inlineStr">
@@ -48725,12 +48725,12 @@
     <row r="1075">
       <c r="A1075" s="4" t="inlineStr">
         <is>
-          <t>Notino</t>
+          <t>Dedeman</t>
         </is>
       </c>
       <c r="B1075" s="4" t="inlineStr">
         <is>
-          <t>03 Luxury &amp; Beauty</t>
+          <t>49 Home &amp; Living</t>
         </is>
       </c>
       <c r="C1075" s="4" t="inlineStr">
@@ -48742,12 +48742,12 @@
     <row r="1076">
       <c r="A1076" s="4" t="inlineStr">
         <is>
-          <t>Dedeman</t>
+          <t>Albertsons Companies</t>
         </is>
       </c>
       <c r="B1076" s="4" t="inlineStr">
         <is>
-          <t>49 Home &amp; Living</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1076" s="4" t="inlineStr">
@@ -48759,12 +48759,12 @@
     <row r="1077">
       <c r="A1077" s="4" t="inlineStr">
         <is>
-          <t>Albertsons Companies</t>
+          <t>Sysco</t>
         </is>
       </c>
       <c r="B1077" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>X13 Industrial &amp; MRO Distributio</t>
         </is>
       </c>
       <c r="C1077" s="4" t="inlineStr">
@@ -48776,7 +48776,7 @@
     <row r="1078">
       <c r="A1078" s="4" t="inlineStr">
         <is>
-          <t>Sysco</t>
+          <t>US Foods</t>
         </is>
       </c>
       <c r="B1078" s="4" t="inlineStr">
@@ -48793,7 +48793,7 @@
     <row r="1079">
       <c r="A1079" s="4" t="inlineStr">
         <is>
-          <t>US Foods</t>
+          <t>Performance Food Group</t>
         </is>
       </c>
       <c r="B1079" s="4" t="inlineStr">
@@ -48810,7 +48810,7 @@
     <row r="1080">
       <c r="A1080" s="4" t="inlineStr">
         <is>
-          <t>Performance Food Group</t>
+          <t>Chefs' Warehouse</t>
         </is>
       </c>
       <c r="B1080" s="4" t="inlineStr">
@@ -48827,12 +48827,12 @@
     <row r="1081">
       <c r="A1081" s="4" t="inlineStr">
         <is>
-          <t>Chefs' Warehouse</t>
+          <t>BJ's Wholesale Club</t>
         </is>
       </c>
       <c r="B1081" s="4" t="inlineStr">
         <is>
-          <t>X13 Industrial &amp; MRO Distributio</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1081" s="4" t="inlineStr">
@@ -48844,7 +48844,7 @@
     <row r="1082">
       <c r="A1082" s="4" t="inlineStr">
         <is>
-          <t>BJ's Wholesale Club</t>
+          <t>Dollar General</t>
         </is>
       </c>
       <c r="B1082" s="4" t="inlineStr">
@@ -48861,7 +48861,7 @@
     <row r="1083">
       <c r="A1083" s="4" t="inlineStr">
         <is>
-          <t>Dollar General</t>
+          <t>Dollar Tree</t>
         </is>
       </c>
       <c r="B1083" s="4" t="inlineStr">
@@ -48878,7 +48878,7 @@
     <row r="1084">
       <c r="A1084" s="4" t="inlineStr">
         <is>
-          <t>Dollar Tree</t>
+          <t>Ross Stores</t>
         </is>
       </c>
       <c r="B1084" s="4" t="inlineStr">
@@ -48895,7 +48895,7 @@
     <row r="1085">
       <c r="A1085" s="4" t="inlineStr">
         <is>
-          <t>Ross Stores</t>
+          <t>TJX Companies</t>
         </is>
       </c>
       <c r="B1085" s="4" t="inlineStr">
@@ -48912,12 +48912,12 @@
     <row r="1086">
       <c r="A1086" s="4" t="inlineStr">
         <is>
-          <t>TJX Companies</t>
+          <t>Sanofi</t>
         </is>
       </c>
       <c r="B1086" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>42 Health &amp; Wellness</t>
         </is>
       </c>
       <c r="C1086" s="4" t="inlineStr">
@@ -48929,7 +48929,7 @@
     <row r="1087">
       <c r="A1087" s="4" t="inlineStr">
         <is>
-          <t>Sanofi</t>
+          <t>Roche</t>
         </is>
       </c>
       <c r="B1087" s="4" t="inlineStr">
@@ -48946,7 +48946,7 @@
     <row r="1088">
       <c r="A1088" s="4" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="B1088" s="4" t="inlineStr">
@@ -48963,7 +48963,7 @@
     <row r="1089">
       <c r="A1089" s="4" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>UCB</t>
         </is>
       </c>
       <c r="B1089" s="4" t="inlineStr">
@@ -48980,7 +48980,7 @@
     <row r="1090">
       <c r="A1090" s="4" t="inlineStr">
         <is>
-          <t>UCB</t>
+          <t>Genmab</t>
         </is>
       </c>
       <c r="B1090" s="4" t="inlineStr">
@@ -48997,7 +48997,7 @@
     <row r="1091">
       <c r="A1091" s="4" t="inlineStr">
         <is>
-          <t>Genmab</t>
+          <t>Zealand Pharma</t>
         </is>
       </c>
       <c r="B1091" s="4" t="inlineStr">
@@ -49014,7 +49014,7 @@
     <row r="1092">
       <c r="A1092" s="4" t="inlineStr">
         <is>
-          <t>Zealand Pharma</t>
+          <t>Alcon</t>
         </is>
       </c>
       <c r="B1092" s="4" t="inlineStr">
@@ -49031,7 +49031,7 @@
     <row r="1093">
       <c r="A1093" s="4" t="inlineStr">
         <is>
-          <t>Alcon</t>
+          <t>Smith and Nephew</t>
         </is>
       </c>
       <c r="B1093" s="4" t="inlineStr">
@@ -49048,7 +49048,7 @@
     <row r="1094">
       <c r="A1094" s="4" t="inlineStr">
         <is>
-          <t>Smith and Nephew</t>
+          <t>Coloplast</t>
         </is>
       </c>
       <c r="B1094" s="4" t="inlineStr">
@@ -49065,7 +49065,7 @@
     <row r="1095">
       <c r="A1095" s="4" t="inlineStr">
         <is>
-          <t>Coloplast</t>
+          <t>Demant</t>
         </is>
       </c>
       <c r="B1095" s="4" t="inlineStr">
@@ -49082,12 +49082,12 @@
     <row r="1096">
       <c r="A1096" s="4" t="inlineStr">
         <is>
-          <t>Demant</t>
+          <t>Wealth Enhancement Group</t>
         </is>
       </c>
       <c r="B1096" s="4" t="inlineStr">
         <is>
-          <t>42 Health &amp; Wellness</t>
+          <t>X25 Wealth Mgmt &amp; Private Banking</t>
         </is>
       </c>
       <c r="C1096" s="4" t="inlineStr">
@@ -49099,7 +49099,7 @@
     <row r="1097">
       <c r="A1097" s="4" t="inlineStr">
         <is>
-          <t>Wealth Enhancement Group</t>
+          <t>Mariner Wealth Advisors</t>
         </is>
       </c>
       <c r="B1097" s="4" t="inlineStr">
@@ -49116,12 +49116,12 @@
     <row r="1098">
       <c r="A1098" s="4" t="inlineStr">
         <is>
-          <t>Mariner Wealth Advisors</t>
+          <t>Vizient</t>
         </is>
       </c>
       <c r="B1098" s="4" t="inlineStr">
         <is>
-          <t>X25 Wealth Mgmt &amp; Private Banking</t>
+          <t>42 Health &amp; Wellness</t>
         </is>
       </c>
       <c r="C1098" s="4" t="inlineStr">
@@ -49133,7 +49133,7 @@
     <row r="1099">
       <c r="A1099" s="4" t="inlineStr">
         <is>
-          <t>Vizient</t>
+          <t>Opella</t>
         </is>
       </c>
       <c r="B1099" s="4" t="inlineStr">
@@ -49150,7 +49150,7 @@
     <row r="1100">
       <c r="A1100" s="4" t="inlineStr">
         <is>
-          <t>Opella</t>
+          <t>Zentiva</t>
         </is>
       </c>
       <c r="B1100" s="4" t="inlineStr">
@@ -49167,7 +49167,7 @@
     <row r="1101">
       <c r="A1101" s="4" t="inlineStr">
         <is>
-          <t>Zentiva</t>
+          <t>Neuraxpharm</t>
         </is>
       </c>
       <c r="B1101" s="4" t="inlineStr">
@@ -49184,7 +49184,7 @@
     <row r="1102">
       <c r="A1102" s="4" t="inlineStr">
         <is>
-          <t>Neuraxpharm</t>
+          <t>Advanz Pharma</t>
         </is>
       </c>
       <c r="B1102" s="4" t="inlineStr">
@@ -49201,12 +49201,12 @@
     <row r="1103">
       <c r="A1103" s="4" t="inlineStr">
         <is>
-          <t>Advanz Pharma</t>
+          <t>Topgolf</t>
         </is>
       </c>
       <c r="B1103" s="4" t="inlineStr">
         <is>
-          <t>42 Health &amp; Wellness</t>
+          <t>X08 Sporting Goods &amp; Fitness</t>
         </is>
       </c>
       <c r="C1103" s="4" t="inlineStr">
@@ -49218,12 +49218,12 @@
     <row r="1104">
       <c r="A1104" s="4" t="inlineStr">
         <is>
-          <t>Topgolf</t>
+          <t>Staples</t>
         </is>
       </c>
       <c r="B1104" s="4" t="inlineStr">
         <is>
-          <t>X08 Sporting Goods &amp; Fitness</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1104" s="4" t="inlineStr">
@@ -49235,12 +49235,12 @@
     <row r="1105">
       <c r="A1105" s="4" t="inlineStr">
         <is>
-          <t>Staples</t>
+          <t>Revelyst</t>
         </is>
       </c>
       <c r="B1105" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>X08 Sporting Goods &amp; Fitness</t>
         </is>
       </c>
       <c r="C1105" s="4" t="inlineStr">
@@ -49252,12 +49252,12 @@
     <row r="1106">
       <c r="A1106" s="4" t="inlineStr">
         <is>
-          <t>Revelyst</t>
+          <t>Koc Holding</t>
         </is>
       </c>
       <c r="B1106" s="4" t="inlineStr">
         <is>
-          <t>X08 Sporting Goods &amp; Fitness</t>
+          <t>X01 Asset Mgmt, PE &amp; Trading Fir</t>
         </is>
       </c>
       <c r="C1106" s="4" t="inlineStr">
@@ -49269,7 +49269,7 @@
     <row r="1107">
       <c r="A1107" s="4" t="inlineStr">
         <is>
-          <t>Koc Holding</t>
+          <t>Sabanci Holding</t>
         </is>
       </c>
       <c r="B1107" s="4" t="inlineStr">
@@ -49286,12 +49286,12 @@
     <row r="1108">
       <c r="A1108" s="4" t="inlineStr">
         <is>
-          <t>Sabanci Holding</t>
+          <t>Pegasus Airlines</t>
         </is>
       </c>
       <c r="B1108" s="4" t="inlineStr">
         <is>
-          <t>X01 Asset Mgmt, PE &amp; Trading Fir</t>
+          <t>16 Travel &amp; Hospitality</t>
         </is>
       </c>
       <c r="C1108" s="4" t="inlineStr">
@@ -49303,12 +49303,12 @@
     <row r="1109">
       <c r="A1109" s="4" t="inlineStr">
         <is>
-          <t>Pegasus Airlines</t>
+          <t>Garanti BBVA</t>
         </is>
       </c>
       <c r="B1109" s="4" t="inlineStr">
         <is>
-          <t>16 Travel &amp; Hospitality</t>
+          <t>01 Banking &amp; Insurance</t>
         </is>
       </c>
       <c r="C1109" s="4" t="inlineStr">
@@ -49320,7 +49320,7 @@
     <row r="1110">
       <c r="A1110" s="4" t="inlineStr">
         <is>
-          <t>Garanti BBVA</t>
+          <t>Akbank</t>
         </is>
       </c>
       <c r="B1110" s="4" t="inlineStr">
@@ -49337,7 +49337,7 @@
     <row r="1111">
       <c r="A1111" s="4" t="inlineStr">
         <is>
-          <t>Akbank</t>
+          <t>Is Bankasi</t>
         </is>
       </c>
       <c r="B1111" s="4" t="inlineStr">
@@ -49354,7 +49354,7 @@
     <row r="1112">
       <c r="A1112" s="4" t="inlineStr">
         <is>
-          <t>Is Bankasi</t>
+          <t>Yapi Kredi</t>
         </is>
       </c>
       <c r="B1112" s="4" t="inlineStr">
@@ -49371,7 +49371,7 @@
     <row r="1113">
       <c r="A1113" s="4" t="inlineStr">
         <is>
-          <t>Yapi Kredi</t>
+          <t>Ziraat Bank</t>
         </is>
       </c>
       <c r="B1113" s="4" t="inlineStr">
@@ -49388,12 +49388,12 @@
     <row r="1114">
       <c r="A1114" s="4" t="inlineStr">
         <is>
-          <t>Ziraat Bank</t>
+          <t>BIM Birlesik Magazalar</t>
         </is>
       </c>
       <c r="B1114" s="4" t="inlineStr">
         <is>
-          <t>01 Banking &amp; Insurance</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1114" s="4" t="inlineStr">
@@ -49405,12 +49405,12 @@
     <row r="1115">
       <c r="A1115" s="4" t="inlineStr">
         <is>
-          <t>BIM Birlesik Magazalar</t>
+          <t>Arcelik</t>
         </is>
       </c>
       <c r="B1115" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>49 Home &amp; Living</t>
         </is>
       </c>
       <c r="C1115" s="4" t="inlineStr">
@@ -49422,12 +49422,12 @@
     <row r="1116">
       <c r="A1116" s="4" t="inlineStr">
         <is>
-          <t>Arcelik</t>
+          <t>Corporacion Favorita</t>
         </is>
       </c>
       <c r="B1116" s="4" t="inlineStr">
         <is>
-          <t>49 Home &amp; Living</t>
+          <t>X41 LatAm Consumer &amp; Retail Champions</t>
         </is>
       </c>
       <c r="C1116" s="4" t="inlineStr">
@@ -49439,12 +49439,12 @@
     <row r="1117">
       <c r="A1117" s="4" t="inlineStr">
         <is>
-          <t>Corporacion Favorita</t>
+          <t>Grupo Vidanta</t>
         </is>
       </c>
       <c r="B1117" s="4" t="inlineStr">
         <is>
-          <t>X41 LatAm Consumer &amp; Retail Champions</t>
+          <t>16 Travel &amp; Hospitality</t>
         </is>
       </c>
       <c r="C1117" s="4" t="inlineStr">
@@ -49456,7 +49456,7 @@
     <row r="1118">
       <c r="A1118" s="4" t="inlineStr">
         <is>
-          <t>Grupo Vidanta</t>
+          <t>Grupo Xcaret</t>
         </is>
       </c>
       <c r="B1118" s="4" t="inlineStr">
@@ -49473,12 +49473,12 @@
     <row r="1119">
       <c r="A1119" s="4" t="inlineStr">
         <is>
-          <t>Grupo Xcaret</t>
+          <t>Rossmann</t>
         </is>
       </c>
       <c r="B1119" s="4" t="inlineStr">
         <is>
-          <t>16 Travel &amp; Hospitality</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1119" s="4" t="inlineStr">
@@ -49490,7 +49490,7 @@
     <row r="1120">
       <c r="A1120" s="4" t="inlineStr">
         <is>
-          <t>Rossmann</t>
+          <t>Mueller Drogerie</t>
         </is>
       </c>
       <c r="B1120" s="4" t="inlineStr">
@@ -49507,12 +49507,12 @@
     <row r="1121">
       <c r="A1121" s="4" t="inlineStr">
         <is>
-          <t>Mueller Drogerie</t>
+          <t>Tengelmann Group (OBI, KiK)</t>
         </is>
       </c>
       <c r="B1121" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>49 Home &amp; Living</t>
         </is>
       </c>
       <c r="C1121" s="4" t="inlineStr">
@@ -49524,12 +49524,12 @@
     <row r="1122">
       <c r="A1122" s="4" t="inlineStr">
         <is>
-          <t>Tengelmann Group (OBI, KiK)</t>
+          <t>Globus Holding</t>
         </is>
       </c>
       <c r="B1122" s="4" t="inlineStr">
         <is>
-          <t>49 Home &amp; Living</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1122" s="4" t="inlineStr">
@@ -49541,7 +49541,7 @@
     <row r="1123">
       <c r="A1123" s="4" t="inlineStr">
         <is>
-          <t>Globus Holding</t>
+          <t>Rewe Group</t>
         </is>
       </c>
       <c r="B1123" s="4" t="inlineStr">
@@ -49558,12 +49558,12 @@
     <row r="1124">
       <c r="A1124" s="4" t="inlineStr">
         <is>
-          <t>Rewe Group</t>
+          <t>Bauhaus</t>
         </is>
       </c>
       <c r="B1124" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>49 Home &amp; Living</t>
         </is>
       </c>
       <c r="C1124" s="4" t="inlineStr">
@@ -49575,12 +49575,12 @@
     <row r="1125">
       <c r="A1125" s="4" t="inlineStr">
         <is>
-          <t>Bauhaus</t>
+          <t>Deichmann</t>
         </is>
       </c>
       <c r="B1125" s="4" t="inlineStr">
         <is>
-          <t>49 Home &amp; Living</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1125" s="4" t="inlineStr">
@@ -49592,12 +49592,12 @@
     <row r="1126">
       <c r="A1126" s="4" t="inlineStr">
         <is>
-          <t>Deichmann</t>
+          <t>Zelos Technology (ZTO ZELOS)</t>
         </is>
       </c>
       <c r="B1126" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>43 Mobility &amp; Automotive</t>
         </is>
       </c>
       <c r="C1126" s="4" t="inlineStr">
@@ -49609,12 +49609,12 @@
     <row r="1127">
       <c r="A1127" s="4" t="inlineStr">
         <is>
-          <t>Zelos Technology (ZTO ZELOS)</t>
+          <t>Sunwoda EVB</t>
         </is>
       </c>
       <c r="B1127" s="4" t="inlineStr">
         <is>
-          <t>43 Mobility &amp; Automotive</t>
+          <t>X10 Batteries, EV, Waste &amp; Water</t>
         </is>
       </c>
       <c r="C1127" s="4" t="inlineStr">
@@ -49626,7 +49626,7 @@
     <row r="1128">
       <c r="A1128" s="4" t="inlineStr">
         <is>
-          <t>Sunwoda EVB</t>
+          <t>Farasis Energy</t>
         </is>
       </c>
       <c r="B1128" s="4" t="inlineStr">
@@ -49643,7 +49643,7 @@
     <row r="1129">
       <c r="A1129" s="4" t="inlineStr">
         <is>
-          <t>Farasis Energy</t>
+          <t>Hithium</t>
         </is>
       </c>
       <c r="B1129" s="4" t="inlineStr">
@@ -49660,7 +49660,7 @@
     <row r="1130">
       <c r="A1130" s="4" t="inlineStr">
         <is>
-          <t>Hithium</t>
+          <t>REPT Battero</t>
         </is>
       </c>
       <c r="B1130" s="4" t="inlineStr">
@@ -49677,7 +49677,7 @@
     <row r="1131">
       <c r="A1131" s="4" t="inlineStr">
         <is>
-          <t>REPT Battero</t>
+          <t>Tianneng Power</t>
         </is>
       </c>
       <c r="B1131" s="4" t="inlineStr">
@@ -49694,12 +49694,12 @@
     <row r="1132">
       <c r="A1132" s="4" t="inlineStr">
         <is>
-          <t>Tianneng Power</t>
+          <t>Trina Solar</t>
         </is>
       </c>
       <c r="B1132" s="4" t="inlineStr">
         <is>
-          <t>X10 Batteries, EV, Waste &amp; Water</t>
+          <t>02 Energy &amp; Industrial</t>
         </is>
       </c>
       <c r="C1132" s="4" t="inlineStr">
@@ -49711,7 +49711,7 @@
     <row r="1133">
       <c r="A1133" s="4" t="inlineStr">
         <is>
-          <t>Trina Solar</t>
+          <t>Jinko Solar</t>
         </is>
       </c>
       <c r="B1133" s="4" t="inlineStr">
@@ -49728,7 +49728,7 @@
     <row r="1134">
       <c r="A1134" s="4" t="inlineStr">
         <is>
-          <t>Jinko Solar</t>
+          <t>Goldwind</t>
         </is>
       </c>
       <c r="B1134" s="4" t="inlineStr">
@@ -49745,12 +49745,12 @@
     <row r="1135">
       <c r="A1135" s="4" t="inlineStr">
         <is>
-          <t>Goldwind</t>
+          <t>Auntea Jenny (Chayan Yuese)</t>
         </is>
       </c>
       <c r="B1135" s="4" t="inlineStr">
         <is>
-          <t>02 Energy &amp; Industrial</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C1135" s="4" t="inlineStr">
@@ -49762,24 +49762,24 @@
     <row r="1136">
       <c r="A1136" s="4" t="inlineStr">
         <is>
-          <t>Auntea Jenny (Chayan Yuese)</t>
+          <t>Valo Health</t>
         </is>
       </c>
       <c r="B1136" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>42 Health &amp; Wellness</t>
         </is>
       </c>
       <c r="C1136" s="4" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="1137">
       <c r="A1137" s="4" t="inlineStr">
         <is>
-          <t>Valo Health</t>
+          <t>WeDoctor</t>
         </is>
       </c>
       <c r="B1137" s="4" t="inlineStr">
@@ -49796,12 +49796,12 @@
     <row r="1138">
       <c r="A1138" s="4" t="inlineStr">
         <is>
-          <t>WeDoctor</t>
+          <t>Kraken Technologies</t>
         </is>
       </c>
       <c r="B1138" s="4" t="inlineStr">
         <is>
-          <t>42 Health &amp; Wellness</t>
+          <t>44 Grid &amp; Transformers</t>
         </is>
       </c>
       <c r="C1138" s="4" t="inlineStr">
@@ -49813,12 +49813,12 @@
     <row r="1139">
       <c r="A1139" s="4" t="inlineStr">
         <is>
-          <t>Kraken Technologies</t>
+          <t>Fuse Energy</t>
         </is>
       </c>
       <c r="B1139" s="4" t="inlineStr">
         <is>
-          <t>44 Grid &amp; Transformers</t>
+          <t>X10 Batteries, EV, Waste &amp; Water</t>
         </is>
       </c>
       <c r="C1139" s="4" t="inlineStr">
@@ -49830,7 +49830,7 @@
     <row r="1140">
       <c r="A1140" s="4" t="inlineStr">
         <is>
-          <t>Fuse Energy</t>
+          <t>CMBlu Energy</t>
         </is>
       </c>
       <c r="B1140" s="4" t="inlineStr">
@@ -49847,12 +49847,12 @@
     <row r="1141">
       <c r="A1141" s="4" t="inlineStr">
         <is>
-          <t>CMBlu Energy</t>
+          <t>General Matter</t>
         </is>
       </c>
       <c r="B1141" s="4" t="inlineStr">
         <is>
-          <t>X10 Batteries, EV, Waste &amp; Water</t>
+          <t>02 Energy &amp; Industrial</t>
         </is>
       </c>
       <c r="C1141" s="4" t="inlineStr">
@@ -49864,7 +49864,7 @@
     <row r="1142">
       <c r="A1142" s="4" t="inlineStr">
         <is>
-          <t>General Matter</t>
+          <t>ENN Fusion</t>
         </is>
       </c>
       <c r="B1142" s="4" t="inlineStr">
@@ -49881,12 +49881,12 @@
     <row r="1143">
       <c r="A1143" s="4" t="inlineStr">
         <is>
-          <t>ENN Fusion</t>
+          <t>Rondo Energy</t>
         </is>
       </c>
       <c r="B1143" s="4" t="inlineStr">
         <is>
-          <t>02 Energy &amp; Industrial</t>
+          <t>X10 Batteries, EV, Waste &amp; Water</t>
         </is>
       </c>
       <c r="C1143" s="4" t="inlineStr">
@@ -49898,12 +49898,12 @@
     <row r="1144">
       <c r="A1144" s="4" t="inlineStr">
         <is>
-          <t>Rondo Energy</t>
+          <t>Osapiens</t>
         </is>
       </c>
       <c r="B1144" s="4" t="inlineStr">
         <is>
-          <t>X10 Batteries, EV, Waste &amp; Water</t>
+          <t>02 Energy &amp; Industrial</t>
         </is>
       </c>
       <c r="C1144" s="4" t="inlineStr">
@@ -49915,12 +49915,12 @@
     <row r="1145">
       <c r="A1145" s="4" t="inlineStr">
         <is>
-          <t>Osapiens</t>
+          <t>Canadian Solar</t>
         </is>
       </c>
       <c r="B1145" s="4" t="inlineStr">
         <is>
-          <t>02 Energy &amp; Industrial</t>
+          <t>X10 Batteries, EV, Waste &amp; Water</t>
         </is>
       </c>
       <c r="C1145" s="4" t="inlineStr">
@@ -49932,24 +49932,24 @@
     <row r="1146">
       <c r="A1146" s="4" t="inlineStr">
         <is>
-          <t>Canadian Solar</t>
+          <t>Esselunga</t>
         </is>
       </c>
       <c r="B1146" s="4" t="inlineStr">
         <is>
-          <t>X10 Batteries, EV, Waste &amp; Water</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1146" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
     </row>
     <row r="1147">
       <c r="A1147" s="4" t="inlineStr">
         <is>
-          <t>Esselunga</t>
+          <t>Conad</t>
         </is>
       </c>
       <c r="B1147" s="4" t="inlineStr">
@@ -49966,12 +49966,12 @@
     <row r="1148">
       <c r="A1148" s="4" t="inlineStr">
         <is>
-          <t>Conad</t>
+          <t>Giovanni Rana</t>
         </is>
       </c>
       <c r="B1148" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C1148" s="4" t="inlineStr">
@@ -49983,12 +49983,12 @@
     <row r="1149">
       <c r="A1149" s="4" t="inlineStr">
         <is>
-          <t>Giovanni Rana</t>
+          <t>Coop Switzerland</t>
         </is>
       </c>
       <c r="B1149" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1149" s="4" t="inlineStr">
@@ -50000,12 +50000,12 @@
     <row r="1150">
       <c r="A1150" s="4" t="inlineStr">
         <is>
-          <t>Coop Switzerland</t>
+          <t>Fenaco</t>
         </is>
       </c>
       <c r="B1150" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C1150" s="4" t="inlineStr">
@@ -50017,12 +50017,12 @@
     <row r="1151">
       <c r="A1151" s="4" t="inlineStr">
         <is>
-          <t>Fenaco</t>
+          <t>Spar Austria</t>
         </is>
       </c>
       <c r="B1151" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1151" s="4" t="inlineStr">
@@ -50034,7 +50034,7 @@
     <row r="1152">
       <c r="A1152" s="4" t="inlineStr">
         <is>
-          <t>Spar Austria</t>
+          <t>Grupo Eroski</t>
         </is>
       </c>
       <c r="B1152" s="4" t="inlineStr">
@@ -50051,7 +50051,7 @@
     <row r="1153">
       <c r="A1153" s="4" t="inlineStr">
         <is>
-          <t>Grupo Eroski</t>
+          <t>Tendam</t>
         </is>
       </c>
       <c r="B1153" s="4" t="inlineStr">
@@ -50068,7 +50068,7 @@
     <row r="1154">
       <c r="A1154" s="4" t="inlineStr">
         <is>
-          <t>Tendam</t>
+          <t>Co-op Group</t>
         </is>
       </c>
       <c r="B1154" s="4" t="inlineStr">
@@ -50085,12 +50085,12 @@
     <row r="1155">
       <c r="A1155" s="4" t="inlineStr">
         <is>
-          <t>Co-op Group</t>
+          <t>Arnold Clark</t>
         </is>
       </c>
       <c r="B1155" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>43 Mobility &amp; Automotive</t>
         </is>
       </c>
       <c r="C1155" s="4" t="inlineStr">
@@ -50102,12 +50102,12 @@
     <row r="1156">
       <c r="A1156" s="4" t="inlineStr">
         <is>
-          <t>Arnold Clark</t>
+          <t>StepStone Group</t>
         </is>
       </c>
       <c r="B1156" s="4" t="inlineStr">
         <is>
-          <t>43 Mobility &amp; Automotive</t>
+          <t>X01 Asset Mgmt, PE &amp; Trading Fir</t>
         </is>
       </c>
       <c r="C1156" s="4" t="inlineStr">
@@ -50119,7 +50119,7 @@
     <row r="1157">
       <c r="A1157" s="4" t="inlineStr">
         <is>
-          <t>StepStone Group</t>
+          <t>Hamilton Lane</t>
         </is>
       </c>
       <c r="B1157" s="4" t="inlineStr">
@@ -50136,12 +50136,12 @@
     <row r="1158">
       <c r="A1158" s="4" t="inlineStr">
         <is>
-          <t>Hamilton Lane</t>
+          <t>Rollins</t>
         </is>
       </c>
       <c r="B1158" s="4" t="inlineStr">
         <is>
-          <t>X01 Asset Mgmt, PE &amp; Trading Fir</t>
+          <t>18 Services &amp; Other</t>
         </is>
       </c>
       <c r="C1158" s="4" t="inlineStr">
@@ -50153,12 +50153,12 @@
     <row r="1159">
       <c r="A1159" s="4" t="inlineStr">
         <is>
-          <t>Rollins</t>
+          <t>Kimberly-Clark</t>
         </is>
       </c>
       <c r="B1159" s="4" t="inlineStr">
         <is>
-          <t>18 Services &amp; Other</t>
+          <t>53 Consumer &amp; Lifestyle</t>
         </is>
       </c>
       <c r="C1159" s="4" t="inlineStr">
@@ -50170,12 +50170,12 @@
     <row r="1160">
       <c r="A1160" s="4" t="inlineStr">
         <is>
-          <t>Kimberly-Clark</t>
+          <t>Couche-Tard</t>
         </is>
       </c>
       <c r="B1160" s="4" t="inlineStr">
         <is>
-          <t>53 Consumer &amp; Lifestyle</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1160" s="4" t="inlineStr">
@@ -50187,7 +50187,7 @@
     <row r="1161">
       <c r="A1161" s="4" t="inlineStr">
         <is>
-          <t>Couche-Tard</t>
+          <t>Dollarama</t>
         </is>
       </c>
       <c r="B1161" s="4" t="inlineStr">
@@ -50204,7 +50204,7 @@
     <row r="1162">
       <c r="A1162" s="4" t="inlineStr">
         <is>
-          <t>Dollarama</t>
+          <t>Empire Company</t>
         </is>
       </c>
       <c r="B1162" s="4" t="inlineStr">
@@ -50221,12 +50221,12 @@
     <row r="1163">
       <c r="A1163" s="4" t="inlineStr">
         <is>
-          <t>Empire Company</t>
+          <t>Saputo</t>
         </is>
       </c>
       <c r="B1163" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C1163" s="4" t="inlineStr">
@@ -50238,12 +50238,12 @@
     <row r="1164">
       <c r="A1164" s="4" t="inlineStr">
         <is>
-          <t>Saputo</t>
+          <t>FirstService</t>
         </is>
       </c>
       <c r="B1164" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>X02 Real Estate &amp; Building Produ</t>
         </is>
       </c>
       <c r="C1164" s="4" t="inlineStr">
@@ -50255,12 +50255,12 @@
     <row r="1165">
       <c r="A1165" s="4" t="inlineStr">
         <is>
-          <t>FirstService</t>
+          <t>Canadian Pacific Kansas City</t>
         </is>
       </c>
       <c r="B1165" s="4" t="inlineStr">
         <is>
-          <t>X02 Real Estate &amp; Building Produ</t>
+          <t>X12 Rail, Transit &amp; Road Infra</t>
         </is>
       </c>
       <c r="C1165" s="4" t="inlineStr">
@@ -50272,24 +50272,24 @@
     <row r="1166">
       <c r="A1166" s="4" t="inlineStr">
         <is>
-          <t>Canadian Pacific Kansas City</t>
+          <t>Electra.aero</t>
         </is>
       </c>
       <c r="B1166" s="4" t="inlineStr">
         <is>
-          <t>X12 Rail, Transit &amp; Road Infra</t>
+          <t>Aviation &amp; Aerospace Supplie</t>
         </is>
       </c>
       <c r="C1166" s="4" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="1167">
       <c r="A1167" s="4" t="inlineStr">
         <is>
-          <t>Electra.aero</t>
+          <t>Overair</t>
         </is>
       </c>
       <c r="B1167" s="4" t="inlineStr">
@@ -50306,7 +50306,7 @@
     <row r="1168">
       <c r="A1168" s="4" t="inlineStr">
         <is>
-          <t>Overair</t>
+          <t>CPI Aerostructures</t>
         </is>
       </c>
       <c r="B1168" s="4" t="inlineStr">
@@ -50323,7 +50323,7 @@
     <row r="1169">
       <c r="A1169" s="4" t="inlineStr">
         <is>
-          <t>CPI Aerostructures</t>
+          <t>Innovative Solutions &amp; Support</t>
         </is>
       </c>
       <c r="B1169" s="4" t="inlineStr">
@@ -50340,12 +50340,12 @@
     <row r="1170">
       <c r="A1170" s="4" t="inlineStr">
         <is>
-          <t>Innovative Solutions &amp; Support</t>
+          <t>Meyer Werft</t>
         </is>
       </c>
       <c r="B1170" s="4" t="inlineStr">
         <is>
-          <t>Aviation &amp; Aerospace Supplie</t>
+          <t>Maritime, Shipping &amp; Ports</t>
         </is>
       </c>
       <c r="C1170" s="4" t="inlineStr">
@@ -50357,7 +50357,7 @@
     <row r="1171">
       <c r="A1171" s="4" t="inlineStr">
         <is>
-          <t>Meyer Werft</t>
+          <t>Costamare Inc.</t>
         </is>
       </c>
       <c r="B1171" s="4" t="inlineStr">
@@ -50374,7 +50374,7 @@
     <row r="1172">
       <c r="A1172" s="4" t="inlineStr">
         <is>
-          <t>Costamare Inc.</t>
+          <t>HHLA (Hamburger Hafen und Logistik)</t>
         </is>
       </c>
       <c r="B1172" s="4" t="inlineStr">
@@ -50391,7 +50391,7 @@
     <row r="1173">
       <c r="A1173" s="4" t="inlineStr">
         <is>
-          <t>HHLA (Hamburger Hafen und Logistik)</t>
+          <t>Danaos Corporation</t>
         </is>
       </c>
       <c r="B1173" s="4" t="inlineStr">
@@ -50408,12 +50408,12 @@
     <row r="1174">
       <c r="A1174" s="4" t="inlineStr">
         <is>
-          <t>Danaos Corporation</t>
+          <t>SES AI</t>
         </is>
       </c>
       <c r="B1174" s="4" t="inlineStr">
         <is>
-          <t>Maritime, Shipping &amp; Ports</t>
+          <t>Batteries, EV, Waste &amp; Water</t>
         </is>
       </c>
       <c r="C1174" s="4" t="inlineStr">
@@ -50425,7 +50425,7 @@
     <row r="1175">
       <c r="A1175" s="4" t="inlineStr">
         <is>
-          <t>SES AI</t>
+          <t>Stem Inc</t>
         </is>
       </c>
       <c r="B1175" s="4" t="inlineStr">
@@ -50442,24 +50442,24 @@
     <row r="1176">
       <c r="A1176" s="4" t="inlineStr">
         <is>
-          <t>Stem Inc</t>
+          <t>Advance Intelligence Group</t>
         </is>
       </c>
       <c r="B1176" s="4" t="inlineStr">
         <is>
-          <t>Batteries, EV, Waste &amp; Water</t>
+          <t>09 Fintech</t>
         </is>
       </c>
       <c r="C1176" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="1177">
       <c r="A1177" s="4" t="inlineStr">
         <is>
-          <t>Advance Intelligence Group</t>
+          <t>BharatPe</t>
         </is>
       </c>
       <c r="B1177" s="4" t="inlineStr">
@@ -50476,12 +50476,12 @@
     <row r="1178">
       <c r="A1178" s="4" t="inlineStr">
         <is>
-          <t>BharatPe</t>
+          <t>Sygnum Bank</t>
         </is>
       </c>
       <c r="B1178" s="4" t="inlineStr">
         <is>
-          <t>09 Fintech</t>
+          <t>12 Trading &amp; Crypto</t>
         </is>
       </c>
       <c r="C1178" s="4" t="inlineStr">
@@ -50493,12 +50493,12 @@
     <row r="1179">
       <c r="A1179" s="4" t="inlineStr">
         <is>
-          <t>Sygnum Bank</t>
+          <t>Thought Machine</t>
         </is>
       </c>
       <c r="B1179" s="4" t="inlineStr">
         <is>
-          <t>12 Trading &amp; Crypto</t>
+          <t>09 Fintech</t>
         </is>
       </c>
       <c r="C1179" s="4" t="inlineStr">
@@ -50510,12 +50510,12 @@
     <row r="1180">
       <c r="A1180" s="4" t="inlineStr">
         <is>
-          <t>Thought Machine</t>
+          <t>Bestow</t>
         </is>
       </c>
       <c r="B1180" s="4" t="inlineStr">
         <is>
-          <t>09 Fintech</t>
+          <t>01 Banking &amp; Insurance</t>
         </is>
       </c>
       <c r="C1180" s="4" t="inlineStr">
@@ -50527,12 +50527,12 @@
     <row r="1181">
       <c r="A1181" s="4" t="inlineStr">
         <is>
-          <t>Bestow</t>
+          <t>Blockstream</t>
         </is>
       </c>
       <c r="B1181" s="4" t="inlineStr">
         <is>
-          <t>01 Banking &amp; Insurance</t>
+          <t>12 Trading &amp; Crypto</t>
         </is>
       </c>
       <c r="C1181" s="4" t="inlineStr">
@@ -50544,12 +50544,12 @@
     <row r="1182">
       <c r="A1182" s="4" t="inlineStr">
         <is>
-          <t>Blockstream</t>
+          <t>Geidea</t>
         </is>
       </c>
       <c r="B1182" s="4" t="inlineStr">
         <is>
-          <t>12 Trading &amp; Crypto</t>
+          <t>09 Fintech</t>
         </is>
       </c>
       <c r="C1182" s="4" t="inlineStr">
@@ -50561,12 +50561,12 @@
     <row r="1183">
       <c r="A1183" s="4" t="inlineStr">
         <is>
-          <t>Geidea</t>
+          <t>Matrixport</t>
         </is>
       </c>
       <c r="B1183" s="4" t="inlineStr">
         <is>
-          <t>09 Fintech</t>
+          <t>12 Trading &amp; Crypto</t>
         </is>
       </c>
       <c r="C1183" s="4" t="inlineStr">
@@ -50578,12 +50578,12 @@
     <row r="1184">
       <c r="A1184" s="4" t="inlineStr">
         <is>
-          <t>Matrixport</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="B1184" s="4" t="inlineStr">
         <is>
-          <t>12 Trading &amp; Crypto</t>
+          <t>09 Fintech</t>
         </is>
       </c>
       <c r="C1184" s="4" t="inlineStr">
@@ -50595,7 +50595,7 @@
     <row r="1185">
       <c r="A1185" s="4" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Vise</t>
         </is>
       </c>
       <c r="B1185" s="4" t="inlineStr">
@@ -50612,12 +50612,12 @@
     <row r="1186">
       <c r="A1186" s="4" t="inlineStr">
         <is>
-          <t>Vise</t>
+          <t>Back Market</t>
         </is>
       </c>
       <c r="B1186" s="4" t="inlineStr">
         <is>
-          <t>09 Fintech</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1186" s="4" t="inlineStr">
@@ -50629,12 +50629,12 @@
     <row r="1187">
       <c r="A1187" s="4" t="inlineStr">
         <is>
-          <t>Back Market</t>
+          <t>Jam City</t>
         </is>
       </c>
       <c r="B1187" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>29 Tech Media &amp; Gaming</t>
         </is>
       </c>
       <c r="C1187" s="4" t="inlineStr">
@@ -50646,12 +50646,12 @@
     <row r="1188">
       <c r="A1188" s="4" t="inlineStr">
         <is>
-          <t>Jam City</t>
+          <t>NotCo</t>
         </is>
       </c>
       <c r="B1188" s="4" t="inlineStr">
         <is>
-          <t>29 Tech Media &amp; Gaming</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C1188" s="4" t="inlineStr">
@@ -50663,12 +50663,12 @@
     <row r="1189">
       <c r="A1189" s="4" t="inlineStr">
         <is>
-          <t>NotCo</t>
+          <t>SuperPlay</t>
         </is>
       </c>
       <c r="B1189" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>29 Tech Media &amp; Gaming</t>
         </is>
       </c>
       <c r="C1189" s="4" t="inlineStr">
@@ -50680,12 +50680,12 @@
     <row r="1190">
       <c r="A1190" s="4" t="inlineStr">
         <is>
-          <t>SuperPlay</t>
+          <t>Perfect Day</t>
         </is>
       </c>
       <c r="B1190" s="4" t="inlineStr">
         <is>
-          <t>29 Tech Media &amp; Gaming</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C1190" s="4" t="inlineStr">
@@ -50697,12 +50697,12 @@
     <row r="1191">
       <c r="A1191" s="4" t="inlineStr">
         <is>
-          <t>Perfect Day</t>
+          <t>Nana Direct</t>
         </is>
       </c>
       <c r="B1191" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1191" s="4" t="inlineStr">
@@ -50714,7 +50714,7 @@
     <row r="1192">
       <c r="A1192" s="4" t="inlineStr">
         <is>
-          <t>Nana Direct</t>
+          <t>Petlove</t>
         </is>
       </c>
       <c r="B1192" s="4" t="inlineStr">
@@ -50731,12 +50731,12 @@
     <row r="1193">
       <c r="A1193" s="4" t="inlineStr">
         <is>
-          <t>Petlove</t>
+          <t>Thyme Care</t>
         </is>
       </c>
       <c r="B1193" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>X03 CDMO, CRO &amp; Life-Science Tools</t>
         </is>
       </c>
       <c r="C1193" s="4" t="inlineStr">
@@ -50748,12 +50748,12 @@
     <row r="1194">
       <c r="A1194" s="4" t="inlineStr">
         <is>
-          <t>Thyme Care</t>
+          <t>Nihon Kohden</t>
         </is>
       </c>
       <c r="B1194" s="4" t="inlineStr">
         <is>
-          <t>X03 CDMO, CRO &amp; Life-Science Tools</t>
+          <t>42 Health &amp; Wellness</t>
         </is>
       </c>
       <c r="C1194" s="4" t="inlineStr">
@@ -50765,7 +50765,7 @@
     <row r="1195">
       <c r="A1195" s="4" t="inlineStr">
         <is>
-          <t>Nihon Kohden</t>
+          <t>MiRus</t>
         </is>
       </c>
       <c r="B1195" s="4" t="inlineStr">
@@ -50782,29 +50782,29 @@
     <row r="1196">
       <c r="A1196" s="4" t="inlineStr">
         <is>
-          <t>MiRus</t>
+          <t>Bigo</t>
         </is>
       </c>
       <c r="B1196" s="4" t="inlineStr">
         <is>
-          <t>42 Health &amp; Wellness</t>
+          <t>29 Tech Media &amp; Gaming</t>
         </is>
       </c>
       <c r="C1196" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
     </row>
     <row r="1197">
       <c r="A1197" s="4" t="inlineStr">
         <is>
-          <t>Bigo</t>
+          <t>Olam Agri</t>
         </is>
       </c>
       <c r="B1197" s="4" t="inlineStr">
         <is>
-          <t>29 Tech Media &amp; Gaming</t>
+          <t>X05 Agriculture &amp; AgTech</t>
         </is>
       </c>
       <c r="C1197" s="4" t="inlineStr">
@@ -50816,12 +50816,12 @@
     <row r="1198">
       <c r="A1198" s="4" t="inlineStr">
         <is>
-          <t>Olam Agri</t>
+          <t>VNLife (VNPay)</t>
         </is>
       </c>
       <c r="B1198" s="4" t="inlineStr">
         <is>
-          <t>X05 Agriculture &amp; AgTech</t>
+          <t>09 Fintech</t>
         </is>
       </c>
       <c r="C1198" s="4" t="inlineStr">
@@ -50833,12 +50833,12 @@
     <row r="1199">
       <c r="A1199" s="4" t="inlineStr">
         <is>
-          <t>VNLife (VNPay)</t>
+          <t>Press Metal</t>
         </is>
       </c>
       <c r="B1199" s="4" t="inlineStr">
         <is>
-          <t>09 Fintech</t>
+          <t>X04 Mining, Metals &amp; Commodities</t>
         </is>
       </c>
       <c r="C1199" s="4" t="inlineStr">
@@ -50850,12 +50850,12 @@
     <row r="1200">
       <c r="A1200" s="4" t="inlineStr">
         <is>
-          <t>Press Metal</t>
+          <t>Top Glove</t>
         </is>
       </c>
       <c r="B1200" s="4" t="inlineStr">
         <is>
-          <t>X04 Mining, Metals &amp; Commodities</t>
+          <t>42 Health &amp; Wellness</t>
         </is>
       </c>
       <c r="C1200" s="4" t="inlineStr">
@@ -50867,12 +50867,12 @@
     <row r="1201">
       <c r="A1201" s="4" t="inlineStr">
         <is>
-          <t>Top Glove</t>
+          <t>Genting Group</t>
         </is>
       </c>
       <c r="B1201" s="4" t="inlineStr">
         <is>
-          <t>42 Health &amp; Wellness</t>
+          <t>16 Travel &amp; Hospitality</t>
         </is>
       </c>
       <c r="C1201" s="4" t="inlineStr">
@@ -50884,12 +50884,12 @@
     <row r="1202">
       <c r="A1202" s="4" t="inlineStr">
         <is>
-          <t>Genting Group</t>
+          <t>Touch n Go Digital</t>
         </is>
       </c>
       <c r="B1202" s="4" t="inlineStr">
         <is>
-          <t>16 Travel &amp; Hospitality</t>
+          <t>09 Fintech</t>
         </is>
       </c>
       <c r="C1202" s="4" t="inlineStr">
@@ -50901,12 +50901,12 @@
     <row r="1203">
       <c r="A1203" s="4" t="inlineStr">
         <is>
-          <t>Touch n Go Digital</t>
+          <t>Aerodyne Group</t>
         </is>
       </c>
       <c r="B1203" s="4" t="inlineStr">
         <is>
-          <t>09 Fintech</t>
+          <t>33 Automation &amp; Robotics</t>
         </is>
       </c>
       <c r="C1203" s="4" t="inlineStr">
@@ -50918,12 +50918,12 @@
     <row r="1204">
       <c r="A1204" s="4" t="inlineStr">
         <is>
-          <t>Aerodyne Group</t>
+          <t>GCash (Mynt)</t>
         </is>
       </c>
       <c r="B1204" s="4" t="inlineStr">
         <is>
-          <t>33 Automation &amp; Robotics</t>
+          <t>09 Fintech</t>
         </is>
       </c>
       <c r="C1204" s="4" t="inlineStr">
@@ -50935,12 +50935,12 @@
     <row r="1205">
       <c r="A1205" s="4" t="inlineStr">
         <is>
-          <t>GCash (Mynt)</t>
+          <t>Converge ICT</t>
         </is>
       </c>
       <c r="B1205" s="4" t="inlineStr">
         <is>
-          <t>09 Fintech</t>
+          <t>48 Telecom &amp; Space</t>
         </is>
       </c>
       <c r="C1205" s="4" t="inlineStr">
@@ -50952,12 +50952,12 @@
     <row r="1206">
       <c r="A1206" s="4" t="inlineStr">
         <is>
-          <t>Converge ICT</t>
+          <t>Unilever</t>
         </is>
       </c>
       <c r="B1206" s="4" t="inlineStr">
         <is>
-          <t>48 Telecom &amp; Space</t>
+          <t>53 Consumer &amp; Lifestyle</t>
         </is>
       </c>
       <c r="C1206" s="4" t="inlineStr">
@@ -50969,12 +50969,12 @@
     <row r="1207">
       <c r="A1207" s="4" t="inlineStr">
         <is>
-          <t>Unilever</t>
+          <t>Pernod Ricard</t>
         </is>
       </c>
       <c r="B1207" s="4" t="inlineStr">
         <is>
-          <t>53 Consumer &amp; Lifestyle</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C1207" s="4" t="inlineStr">
@@ -50986,7 +50986,7 @@
     <row r="1208">
       <c r="A1208" s="4" t="inlineStr">
         <is>
-          <t>Pernod Ricard</t>
+          <t>Lindt &amp; Spruengli</t>
         </is>
       </c>
       <c r="B1208" s="4" t="inlineStr">
@@ -51003,7 +51003,7 @@
     <row r="1209">
       <c r="A1209" s="4" t="inlineStr">
         <is>
-          <t>Lindt &amp; Spruengli</t>
+          <t>Lotus Bakeries</t>
         </is>
       </c>
       <c r="B1209" s="4" t="inlineStr">
@@ -51020,7 +51020,7 @@
     <row r="1210">
       <c r="A1210" s="4" t="inlineStr">
         <is>
-          <t>Lotus Bakeries</t>
+          <t>Emmi</t>
         </is>
       </c>
       <c r="B1210" s="4" t="inlineStr">
@@ -51037,12 +51037,12 @@
     <row r="1211">
       <c r="A1211" s="4" t="inlineStr">
         <is>
-          <t>Emmi</t>
+          <t>J Sainsbury</t>
         </is>
       </c>
       <c r="B1211" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1211" s="4" t="inlineStr">
@@ -51054,7 +51054,7 @@
     <row r="1212">
       <c r="A1212" s="4" t="inlineStr">
         <is>
-          <t>J Sainsbury</t>
+          <t>Marks and Spencer</t>
         </is>
       </c>
       <c r="B1212" s="4" t="inlineStr">
@@ -51071,7 +51071,7 @@
     <row r="1213">
       <c r="A1213" s="4" t="inlineStr">
         <is>
-          <t>Marks and Spencer</t>
+          <t>Zabka Group</t>
         </is>
       </c>
       <c r="B1213" s="4" t="inlineStr">
@@ -51088,7 +51088,7 @@
     <row r="1214">
       <c r="A1214" s="4" t="inlineStr">
         <is>
-          <t>Zabka Group</t>
+          <t>Dino Polska</t>
         </is>
       </c>
       <c r="B1214" s="4" t="inlineStr">
@@ -51105,7 +51105,7 @@
     <row r="1215">
       <c r="A1215" s="4" t="inlineStr">
         <is>
-          <t>Dino Polska</t>
+          <t>Maplebear (Instacart)</t>
         </is>
       </c>
       <c r="B1215" s="4" t="inlineStr">
@@ -51122,12 +51122,12 @@
     <row r="1216">
       <c r="A1216" s="4" t="inlineStr">
         <is>
-          <t>Maplebear (Instacart)</t>
+          <t>CloudKitchens</t>
         </is>
       </c>
       <c r="B1216" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>18 Services &amp; Other</t>
         </is>
       </c>
       <c r="C1216" s="4" t="inlineStr">
@@ -51139,12 +51139,12 @@
     <row r="1217">
       <c r="A1217" s="4" t="inlineStr">
         <is>
-          <t>CloudKitchens</t>
+          <t>Tito's Handmade Vodka</t>
         </is>
       </c>
       <c r="B1217" s="4" t="inlineStr">
         <is>
-          <t>18 Services &amp; Other</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C1217" s="4" t="inlineStr">
@@ -51156,7 +51156,7 @@
     <row r="1218">
       <c r="A1218" s="4" t="inlineStr">
         <is>
-          <t>Tito's Handmade Vodka</t>
+          <t>Tillamook County Creamery Association</t>
         </is>
       </c>
       <c r="B1218" s="4" t="inlineStr">
@@ -51173,7 +51173,7 @@
     <row r="1219">
       <c r="A1219" s="4" t="inlineStr">
         <is>
-          <t>Tillamook County Creamery Association</t>
+          <t>Southern Glazer's Wine &amp; Spirits</t>
         </is>
       </c>
       <c r="B1219" s="4" t="inlineStr">
@@ -51190,12 +51190,12 @@
     <row r="1220">
       <c r="A1220" s="4" t="inlineStr">
         <is>
-          <t>Southern Glazer's Wine &amp; Spirits</t>
+          <t>Ariat International</t>
         </is>
       </c>
       <c r="B1220" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>X08 Sporting Goods &amp; Fitness</t>
         </is>
       </c>
       <c r="C1220" s="4" t="inlineStr">
@@ -51207,12 +51207,12 @@
     <row r="1221">
       <c r="A1221" s="4" t="inlineStr">
         <is>
-          <t>Ariat International</t>
+          <t>Backcountry.com</t>
         </is>
       </c>
       <c r="B1221" s="4" t="inlineStr">
         <is>
-          <t>X08 Sporting Goods &amp; Fitness</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1221" s="4" t="inlineStr">
@@ -51224,12 +51224,12 @@
     <row r="1222">
       <c r="A1222" s="4" t="inlineStr">
         <is>
-          <t>Backcountry.com</t>
+          <t>Uniswap Labs</t>
         </is>
       </c>
       <c r="B1222" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>12 Trading &amp; Crypto</t>
         </is>
       </c>
       <c r="C1222" s="4" t="inlineStr">
@@ -51241,7 +51241,7 @@
     <row r="1223">
       <c r="A1223" s="4" t="inlineStr">
         <is>
-          <t>Uniswap Labs</t>
+          <t>Tools for Humanity (World)</t>
         </is>
       </c>
       <c r="B1223" s="4" t="inlineStr">
@@ -51258,7 +51258,7 @@
     <row r="1224">
       <c r="A1224" s="4" t="inlineStr">
         <is>
-          <t>Tools for Humanity (World)</t>
+          <t>Offchain Labs</t>
         </is>
       </c>
       <c r="B1224" s="4" t="inlineStr">
@@ -51275,12 +51275,12 @@
     <row r="1225">
       <c r="A1225" s="4" t="inlineStr">
         <is>
-          <t>Offchain Labs</t>
+          <t>Zijin Mining</t>
         </is>
       </c>
       <c r="B1225" s="4" t="inlineStr">
         <is>
-          <t>12 Trading &amp; Crypto</t>
+          <t>X04 Mining, Metals &amp; Commodities</t>
         </is>
       </c>
       <c r="C1225" s="4" t="inlineStr">
@@ -51292,12 +51292,12 @@
     <row r="1226">
       <c r="A1226" s="4" t="inlineStr">
         <is>
-          <t>Zijin Mining</t>
+          <t>Hengli Group</t>
         </is>
       </c>
       <c r="B1226" s="4" t="inlineStr">
         <is>
-          <t>X04 Mining, Metals &amp; Commodities</t>
+          <t>21 Materials &amp; Mech Parts</t>
         </is>
       </c>
       <c r="C1226" s="4" t="inlineStr">
@@ -51309,12 +51309,12 @@
     <row r="1227">
       <c r="A1227" s="4" t="inlineStr">
         <is>
-          <t>Hengli Group</t>
+          <t>Zeekr Intelligent Technology</t>
         </is>
       </c>
       <c r="B1227" s="4" t="inlineStr">
         <is>
-          <t>21 Materials &amp; Mech Parts</t>
+          <t>43 Mobility &amp; Automotive</t>
         </is>
       </c>
       <c r="C1227" s="4" t="inlineStr">
@@ -51326,7 +51326,7 @@
     <row r="1228">
       <c r="A1228" s="4" t="inlineStr">
         <is>
-          <t>Zeekr Intelligent Technology</t>
+          <t>Avatr Technology</t>
         </is>
       </c>
       <c r="B1228" s="4" t="inlineStr">
@@ -51343,12 +51343,12 @@
     <row r="1229">
       <c r="A1229" s="4" t="inlineStr">
         <is>
-          <t>Avatr Technology</t>
+          <t>State Grid Corporation of China</t>
         </is>
       </c>
       <c r="B1229" s="4" t="inlineStr">
         <is>
-          <t>43 Mobility &amp; Automotive</t>
+          <t>44 Grid &amp; Transformers</t>
         </is>
       </c>
       <c r="C1229" s="4" t="inlineStr">
@@ -51360,12 +51360,12 @@
     <row r="1230">
       <c r="A1230" s="4" t="inlineStr">
         <is>
-          <t>State Grid Corporation of China</t>
+          <t>CRRC Corporation</t>
         </is>
       </c>
       <c r="B1230" s="4" t="inlineStr">
         <is>
-          <t>44 Grid &amp; Transformers</t>
+          <t>X12 Rail, Transit &amp; Road Infra</t>
         </is>
       </c>
       <c r="C1230" s="4" t="inlineStr">
@@ -51377,12 +51377,12 @@
     <row r="1231">
       <c r="A1231" s="4" t="inlineStr">
         <is>
-          <t>CRRC Corporation</t>
+          <t>Spring Airlines</t>
         </is>
       </c>
       <c r="B1231" s="4" t="inlineStr">
         <is>
-          <t>X12 Rail, Transit &amp; Road Infra</t>
+          <t>16 Travel &amp; Hospitality</t>
         </is>
       </c>
       <c r="C1231" s="4" t="inlineStr">
@@ -51394,12 +51394,12 @@
     <row r="1232">
       <c r="A1232" s="4" t="inlineStr">
         <is>
-          <t>Spring Airlines</t>
+          <t>Eastroc Beverage (Dongpeng)</t>
         </is>
       </c>
       <c r="B1232" s="4" t="inlineStr">
         <is>
-          <t>16 Travel &amp; Hospitality</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C1232" s="4" t="inlineStr">
@@ -51411,12 +51411,12 @@
     <row r="1233">
       <c r="A1233" s="4" t="inlineStr">
         <is>
-          <t>Eastroc Beverage (Dongpeng)</t>
+          <t>Baichuan Intelligence</t>
         </is>
       </c>
       <c r="B1233" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>17 AI Cloud &amp; Data</t>
         </is>
       </c>
       <c r="C1233" s="4" t="inlineStr">
@@ -51428,12 +51428,12 @@
     <row r="1234">
       <c r="A1234" s="4" t="inlineStr">
         <is>
-          <t>Baichuan Intelligence</t>
+          <t>CMOC Group</t>
         </is>
       </c>
       <c r="B1234" s="4" t="inlineStr">
         <is>
-          <t>17 AI Cloud &amp; Data</t>
+          <t>X04 Mining, Metals &amp; Commodities</t>
         </is>
       </c>
       <c r="C1234" s="4" t="inlineStr">
@@ -51445,24 +51445,24 @@
     <row r="1235">
       <c r="A1235" s="4" t="inlineStr">
         <is>
-          <t>CMOC Group</t>
+          <t>Heven AeroTech</t>
         </is>
       </c>
       <c r="B1235" s="4" t="inlineStr">
         <is>
-          <t>X04 Mining, Metals &amp; Commodities</t>
+          <t>56 Robotics AI</t>
         </is>
       </c>
       <c r="C1235" s="4" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="1236">
       <c r="A1236" s="4" t="inlineStr">
         <is>
-          <t>Heven AeroTech</t>
+          <t>Lightwheel</t>
         </is>
       </c>
       <c r="B1236" s="4" t="inlineStr">
@@ -51479,7 +51479,7 @@
     <row r="1237">
       <c r="A1237" s="4" t="inlineStr">
         <is>
-          <t>Lightwheel</t>
+          <t>PaXini Tech</t>
         </is>
       </c>
       <c r="B1237" s="4" t="inlineStr">
@@ -51496,12 +51496,12 @@
     <row r="1238">
       <c r="A1238" s="4" t="inlineStr">
         <is>
-          <t>PaXini Tech</t>
+          <t>UForce</t>
         </is>
       </c>
       <c r="B1238" s="4" t="inlineStr">
         <is>
-          <t>56 Robotics AI</t>
+          <t>32 Defense &amp; Industrial AI</t>
         </is>
       </c>
       <c r="C1238" s="4" t="inlineStr">
@@ -51513,12 +51513,12 @@
     <row r="1239">
       <c r="A1239" s="4" t="inlineStr">
         <is>
-          <t>UForce</t>
+          <t>ZaiNar</t>
         </is>
       </c>
       <c r="B1239" s="4" t="inlineStr">
         <is>
-          <t>32 Defense &amp; Industrial AI</t>
+          <t>56 Robotics AI</t>
         </is>
       </c>
       <c r="C1239" s="4" t="inlineStr">
@@ -51530,12 +51530,12 @@
     <row r="1240">
       <c r="A1240" s="4" t="inlineStr">
         <is>
-          <t>ZaiNar</t>
+          <t>Blue Origin</t>
         </is>
       </c>
       <c r="B1240" s="4" t="inlineStr">
         <is>
-          <t>56 Robotics AI</t>
+          <t>48 Telecom &amp; Space</t>
         </is>
       </c>
       <c r="C1240" s="4" t="inlineStr">
@@ -51547,7 +51547,7 @@
     <row r="1241">
       <c r="A1241" s="4" t="inlineStr">
         <is>
-          <t>Blue Origin</t>
+          <t>Gilmour Space Technologies</t>
         </is>
       </c>
       <c r="B1241" s="4" t="inlineStr">
@@ -51564,7 +51564,7 @@
     <row r="1242">
       <c r="A1242" s="4" t="inlineStr">
         <is>
-          <t>Gilmour Space Technologies</t>
+          <t>Synspective</t>
         </is>
       </c>
       <c r="B1242" s="4" t="inlineStr">
@@ -51581,12 +51581,12 @@
     <row r="1243">
       <c r="A1243" s="4" t="inlineStr">
         <is>
-          <t>Synspective</t>
+          <t>TAE Technologies</t>
         </is>
       </c>
       <c r="B1243" s="4" t="inlineStr">
         <is>
-          <t>48 Telecom &amp; Space</t>
+          <t>32 Defense &amp; Industrial AI</t>
         </is>
       </c>
       <c r="C1243" s="4" t="inlineStr">
@@ -51598,12 +51598,12 @@
     <row r="1244">
       <c r="A1244" s="4" t="inlineStr">
         <is>
-          <t>TAE Technologies</t>
+          <t>Arena</t>
         </is>
       </c>
       <c r="B1244" s="4" t="inlineStr">
         <is>
-          <t>32 Defense &amp; Industrial AI</t>
+          <t>08 Devtools &amp; Integration</t>
         </is>
       </c>
       <c r="C1244" s="4" t="inlineStr">
@@ -51615,12 +51615,12 @@
     <row r="1245">
       <c r="A1245" s="4" t="inlineStr">
         <is>
-          <t>Arena</t>
+          <t>Radiology Partners</t>
         </is>
       </c>
       <c r="B1245" s="4" t="inlineStr">
         <is>
-          <t>08 Devtools &amp; Integration</t>
+          <t>42 Health &amp; Wellness</t>
         </is>
       </c>
       <c r="C1245" s="4" t="inlineStr">
@@ -51632,7 +51632,7 @@
     <row r="1246">
       <c r="A1246" s="4" t="inlineStr">
         <is>
-          <t>Radiology Partners</t>
+          <t>Colossal Biosciences</t>
         </is>
       </c>
       <c r="B1246" s="4" t="inlineStr">
@@ -51649,7 +51649,7 @@
     <row r="1247">
       <c r="A1247" s="4" t="inlineStr">
         <is>
-          <t>Colossal Biosciences</t>
+          <t>Ascentage Pharma</t>
         </is>
       </c>
       <c r="B1247" s="4" t="inlineStr">
@@ -51666,7 +51666,7 @@
     <row r="1248">
       <c r="A1248" s="4" t="inlineStr">
         <is>
-          <t>Ascentage Pharma</t>
+          <t>Elekta</t>
         </is>
       </c>
       <c r="B1248" s="4" t="inlineStr">
@@ -51683,7 +51683,7 @@
     <row r="1249">
       <c r="A1249" s="4" t="inlineStr">
         <is>
-          <t>Elekta</t>
+          <t>Hemab Therapeutics</t>
         </is>
       </c>
       <c r="B1249" s="4" t="inlineStr">
@@ -51700,7 +51700,7 @@
     <row r="1250">
       <c r="A1250" s="4" t="inlineStr">
         <is>
-          <t>Hemab Therapeutics</t>
+          <t>Parabilis Medicines</t>
         </is>
       </c>
       <c r="B1250" s="4" t="inlineStr">
@@ -51717,7 +51717,7 @@
     <row r="1251">
       <c r="A1251" s="4" t="inlineStr">
         <is>
-          <t>Parabilis Medicines</t>
+          <t>Kestra Medical Technologies</t>
         </is>
       </c>
       <c r="B1251" s="4" t="inlineStr">
@@ -51734,7 +51734,7 @@
     <row r="1252">
       <c r="A1252" s="4" t="inlineStr">
         <is>
-          <t>Kestra Medical Technologies</t>
+          <t>Kriya Therapeutics</t>
         </is>
       </c>
       <c r="B1252" s="4" t="inlineStr">
@@ -51751,7 +51751,7 @@
     <row r="1253">
       <c r="A1253" s="4" t="inlineStr">
         <is>
-          <t>Kriya Therapeutics</t>
+          <t>Everest Medicines</t>
         </is>
       </c>
       <c r="B1253" s="4" t="inlineStr">
@@ -51768,7 +51768,7 @@
     <row r="1254">
       <c r="A1254" s="4" t="inlineStr">
         <is>
-          <t>Everest Medicines</t>
+          <t>Galapagos NV</t>
         </is>
       </c>
       <c r="B1254" s="4" t="inlineStr">
@@ -51785,29 +51785,29 @@
     <row r="1255">
       <c r="A1255" s="4" t="inlineStr">
         <is>
-          <t>Galapagos NV</t>
+          <t>Cuckoo Electronics</t>
         </is>
       </c>
       <c r="B1255" s="4" t="inlineStr">
         <is>
-          <t>42 Health &amp; Wellness</t>
+          <t>49 Home &amp; Living</t>
         </is>
       </c>
       <c r="C1255" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
     </row>
     <row r="1256">
       <c r="A1256" s="4" t="inlineStr">
         <is>
-          <t>Cuckoo Electronics</t>
+          <t>Saigon Co.op</t>
         </is>
       </c>
       <c r="B1256" s="4" t="inlineStr">
         <is>
-          <t>49 Home &amp; Living</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1256" s="4" t="inlineStr">
@@ -51819,12 +51819,12 @@
     <row r="1257">
       <c r="A1257" s="4" t="inlineStr">
         <is>
-          <t>Saigon Co.op</t>
+          <t>VNG Corporation</t>
         </is>
       </c>
       <c r="B1257" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>29 Tech Media &amp; Gaming</t>
         </is>
       </c>
       <c r="C1257" s="4" t="inlineStr">
@@ -51836,12 +51836,12 @@
     <row r="1258">
       <c r="A1258" s="4" t="inlineStr">
         <is>
-          <t>VNG Corporation</t>
+          <t>Alabbar Enterprises</t>
         </is>
       </c>
       <c r="B1258" s="4" t="inlineStr">
         <is>
-          <t>29 Tech Media &amp; Gaming</t>
+          <t>19 Gulf Sovereign &amp; Tourism</t>
         </is>
       </c>
       <c r="C1258" s="4" t="inlineStr">
@@ -51853,12 +51853,12 @@
     <row r="1259">
       <c r="A1259" s="4" t="inlineStr">
         <is>
-          <t>Alabbar Enterprises</t>
+          <t>Boyner Group</t>
         </is>
       </c>
       <c r="B1259" s="4" t="inlineStr">
         <is>
-          <t>19 Gulf Sovereign &amp; Tourism</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1259" s="4" t="inlineStr">
@@ -51870,12 +51870,12 @@
     <row r="1260">
       <c r="A1260" s="4" t="inlineStr">
         <is>
-          <t>Boyner Group</t>
+          <t>DeFacto</t>
         </is>
       </c>
       <c r="B1260" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>53 Consumer &amp; Lifestyle</t>
         </is>
       </c>
       <c r="C1260" s="4" t="inlineStr">
@@ -51887,12 +51887,12 @@
     <row r="1261">
       <c r="A1261" s="4" t="inlineStr">
         <is>
-          <t>DeFacto</t>
+          <t>Sahibinden</t>
         </is>
       </c>
       <c r="B1261" s="4" t="inlineStr">
         <is>
-          <t>53 Consumer &amp; Lifestyle</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C1261" s="4" t="inlineStr">
@@ -51904,12 +51904,12 @@
     <row r="1262">
       <c r="A1262" s="4" t="inlineStr">
         <is>
-          <t>Sahibinden</t>
+          <t>Eti Gida</t>
         </is>
       </c>
       <c r="B1262" s="4" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>04 Food &amp; Beverage</t>
         </is>
       </c>
       <c r="C1262" s="4" t="inlineStr">
@@ -51921,7 +51921,7 @@
     <row r="1263">
       <c r="A1263" s="4" t="inlineStr">
         <is>
-          <t>Eti Gida</t>
+          <t>Bauducco</t>
         </is>
       </c>
       <c r="B1263" s="4" t="inlineStr">
@@ -51938,7 +51938,7 @@
     <row r="1264">
       <c r="A1264" s="4" t="inlineStr">
         <is>
-          <t>Bauducco</t>
+          <t>Arcor</t>
         </is>
       </c>
       <c r="B1264" s="4" t="inlineStr">
@@ -51955,12 +51955,12 @@
     <row r="1265">
       <c r="A1265" s="4" t="inlineStr">
         <is>
-          <t>Arcor</t>
+          <t>Amplifon</t>
         </is>
       </c>
       <c r="B1265" s="4" t="inlineStr">
         <is>
-          <t>04 Food &amp; Beverage</t>
+          <t>42 Health &amp; Wellness</t>
         </is>
       </c>
       <c r="C1265" s="4" t="inlineStr">
@@ -51972,7 +51972,7 @@
     <row r="1266">
       <c r="A1266" s="4" t="inlineStr">
         <is>
-          <t>Amplifon</t>
+          <t>Fresenius SE</t>
         </is>
       </c>
       <c r="B1266" s="4" t="inlineStr">
@@ -51989,7 +51989,7 @@
     <row r="1267">
       <c r="A1267" s="4" t="inlineStr">
         <is>
-          <t>Fresenius SE</t>
+          <t>Convatec</t>
         </is>
       </c>
       <c r="B1267" s="4" t="inlineStr">
@@ -52006,7 +52006,7 @@
     <row r="1268">
       <c r="A1268" s="4" t="inlineStr">
         <is>
-          <t>Convatec</t>
+          <t>Sandoz</t>
         </is>
       </c>
       <c r="B1268" s="4" t="inlineStr">
@@ -52023,7 +52023,7 @@
     <row r="1269">
       <c r="A1269" s="4" t="inlineStr">
         <is>
-          <t>Sandoz</t>
+          <t>Grifols</t>
         </is>
       </c>
       <c r="B1269" s="4" t="inlineStr">
@@ -52040,12 +52040,12 @@
     <row r="1270">
       <c r="A1270" s="4" t="inlineStr">
         <is>
-          <t>Grifols</t>
+          <t>Nordea</t>
         </is>
       </c>
       <c r="B1270" s="4" t="inlineStr">
         <is>
-          <t>42 Health &amp; Wellness</t>
+          <t>01 Banking &amp; Insurance</t>
         </is>
       </c>
       <c r="C1270" s="4" t="inlineStr">
@@ -52057,7 +52057,7 @@
     <row r="1271">
       <c r="A1271" s="4" t="inlineStr">
         <is>
-          <t>Nordea</t>
+          <t>Danske Bank</t>
         </is>
       </c>
       <c r="B1271" s="4" t="inlineStr">
@@ -52074,7 +52074,7 @@
     <row r="1272">
       <c r="A1272" s="4" t="inlineStr">
         <is>
-          <t>Danske Bank</t>
+          <t>DNB</t>
         </is>
       </c>
       <c r="B1272" s="4" t="inlineStr">
@@ -52091,7 +52091,7 @@
     <row r="1273">
       <c r="A1273" s="4" t="inlineStr">
         <is>
-          <t>DNB</t>
+          <t>ABN AMRO</t>
         </is>
       </c>
       <c r="B1273" s="4" t="inlineStr">
@@ -52108,17 +52108,17 @@
     <row r="1274">
       <c r="A1274" s="4" t="inlineStr">
         <is>
-          <t>ABN AMRO</t>
+          <t>Motive (formerly KeepTruckin)</t>
         </is>
       </c>
       <c r="B1274" s="4" t="inlineStr">
         <is>
-          <t>01 Banking &amp; Insurance</t>
+          <t>24 Logistics</t>
         </is>
       </c>
       <c r="C1274" s="4" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>B</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wave 14 v3: 304 verified; Krafton excluded for team licensing deals
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TE8a9ptd2NGPUtY6iZfzkb
</commit_message>
<xml_diff>
--- a/reports/F1-Wave14-V3-Broad-2026-10.xlsx
+++ b/reports/F1-Wave14-V3-Broad-2026-10.xlsx
@@ -90,7 +90,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'24 Logistics'!$A$3:$T$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'25 IT Services &amp; Consulting'!$A$3:$T$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'28 AI Data Services'!$A$3:$T$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'29 Tech Media &amp; Gaming'!$A$3:$T$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'29 Tech Media &amp; Gaming'!$A$3:$T$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'32 Defense &amp; Industrial AI'!$A$3:$T$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'33 Automation &amp; Robotics'!$A$3:$T$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'34 DC Power &amp; Cooling'!$A$3:$T$4</definedName>
@@ -658,7 +658,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Status: IN PROGRESS — verified 304 | kept 221 (55 Yes / 106 Stretch / 60 Low-value) | rejected 83 | pending 1457 | up-and-coming 102</t>
+          <t>Status: IN PROGRESS — verified 304 | kept 220 (55 Yes / 105 Stretch / 60 Low-value) | rejected 84 | pending 1457 | up-and-coming 102</t>
         </is>
       </c>
     </row>
@@ -1195,13 +1195,13 @@
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C34" s="4" t="n">
         <v>3</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E34" s="4" t="n">
         <v>3</v>
@@ -17215,7 +17215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T10"/>
+  <dimension ref="A1:T9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -17243,7 +17243,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>29 Tech Media &amp; Gaming — Wave 14 (v3) — 7 new brands: 3 Yes / 1 Stretch / 3 Low-value</t>
+          <t>29 Tech Media &amp; Gaming — Wave 14 (v3) — 6 new brands: 3 Yes / 0 Stretch / 3 Low-value</t>
         </is>
       </c>
     </row>
@@ -17645,98 +17645,98 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n">
+      <c r="A7" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="9" t="n">
-        <v>58</v>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>Krafton</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="B7" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Nippon Television Holdings</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>29 Tech Media &amp; Gaming</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>krafton.com</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>Seongnam, South Korea</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr">
-        <is>
-          <t>Publicly listed (KRX: 259960); founder-led (Chang Byung-gyu); Tencent a major minority holder (est)</t>
-        </is>
-      </c>
-      <c r="I7" s="9" t="inlineStr">
-        <is>
-          <t>PUBG: Battlegrounds / PUBG Mobile (co-developed with Tencent), inZOI, Subnautica, Dinkum</t>
-        </is>
-      </c>
-      <c r="J7" s="9" t="inlineStr">
-        <is>
-          <t>1k-5k (~1,684 at 30 Jun 2026; 2,119 Mar 2026 per Revelio; 271 left in Jan 2026 resignation programme)</t>
-        </is>
-      </c>
-      <c r="K7" s="9" t="inlineStr">
-        <is>
-          <t>KRW 3.3266T (~USD 2.4B) FY2025, +22.8%; operating profit KRW 1.0544T (Krafton press release, Feb 2026)</t>
-        </is>
-      </c>
-      <c r="L7" s="9" t="inlineStr">
-        <is>
-          <t>Market cap KRW 8.6T (~USD 6.35B) at 25 Sep 2026, -37.6% in 12 months (stockanalysis.com)</t>
-        </is>
-      </c>
-      <c r="M7" s="9" t="inlineStr">
-        <is>
-          <t>n/a (listed, profitable; USD 686M shareholder returns committed, Feb 2026)</t>
-        </is>
-      </c>
-      <c r="N7" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="O7" s="9" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>ntv.co.jp</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>Tokyo, Japan</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Publicly listed (TSE 9404)</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>TV network (NTV), Studio Ghibli stake, Hulu Japan, content and events</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>5k-10k</t>
+        </is>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>JPY 484.4B (~USD 3.07B at 158) FY2026, +4.9% (companiesmarketcap/edinetdb, searched Oct 2026)</t>
+        </is>
+      </c>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>Market cap JPY 712.0B (~USD 4.5B at 158), Oct 2026 (investing.com/companiesmarketcap)</t>
+        </is>
+      </c>
+      <c r="M7" s="10" t="inlineStr">
+        <is>
+          <t>n/a (listed; no raise found)</t>
+        </is>
+      </c>
+      <c r="N7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" s="10" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="P7" s="9" t="inlineStr">
-        <is>
-          <t>Stretch</t>
-        </is>
-      </c>
-      <c r="Q7" s="9" t="inlineStr">
-        <is>
-          <t>Passes hard filters on financials (market cap ~USD 6.35B, ~1.7-2.1k staff, operating profit KRW 1.05T, no sanctions). Reservation: confirmed repeated licensing collaborations with McLaren (2024-25) and Ferrari (Jul-Sep 2026), which are in-game collabs rather than team sponsorships or global partnerships; judged a flag, not a hard tie, but needs caller confirmation that these do not count as an F1 team partner tie.</t>
-        </is>
-      </c>
-      <c r="R7" s="9" t="inlineStr">
-        <is>
-          <t>Convert proven F1 in-game collab results into a paid partnership for PUBG or inZOI with a team not already collaborating (Williams, Racing Bulls, Haas, Audi, Cadillac) or a US race promoter (est).</t>
-        </is>
-      </c>
-      <c r="S7" s="9" t="inlineStr">
-        <is>
-          <t>existing F1 team collaborations (licensing, not sponsorship): PUBG Mobile x McLaren F1 in-game collab 22 Nov 2024-7 Jan 2025 (via SPORTFIVE release); PUBG Mobile x Ferrari/Scuderia Ferrari HP collab 10 Jul-8 Sep 2026 announced by Krafton; workforce reduction Jan 2026 (271 exits, voluntary programme) at a profitable company: cost programme; market cap -37.6% YoY; revenue concentrated in PUBG franchise</t>
-        </is>
-      </c>
-      <c r="T7" s="9" t="inlineStr">
-        <is>
-          <t>Markets 1 (global PUBG audience incl. US, Europe, Japan, Middle East); buyers 1 (gamers 18-34 plus senior industry decision makers); story 1 (technology/performance); category 0 (gaming/tech entertainment already well represented on grid).</t>
+      <c r="P7" s="10" t="inlineStr">
+        <is>
+          <t>Low-value</t>
+        </is>
+      </c>
+      <c r="Q7" s="10" t="inlineStr">
+        <is>
+          <t>Passes hard filters (mkt cap ~USD 4.5B, 5k+ staff, no F1 tie) but fit 1: domestic broadcaster with no international sales and rival Fuji TV owns the F1 relationship in Japan.</t>
+        </is>
+      </c>
+      <c r="R7" s="10" t="inlineStr">
+        <is>
+          <t>Ghibli/anime content partnership with an F1 team for Japanese-market fans only (est); low conversion likelihood</t>
+        </is>
+      </c>
+      <c r="S7" s="10" t="inlineStr">
+        <is>
+          <t>F1 Japan broadcast rights held by rival Fuji TV through 2030 (Fuji TV is a separate company, not a tie); headcount sources vary 5.9k-11.0k (parent vs group)</t>
+        </is>
+      </c>
+      <c r="T7" s="10" t="inlineStr">
+        <is>
+          <t>Markets 0 (domestic); buyers 0; story 0; category 1 (broadcaster not a grid sponsor category; note Fuji TV holds F1 Japan rights to 2030, separate group)</t>
         </is>
       </c>
     </row>
@@ -17749,7 +17749,7 @@
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>Nippon Television Holdings</t>
+          <t>Sankyo Co (pachinko)</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
@@ -17764,7 +17764,7 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>ntv.co.jp</t>
+          <t>sankyo-fever.co.jp</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -17774,32 +17774,32 @@
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>Publicly listed (TSE 9404)</t>
+          <t>Publicly listed (TSE 6417)</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
-          <t>TV network (NTV), Studio Ghibli stake, Hulu Japan, content and events</t>
+          <t>Pachinko and pachislot machines (Fever), ball-supply systems (Japan)</t>
         </is>
       </c>
       <c r="J8" s="10" t="inlineStr">
         <is>
-          <t>5k-10k</t>
+          <t>201-1k</t>
         </is>
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
-          <t>JPY 484.4B (~USD 3.07B at 158) FY2026, +4.9% (companiesmarketcap/edinetdb, searched Oct 2026)</t>
+          <t>JPY 179.2B FY2026 (~USD 1.2B at ~JPY150/USD (est)) (stockanalysis.com, searched Oct 2026)</t>
         </is>
       </c>
       <c r="L8" s="10" t="inlineStr">
         <is>
-          <t>Market cap JPY 712.0B (~USD 4.5B at 158), Oct 2026 (investing.com/companiesmarketcap)</t>
+          <t>Market cap JPY 382.3B (~USD 2.5B at ~JPY150/USD (est)) as of 12 Aug 2026 (stockanalysis.com)</t>
         </is>
       </c>
       <c r="M8" s="10" t="inlineStr">
         <is>
-          <t>n/a (listed; no raise found)</t>
+          <t>n/a (listed, cash-rich)</t>
         </is>
       </c>
       <c r="N8" s="10" t="n">
@@ -17817,22 +17817,22 @@
       </c>
       <c r="Q8" s="10" t="inlineStr">
         <is>
-          <t>Passes hard filters (mkt cap ~USD 4.5B, 5k+ staff, no F1 tie) but fit 1: domestic broadcaster with no international sales and rival Fuji TV owns the F1 relationship in Japan.</t>
+          <t>Passes hard filters (USD ~2.5B mkt cap; 886 staff; no distress; no F1 tie). Fit 1: gambling-adjacent Japan-only hall-equipment maker whose buyers are hall operators; F1 brand-safety and regulatory fit is poor.</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
         <is>
-          <t>Ghibli/anime content partnership with an F1 team for Japanese-market fans only (est); low conversion likelihood</t>
+          <t>None credible; at most Japanese GP hospitality for hall-operator customers (est).</t>
         </is>
       </c>
       <c r="S8" s="10" t="inlineStr">
         <is>
-          <t>F1 Japan broadcast rights held by rival Fuji TV through 2030 (Fuji TV is a separate company, not a tie); headcount sources vary 5.9k-11.0k (parent vs group)</t>
+          <t>gambling; Japan-only; B2B to pachinko hall operators; no F1 tie found; the F1 'Fever' partner (live-entertainment ticketing) is an unrelated company; employees 886 (hint 1,500 was high)</t>
         </is>
       </c>
       <c r="T8" s="10" t="inlineStr">
         <is>
-          <t>Markets 0 (domestic); buyers 0; story 0; category 1 (broadcaster not a grid sponsor category; note Fuji TV holds F1 Japan rights to 2030, separate group)</t>
+          <t>Markets 3+: 0 (Japan only). Affluent 25-54 / senior buyers: 0 (B2B sales to pachinko halls). Brand story: 0. Category untaken: 1.</t>
         </is>
       </c>
     </row>
@@ -17845,7 +17845,7 @@
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Sankyo Co (pachinko)</t>
+          <t>TBS Holdings</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -17860,7 +17860,7 @@
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>sankyo-fever.co.jp</t>
+          <t>tbsholdings.co.jp</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
@@ -17870,32 +17870,32 @@
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
-          <t>Publicly listed (TSE 6417)</t>
+          <t>Publicly listed (TSE 9401)</t>
         </is>
       </c>
       <c r="I9" s="10" t="inlineStr">
         <is>
-          <t>Pachinko and pachislot machines (Fever), ball-supply systems (Japan)</t>
+          <t>TV network (TBS), real estate (Akasaka), content and events</t>
         </is>
       </c>
       <c r="J9" s="10" t="inlineStr">
         <is>
-          <t>201-1k</t>
+          <t>5k-10k</t>
         </is>
       </c>
       <c r="K9" s="10" t="inlineStr">
         <is>
-          <t>JPY 179.2B FY2026 (~USD 1.2B at ~JPY150/USD (est)) (stockanalysis.com, searched Oct 2026)</t>
+          <t>JPY 424.85B (~USD 2.7B at 158) FY to 31 Mar 2026, record; operating profit JPY 24.75B (Globe and Mail/TipRanks, searched Oct 2026)</t>
         </is>
       </c>
       <c r="L9" s="10" t="inlineStr">
         <is>
-          <t>Market cap JPY 382.3B (~USD 2.5B at ~JPY150/USD (est)) as of 12 Aug 2026 (stockanalysis.com)</t>
+          <t>Market cap JPY 910.8B (~USD 5.8B at 158) (TipRanks report, 2026; companiesmarketcap USD 5.73B)</t>
         </is>
       </c>
       <c r="M9" s="10" t="inlineStr">
         <is>
-          <t>n/a (listed, cash-rich)</t>
+          <t>n/a (listed; no raise found)</t>
         </is>
       </c>
       <c r="N9" s="10" t="n">
@@ -17913,123 +17913,27 @@
       </c>
       <c r="Q9" s="10" t="inlineStr">
         <is>
-          <t>Passes hard filters (USD ~2.5B mkt cap; 886 staff; no distress; no F1 tie). Fit 1: gambling-adjacent Japan-only hall-equipment maker whose buyers are hall operators; F1 brand-safety and regulatory fit is poor.</t>
+          <t>Passes hard filters (mkt cap ~USD 5.8B, 8.5k staff, profitable, no F1 tie found) but fit 1: domestic broadcaster, no international consumer sales, Fuji TV holds F1 Japan rights.</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
-          <t>None credible; at most Japanese GP hospitality for hall-operator customers (est).</t>
+          <t>Global drama-format/content partnership with an F1 team (est); low conversion likelihood</t>
         </is>
       </c>
       <c r="S9" s="10" t="inlineStr">
         <is>
-          <t>gambling; Japan-only; B2B to pachinko hall operators; no F1 tie found; the F1 'Fever' partner (live-entertainment ticketing) is an unrelated company; employees 886 (hint 1,500 was high)</t>
+          <t>real estate arm; headcount sources vary 8.5k-16.6k (parent vs group)</t>
         </is>
       </c>
       <c r="T9" s="10" t="inlineStr">
         <is>
-          <t>Markets 3+: 0 (Japan only). Affluent 25-54 / senior buyers: 0 (B2B sales to pachinko halls). Brand story: 0. Category untaken: 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="10" t="n">
-        <v>24</v>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>TBS Holdings</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>29 Tech Media &amp; Gaming</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F10" s="10" t="inlineStr">
-        <is>
-          <t>tbsholdings.co.jp</t>
-        </is>
-      </c>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>Tokyo, Japan</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>Publicly listed (TSE 9401)</t>
-        </is>
-      </c>
-      <c r="I10" s="10" t="inlineStr">
-        <is>
-          <t>TV network (TBS), real estate (Akasaka), content and events</t>
-        </is>
-      </c>
-      <c r="J10" s="10" t="inlineStr">
-        <is>
-          <t>5k-10k</t>
-        </is>
-      </c>
-      <c r="K10" s="10" t="inlineStr">
-        <is>
-          <t>JPY 424.85B (~USD 2.7B at 158) FY to 31 Mar 2026, record; operating profit JPY 24.75B (Globe and Mail/TipRanks, searched Oct 2026)</t>
-        </is>
-      </c>
-      <c r="L10" s="10" t="inlineStr">
-        <is>
-          <t>Market cap JPY 910.8B (~USD 5.8B at 158) (TipRanks report, 2026; companiesmarketcap USD 5.73B)</t>
-        </is>
-      </c>
-      <c r="M10" s="10" t="inlineStr">
-        <is>
-          <t>n/a (listed; no raise found)</t>
-        </is>
-      </c>
-      <c r="N10" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" s="10" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="P10" s="10" t="inlineStr">
-        <is>
-          <t>Low-value</t>
-        </is>
-      </c>
-      <c r="Q10" s="10" t="inlineStr">
-        <is>
-          <t>Passes hard filters (mkt cap ~USD 5.8B, 8.5k staff, profitable, no F1 tie found) but fit 1: domestic broadcaster, no international consumer sales, Fuji TV holds F1 Japan rights.</t>
-        </is>
-      </c>
-      <c r="R10" s="10" t="inlineStr">
-        <is>
-          <t>Global drama-format/content partnership with an F1 team (est); low conversion likelihood</t>
-        </is>
-      </c>
-      <c r="S10" s="10" t="inlineStr">
-        <is>
-          <t>real estate arm; headcount sources vary 8.5k-16.6k (parent vs group)</t>
-        </is>
-      </c>
-      <c r="T10" s="10" t="inlineStr">
-        <is>
           <t>Markets 0 (domestic broadcaster, minor format exports); buyers 0; story 0; category 1 (not on grid)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:T10"/>
+  <autoFilter ref="A3:T9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -63506,7 +63410,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D86"/>
+  <dimension ref="A1:D87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -63518,7 +63422,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Failed a v3 hard filter — 83 names</t>
+          <t>Failed a v3 hard filter — 84 names</t>
         </is>
       </c>
     </row>
@@ -63701,12 +63605,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Substrate</t>
+          <t>Krafton</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>35 Semiconductor Equipment</t>
+          <t>29 Tech Media &amp; Gaming</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -63716,19 +63620,19 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 2 failed (headcount &gt;= 51): ~35 employees at 31 Mar 2026 per Tracxn, ~50 per Oct 2025 press, 'under 100' in other coverage; no source shows 51+. Valuation (USD ~1B+, Oct 2025) and funding otherwise pass; no F1 tie found.</t>
+          <t>F1 tie: PUBG Mobile ran official in-game collaborations with McLaren F1 (Nov 2024 to Jan 2025) and Scuderia Ferrari HP (Jul to Sep 2026). Existing commercial relationships with two current teams count as a tie under rule 4.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Verdiva Bio</t>
+          <t>Substrate</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>42 Health &amp; Wellness</t>
+          <t>35 Semiconductor Equipment</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -63738,19 +63642,19 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 failed: no published valuation above USD 1B (hint's 'USD 1B+' unsupported; USD 411M raise alone does not establish it) and pre-revenue passes only if valued &gt; USD 1B. Filter 2 also doubtful (41 employees per PitchBook).</t>
+          <t>Hard filter 2 failed (headcount &gt;= 51): ~35 employees at 31 Mar 2026 per Tracxn, ~50 per Oct 2025 press, 'under 100' in other coverage; no source shows 51+. Valuation (USD ~1B+, Oct 2025) and funding otherwise pass; no F1 tie found.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Tractian</t>
+          <t>Verdiva Bio</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>47 Vertical SaaS</t>
+          <t>42 Health &amp; Wellness</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -63760,36 +63664,36 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 failed (valuation &gt; USD 1B): latest priced round Series C Dec 2024 at USD 720M; no 2025-26 round or USD 1B+ valuation found. Headcount, capacity and F1-tie filters pass.</t>
+          <t>Hard filter 1 failed: no published valuation above USD 1B (hint's 'USD 1B+' unsupported; USD 411M raise alone does not establish it) and pre-revenue passes only if valued &gt; USD 1B. Filter 2 also doubtful (41 employees per PitchBook).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Eisler Capital</t>
+          <t>Tractian</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>X01 Asset Mgmt, PE &amp; Trading Fir</t>
+          <t>47 Vertical SaaS</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 3 (capacity to spend) failed: Eisler announced on 29 Sep 2025 it would shut its hedge fund after poor returns and high costs, estimated wind-down costs at 10-15% of NAV, and expected the portfolio fully unwound by 31 Dec 2025 (Reuters, Bloomberg, Hedgeweek). No F1 tie found.</t>
+          <t>Hard filter 1 failed (valuation &gt; USD 1B): latest priced round Series C Dec 2024 at USD 720M; no 2025-26 round or USD 1B+ valuation found. Headcount, capacity and F1-tie filters pass.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>FXTM (ForexTime)</t>
+          <t>Eisler Capital</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -63804,14 +63708,14 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Fails hard filter 1 (valuation): no published valuation, revenue not confirmed above $100M (UK entity only GBP 1.78M in 2024), so neither the &gt;$1B valuation nor the unpublished-valuation exception (revenue &gt;$1B or clear leader) is met. Headcount ~795-824 passes; prior Force India 2017 sponsorship noted as history, not a current tie (search 5 Oct 2026).</t>
+          <t>Hard filter 3 (capacity to spend) failed: Eisler announced on 29 Sep 2025 it would shut its hedge fund after poor returns and high costs, estimated wind-down costs at 10-15% of NAV, and expected the portfolio fully unwound by 31 Dec 2025 (Reuters, Bloomberg, Hedgeweek). No F1 tie found.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>HYCM</t>
+          <t>FXTM (ForexTime)</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -63826,14 +63730,14 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Fails hard filter 1 (valuation): no published valuation, revenue est $25-46M (2026), not a market leader, so no &gt;$1B pass or exception. No F1 tie found (search 5 Oct 2026).</t>
+          <t>Fails hard filter 1 (valuation): no published valuation, revenue not confirmed above $100M (UK entity only GBP 1.78M in 2024), so neither the &gt;$1B valuation nor the unpublished-valuation exception (revenue &gt;$1B or clear leader) is met. Headcount ~795-824 passes; prior Force India 2017 sponsorship noted as history, not a current tie (search 5 Oct 2026).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Maven Securities</t>
+          <t>HYCM</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -63848,14 +63752,14 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Fails hard filter 1 (valuation): privately held with no published valuation, and revenue (GBP 101M, FY Jun 2025) is far below USD 1B and Maven is not a clear market leader, so the unpublished-valuation exception does not apply. Headcount 236 (FY2025) and no F1 tie found (search 5 Oct 2026) pass.</t>
+          <t>Fails hard filter 1 (valuation): no published valuation, revenue est $25-46M (2026), not a market leader, so no &gt;$1B pass or exception. No F1 tie found (search 5 Oct 2026).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Old Mission Capital</t>
+          <t>Maven Securities</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -63870,14 +63774,14 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Fails hard filter 1 (valuation): privately held, no published valuation, revenue unverified and at best est $250-500M, well under the USD 1B revenue test and not a clear market leader. Headcount 268-286 (May-Aug 2026) passes; no F1 tie found (search 5 Oct 2026).</t>
+          <t>Fails hard filter 1 (valuation): privately held with no published valuation, and revenue (GBP 101M, FY Jun 2025) is far below USD 1B and Maven is not a clear market leader, so the unpublished-valuation exception does not apply. Headcount 236 (FY2025) and no F1 tie found (search 5 Oct 2026) pass.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>SBI Holdings</t>
+          <t>Old Mission Capital</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -63887,63 +63791,63 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>F1 tie: SBI Holdings became official presenting partner (media category) of the Las Vegas Grand Prix in June 2026. A Grand Prix partnership is a hard-filter tie under v3 rule 4.</t>
+          <t>Fails hard filter 1 (valuation): privately held, no published valuation, revenue unverified and at best est $250-500M, well under the USD 1B revenue test and not a clear market leader. Headcount 268-286 (May-Aug 2026) passes; no F1 tie found (search 5 Oct 2026).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Opendoor Technologies</t>
+          <t>SBI Holdings</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>X02 Real Estate &amp; Building Produ</t>
+          <t>X01 Asset Mgmt, PE &amp; Trading Fir</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Fails hard filter 3 (capacity to spend): Opendoor is in active cost-cutting/restructuring under 'Opendoor 2.0' (CEO Kaz Nejatian since Sept 2025): India operations closed and all 250 staff (18% of workforce) let go on 10 Jun 2026, AI-driven cost cuts, restructuring charges, targeting adjusted breakeven by end 2026; Q2 2026 net loss widened to $162M. Valuation (~$2.74B) and headcount (~1,040) pass and no F1 tie found (search 5 Oct 2026). No going-concern language found; cash is $896M.</t>
+          <t>F1 tie: SBI Holdings became official presenting partner (media category) of the Las Vegas Grand Prix in June 2026. A Grand Prix partnership is a hard-filter tie under v3 rule 4.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>ITM Radiopharma</t>
+          <t>Opendoor Technologies</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>X03 CDMO, CRO &amp; Life-Science Too</t>
+          <t>X02 Real Estate &amp; Building Produ</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Filter 4 (acquired/merged-away): Telix Pharmaceuticals agreed to acquire ITM on 21 Sep 2026 for USD 1.65B upfront; closing expected by end-2026. Acquirer: Telix. Other hard filters pass.</t>
+          <t>Fails hard filter 3 (capacity to spend): Opendoor is in active cost-cutting/restructuring under 'Opendoor 2.0' (CEO Kaz Nejatian since Sept 2025): India operations closed and all 250 staff (18% of workforce) let go on 10 Jun 2026, AI-driven cost cuts, restructuring charges, targeting adjusted breakeven by end 2026; Q2 2026 net loss widened to $162M. Valuation (~$2.74B) and headcount (~1,040) pass and no F1 tie found (search 5 Oct 2026). No going-concern language found; cash is $896M.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Resilience (National Resilience)</t>
+          <t>ITM Radiopharma</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -63953,19 +63857,19 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 3 (capacity to spend): company announced in late 2025 that six of ten sites are being wound down alongside repeated layoffs and a streamlined CDMO strategy supported by bridge financing (FiercePharma, PharmaManufacturing, 2025). Restructuring/wind-down pattern, despite the debt raise.</t>
+          <t>Filter 4 (acquired/merged-away): Telix Pharmaceuticals agreed to acquire ITM on 21 Sep 2026 for USD 1.65B upfront; closing expected by end-2026. Acquirer: Telix. Other hard filters pass.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Univercells</t>
+          <t>Resilience (National Resilience)</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -63980,19 +63884,19 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 4 (acquired/merged-away): Univercells Technologies was acquired by Donaldson Company on 29 June 2023 and is no longer independent. Also fails filter 1: deal value about USD 148M, far under USD 1B. Headcount about 100 at acquisition passes.</t>
+          <t>Hard filter 3 (capacity to spend): company announced in late 2025 that six of ten sites are being wound down alongside repeated layoffs and a streamlined CDMO strategy supported by bridge financing (FiercePharma, PharmaManufacturing, 2025). Restructuring/wind-down pattern, despite the debt raise.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Concord Resources</t>
+          <t>Univercells</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>X04 Mining, Metals &amp; Commodities</t>
+          <t>X03 CDMO, CRO &amp; Life-Science Too</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -64002,14 +63906,14 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 2 (headcount &gt;= 51): about 33 employees across three continents (LinkedIn-derived profile, Aug 2026; earlier Fastmarkets noted about 30 staff). Revenue is USD 4.2B so valuation exemption would have applied, but headcount fails.</t>
+          <t>Hard filter 4 (acquired/merged-away): Univercells Technologies was acquired by Donaldson Company on 29 June 2023 and is no longer independent. Also fails filter 1: deal value about USD 148M, far under USD 1B. Headcount about 100 at acquisition passes.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Lithium Americas</t>
+          <t>Concord Resources</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -64019,46 +63923,46 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 failed: listed company with market cap under USD 1B (USD 919M on 2 Oct 2026, stockanalysis.com; USD 663M on another aggregator).</t>
+          <t>Hard filter 2 (headcount &gt;= 51): about 33 employees across three continents (LinkedIn-derived profile, Aug 2026; earlier Fastmarkets noted about 30 staff). Revenue is USD 4.2B so valuation exemption would have applied, but headcount fails.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Gotham Greens</t>
+          <t>Lithium Americas</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>X05 Agriculture &amp; AgTech</t>
+          <t>X04 Mining, Metals &amp; Commodities</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B): best sourced estimate is USD 500M-1B (2022 Series E era; Dealroom/multiples.vc), no dated source confirms over USD 1B, and the company is VC-backed so the unpublished-valuation exemption does not apply.</t>
+          <t>Filter 1 failed: listed company with market cap under USD 1B (USD 919M on 2 Oct 2026, stockanalysis.com; USD 663M on another aggregator).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Floward</t>
+          <t>Gotham Greens</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>X06 Retail &amp; E-commerce</t>
+          <t>X05 Agriculture &amp; AgTech</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -64068,14 +63972,14 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B): best available EV estimate is USD 624-936M (2026 aggregator) and no sourced figure above USD 1B. If it is in fact listed, it is a listed company under USD 1B, which is also a No.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B): best sourced estimate is USD 500M-1B (2022 Series E era; Dealroom/multiples.vc), no dated source confirms over USD 1B, and the company is VC-backed so the unpublished-valuation exemption does not apply.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>GSF Car Parts (LKQ Euro)</t>
+          <t>Floward</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -64090,14 +63994,14 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B): no published valuation, and the unpublished-valuation exemption applies only to family/foundation/employee-owned firms or revenue above USD 1B or a clear market leader. GSF is PE-owned with revenue about GBP 480M and is not the market leader (Euro Car Parts is larger). Headcount (1,587) passes.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B): best available EV estimate is USD 624-936M (2026 aggregator) and no sourced figure above USD 1B. If it is in fact listed, it is a listed company under USD 1B, which is also a No.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Konga</t>
+          <t>GSF Car Parts (LKQ Euro)</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -64112,14 +64016,14 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B): last credible valuation USD 200M then USD 35M (BusinessDay), the USD 2B claim is unsubstantiated. Zinox ownership is private, so the exemption needs revenue over USD 1B or a clear market leader; Konga is neither (Jumia is larger).</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B): no published valuation, and the unpublished-valuation exemption applies only to family/foundation/employee-owned firms or revenue above USD 1B or a clear market leader. GSF is PE-owned with revenue about GBP 480M and is not the market leader (Euro Car Parts is larger). Headcount (1,587) passes.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Welcia Holdings</t>
+          <t>Konga</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -64129,41 +64033,41 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 4 (acquired/merged-away): Welcia Holdings became a wholly owned subsidiary of Tsuruha Holdings on 1 Dec 2025 and was delisted 27 Nov 2025. Approach Tsuruha Holdings instead if wanted.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B): last credible valuation USD 200M then USD 35M (BusinessDay), the USD 2B claim is unsubstantiated. Zinox ownership is private, so the exemption needs revenue over USD 1B or a clear market leader; Konga is neither (Jumia is larger).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Elliott Aviation</t>
+          <t>Welcia Holdings</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>X07 Aviation &amp; Aerospace Supplie</t>
+          <t>X06 Retail &amp; E-commerce</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: no published valuation, PE-owned (Summit Park), revenue ~$69M (Owler/IncFact 2026), not a clear market leader, so the no-published-valuation exemption does not apply. Headcount ~282-350 (May 2026) passes; no F1 tie found; no distress found.</t>
+          <t>Hard filter 4 (acquired/merged-away): Welcia Holdings became a wholly owned subsidiary of Tsuruha Holdings on 1 Dec 2025 and was delisted 27 Nov 2025. Approach Tsuruha Holdings instead if wanted.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Geven S.p.A</t>
+          <t>Elliott Aviation</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -64178,14 +64082,14 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: no published valuation, revenue ~EUR 52M (FY2024), niche player not a clear market leader. Headcount band 201-500 (LinkedIn/CB Insights) passes; no F1 tie found.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: no published valuation, PE-owned (Summit Park), revenue ~$69M (Owler/IncFact 2026), not a clear market leader, so the no-published-valuation exemption does not apply. Headcount ~282-350 (May 2026) passes; no F1 tie found; no distress found.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Jetex</t>
+          <t>Geven S.p.A</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -64200,14 +64104,14 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: privately held, no published valuation, revenue est $74-161M (2026), not a clear market leader (Signature/Atlantic larger). Headcount (~1.1K Jul 2026) passes; no F1 tie found.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: no published valuation, revenue ~EUR 52M (FY2024), niche player not a clear market leader. Headcount band 201-500 (LinkedIn/CB Insights) passes; no F1 tie found.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>STG Aerospace</t>
+          <t>Jetex</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -64222,14 +64126,14 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: PE-owned subsidiary of Heads Up Technologies (JLL Partners), no published valuation, revenue ~GBP 12M (FY2022). Headcount 68 passes; no F1 tie found.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: privately held, no published valuation, revenue est $74-161M (2026), not a clear market leader (Signature/Atlantic larger). Headcount (~1.1K Jul 2026) passes; no F1 tie found.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Vallair</t>
+          <t>STG Aerospace</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -64244,19 +64148,19 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: no published valuation, no verified revenue above $100M, not a clear market leader. Headcount 308 (2026) passes; no F1 tie found.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: PE-owned subsidiary of Heads Up Technologies (JLL Partners), no published valuation, revenue ~GBP 12M (FY2022). Headcount 68 passes; no F1 tie found.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Fitness First</t>
+          <t>Vallair</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>X08 Sporting Goods &amp; Fitness</t>
+          <t>X07 Aviation &amp; Aerospace Supplie</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -64266,14 +64170,14 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: family-owned (Whelan/Maddox Holdings), no published valuation, revenue ~GBP 38M (FY2024), not a clear market leader. Headcount 623 passes; no F1 tie found.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: no published valuation, no verified revenue above $100M, not a clear market leader. Headcount 308 (2026) passes; no F1 tie found.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Hydrow</t>
+          <t>Fitness First</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -64288,14 +64192,14 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: no current dated valuation above USD 1B (only a 2021 report; last round 2022 at $32M). Capacity (filter 3) is also doubtful: &gt;15% layoffs in 2022, no raise in 24+ months, revenue est $50-100M. No F1 tie found.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: family-owned (Whelan/Maddox Holdings), no published valuation, revenue ~GBP 38M (FY2024), not a clear market leader. Headcount 623 passes; no F1 tie found.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Lotto Sport Italia</t>
+          <t>Hydrow</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -64310,14 +64214,14 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation) failed: no published valuation, FY2024 revenue EUR 30.2M, not a clear market leader. Shrinking revenue is also noted but profitable in 2024, so filter 3 is not the failing filter.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: no current dated valuation above USD 1B (only a 2021 report; last round 2022 at $32M). Capacity (filter 3) is also doubtful: &gt;15% layoffs in 2022, no raise in 24+ months, revenue est $50-100M. No F1 tie found.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Momentous</t>
+          <t>Lotto Sport Italia</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -64332,14 +64236,14 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: VC/growth-backed with only $43.6M raised in total (latest $32M, 2022), no published valuation near USD 1B, revenue est $100-250M; no exemption route. Headcount ~89-94 passes; no F1 tie found.</t>
+          <t>Filter 1 (valuation) failed: no published valuation, FY2024 revenue EUR 30.2M, not a clear market leader. Shrinking revenue is also noted but profitable in 2024, so filter 3 is not the failing filter.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Rapha Racing</t>
+          <t>Momentous</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -64354,14 +64258,14 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: published carrying value GBP 67M (Oct 2025) after a GBP 102M impairment; family-owner exemption does not apply because a valuation is published and revenue is only GBP 89M. Note: capacity also doubtful (ninth loss year, shrinking revenue, job cuts) but the named failing filter is valuation. No F1 tie found.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: VC/growth-backed with only $43.6M raised in total (latest $32M, 2022), no published valuation near USD 1B, revenue est $100-250M; no exemption route. Headcount ~89-94 passes; no F1 tie found.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>TYR Sport</t>
+          <t>Rapha Racing</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -64376,14 +64280,14 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation) failed: private, no published valuation, revenue at most ~US$120M on credible estimates, and swimwear is not led by TYR (Speedo/Arena larger), so the exemption does not apply.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) FAILED: published carrying value GBP 67M (Oct 2025) after a GBP 102M impairment; family-owner exemption does not apply because a valuation is published and revenue is only GBP 89M. Note: capacity also doubtful (ninth loss year, shrinking revenue, job cuts) but the named failing filter is valuation. No F1 tie found.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Venum</t>
+          <t>TYR Sport</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -64398,19 +64302,19 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation) failed: private, no published valuation, revenue ~US$40M so nothing near USD 1B, and not a clear market leader by scale so the unpublished-valuation exemption does not apply. Filter 4 may also fail: Venum is listed among Ocon's brand ambassadorships (driver tie, one source, unconfirmed).</t>
+          <t>Filter 1 (valuation) failed: private, no published valuation, revenue at most ~US$120M on credible estimates, and swimwear is not led by TYR (Speedo/Arena larger), so the exemption does not apply.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Heesen Yachts</t>
+          <t>Venum</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>X09 Maritime, Shipping &amp; Ports</t>
+          <t>X08 Sporting Goods &amp; Fitness</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -64420,14 +64324,14 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation) failed: undisclosed acquisition price, revenue EUR 209M, and Heesen is not a clear global market leader (larger yards exist), so the unpublished-valuation exemption does not apply. Prior v2 audience-concentration ground is no longer a filter.</t>
+          <t>Filter 1 (valuation) failed: private, no published valuation, revenue ~US$40M so nothing near USD 1B, and not a clear market leader by scale so the unpublished-valuation exemption does not apply. Filter 4 may also fail: Venum is listed among Ocon's brand ambassadorships (driver tie, one source, unconfirmed).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Wajer Yachts</t>
+          <t>Heesen Yachts</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -64442,14 +64346,14 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation): no published valuation, family-owned but revenue ~EUR 100M (&lt;USD 1B) and not a clear global market leader, so the unpublished-valuation exemption does not apply. No F1 team/partner tie found (Wolff use is as a customer).</t>
+          <t>Filter 1 (valuation) failed: undisclosed acquisition price, revenue EUR 209M, and Heesen is not a clear global market leader (larger yards exist), so the unpublished-valuation exemption does not apply. Prior v2 audience-concentration ground is no longer a filter.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>ZeroNorth</t>
+          <t>Wajer Yachts</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -64464,19 +64368,19 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation) failed: venture/corporate-backed, no published valuation, ~US$73M raised and ARR ~US$40M, nothing indicates USD 1B; not a family/foundation-owned or clear global market leader.</t>
+          <t>Filter 1 (valuation): no published valuation, family-owned but revenue ~EUR 100M (&lt;USD 1B) and not a clear global market leader, so the unpublished-valuation exemption does not apply. No F1 team/partner tie found (Wolff use is as a customer).</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>AMP Robotics</t>
+          <t>ZeroNorth</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>X10 Batteries, EV, Waste &amp; Water</t>
+          <t>X09 Maritime, Shipping &amp; Ports</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -64486,14 +64390,14 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation): USD 457.7M post-money (Dec 2024) is below USD 1B, no later round or listing found. Prior hint's revenue/staleness reasons are not v3 filters; this is the real failure.</t>
+          <t>Filter 1 (valuation) failed: venture/corporate-backed, no published valuation, ~US$73M raised and ARR ~US$40M, nothing indicates USD 1B; not a family/foundation-owned or clear global market leader.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Ascend Elements</t>
+          <t>AMP Robotics</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -64508,14 +64412,14 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Filter 3 (capacity to spend): insolvency/winding-up - liquidating Chapter 11 plan effective 8 Sep 2026 (TechCrunch, Battery-News, docket sites). Filter 1 also fails (no operating valuation).</t>
+          <t>Filter 1 (valuation): USD 457.7M post-money (Dec 2024) is below USD 1B, no later round or listing found. Prior hint's revenue/staleness reasons are not v3 filters; this is the real failure.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Factorial Energy</t>
+          <t>Ascend Elements</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -64530,14 +64434,14 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation): listed company, market cap ~USD 664M (29 Sep 2026) is below USD 1B. The ~USD 1.3B SPAC valuation (Jun 2026) has not held.</t>
+          <t>Filter 3 (capacity to spend): insolvency/winding-up - liquidating Chapter 11 plan effective 8 Sep 2026 (TechCrunch, Battery-News, docket sites). Filter 1 also fails (no operating valuation).</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Lunar Energy</t>
+          <t>Factorial Energy</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -64547,19 +64451,19 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) failed: only dated valuation is USD 452M post-money (PitchBook, Feb 2026); no credible source above USD 1B.</t>
+          <t>Filter 1 (valuation): listed company, market cap ~USD 664M (29 Sep 2026) is below USD 1B. The ~USD 1.3B SPAC valuation (Jun 2026) has not held.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Monta</t>
+          <t>Lunar Energy</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -64569,19 +64473,19 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation): estimated ~USD 323M, no round or listing at or above USD 1B found. Revenue/staleness reasons in the hint are not v3 filters.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) failed: only dated valuation is USD 452M post-money (PitchBook, Feb 2026); no credible source above USD 1B.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Moxion Power</t>
+          <t>Monta</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -64596,14 +64500,14 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Filter 3 (capacity to spend): ceased operations 26 Jul 2024 and filed Chapter 7 liquidation (Law360, Latitude Media); also fails Filter 2 (no operating headcount) and Filter 1.</t>
+          <t>Filter 1 (valuation): estimated ~USD 323M, no round or listing at or above USD 1B found. Revenue/staleness reasons in the hint are not v3 filters.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Terawatt Infrastructure</t>
+          <t>Moxion Power</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -64618,14 +64522,14 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation): no dated, published valuation above USD 1B; only unverified aggregator estimates, and the unpublished-valuation exemption covers only family/foundation/employee-owned firms with revenue &gt; USD 1B or clear leaders. If the USD 4-6B estimate is accepted this would be Low-value (fit 1, US-only).</t>
+          <t>Filter 3 (capacity to spend): ceased operations 26 Jul 2024 and filed Chapter 7 liquidation (Law360, Latitude Media); also fails Filter 2 (no operating headcount) and Filter 1.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Virta</t>
+          <t>Terawatt Infrastructure</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -64640,19 +64544,19 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation): no published valuation and funding history (~USD 141M total) implies well under USD 1B; family/leader exemption does not apply. Hint's revenue reasoning is not a v3 filter.</t>
+          <t>Filter 1 (valuation): no dated, published valuation above USD 1B; only unverified aggregator estimates, and the unpublished-valuation exemption covers only family/foundation/employee-owned firms with revenue &gt; USD 1B or clear leaders. If the USD 4-6B estimate is accepted this would be Low-value (fit 1, US-only).</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>ENSCO Rail</t>
+          <t>Virta</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>X12 Rail, Transit &amp; Road Infra</t>
+          <t>X10 Batteries, EV, Waste &amp; Water</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -64662,19 +64566,19 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation): privately held, no published valuation, revenue well under USD 1B and not a clear global market leader. Would otherwise be Low-value (pure B2B, concentrated customers, no brand ambition).</t>
+          <t>Filter 1 (valuation): no published valuation and funding history (~USD 141M total) implies well under USD 1B; family/leader exemption does not apply. Hint's revenue reasoning is not a v3 filter.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>C&amp;H Distributors</t>
+          <t>ENSCO Rail</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>X13 Industrial &amp; MRO Distributio</t>
+          <t>X12 Rail, Transit &amp; Road Infra</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -64684,14 +64588,14 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) failed: no published valuation, ~USD 72M revenue, not a market leader, subsidiary of K+K America. Headcount ~88 passes; no F1 tie. Earlier revenue-bar reason is obsolete in v3; this No rests on valuation.</t>
+          <t>Filter 1 (valuation): privately held, no published valuation, revenue well under USD 1B and not a clear global market leader. Would otherwise be Low-value (pure B2B, concentrated customers, no brand ambition).</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Contorion</t>
+          <t>C&amp;H Distributors</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -64706,14 +64610,14 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Acquired company: owned by Hoffmann SE (Hoffmann Group) since June 2017, so no longer independent. Also fails hard filter 1: last valuation EUR 100M (2017), revenue ~USD 64M. Headcount 185+ passes; no F1 tie found for Contorion or Hoffmann.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) failed: no published valuation, ~USD 72M revenue, not a market leader, subsidiary of K+K America. Headcount ~88 passes; no F1 tie. Earlier revenue-bar reason is obsolete in v3; this No rests on valuation.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Essendant</t>
+          <t>Contorion</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -64728,14 +64632,14 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Fails hard filter 3 (capacity to spend). Essendant is winding down its core office-products business and independent-dealer channel (trade press, 4 Sept 2025); WARN filings 3 Aug 2026 cover Lincolnshire HQ and Carol Stream DC, layoffs of at least 1,100, and the company has warned it may cease operations (MDM / Lake McHenry Scanner, Sept 2026); Illinois opened a layoffs investigation (Sept 2026). Headcount 2,466 at 30 Jun 2026 (search result, 2026) and no F1 tie found (search 5 Oct 2026).</t>
+          <t>Acquired company: owned by Hoffmann SE (Hoffmann Group) since June 2017, so no longer independent. Also fails hard filter 1: last valuation EUR 100M (2017), revenue ~USD 64M. Headcount 185+ passes; no F1 tie found for Contorion or Hoffmann.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Womack Machine Supply</t>
+          <t>Essendant</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -64750,19 +64654,19 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Acquired/rebranded company: Womack Machine Supply was bought by Platte River Equity in 2023 and now trades as Evolution Motion Solutions. Also fails hard filter 1: no published valuation, revenue ~USD 51M (est), not a market leader. Headcount passes; no F1 tie.</t>
+          <t>Fails hard filter 3 (capacity to spend). Essendant is winding down its core office-products business and independent-dealer channel (trade press, 4 Sept 2025); WARN filings 3 Aug 2026 cover Lincolnshire HQ and Carol Stream DC, layoffs of at least 1,100, and the company has warned it may cease operations (MDM / Lake McHenry Scanner, Sept 2026); Illinois opened a layoffs investigation (Sept 2026). Headcount 2,466 at 30 Jun 2026 (search result, 2026) and no F1 tie found (search 5 Oct 2026).</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Electromech Material Handling Systems</t>
+          <t>Womack Machine Supply</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>X14 Intralogistics &amp; Warehouse A</t>
+          <t>X13 Industrial &amp; MRO Distributio</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -64772,14 +64676,14 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) failed: no published valuation, revenue ~USD 95M, family/promoter-owned and not a verified clear market leader so the unpublished-valuation pass does not apply. Headcount ~317 passes; capacity fine; no F1 tie.</t>
+          <t>Acquired/rebranded company: Womack Machine Supply was bought by Platte River Equity in 2023 and now trades as Evolution Motion Solutions. Also fails hard filter 1: no published valuation, revenue ~USD 51M (est), not a market leader. Headcount passes; no F1 tie.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Falcon Autotech</t>
+          <t>Electromech Material Handling Systems</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -64794,14 +64698,14 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) failed: USD 97.8M valuation (PitchBook 2026). Headcount ~625 passes; capacity not treated as a fail (no distress evidence); no F1 tie.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) failed: no published valuation, revenue ~USD 95M, family/promoter-owned and not a verified clear market leader so the unpublished-valuation pass does not apply. Headcount ~317 passes; capacity fine; no F1 tie.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Grupo CLN</t>
+          <t>Falcon Autotech</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -64816,19 +64720,19 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) cannot be met: no valuation, revenue or verifiable company identity found. Headcount also unverified. This is an evidence failure, not a confirmed small company; re-open only if the legal entity is identified.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) failed: USD 97.8M valuation (PitchBook 2026). Headcount ~625 passes; capacity not treated as a fail (no distress evidence); no F1 tie.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>FiiO Electronics</t>
+          <t>Grupo CLN</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>X15 Consumer Electronics &amp; Audio</t>
+          <t>X14 Intralogistics &amp; Warehouse A</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -64838,14 +64742,14 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) failed: no published valuation, ~USD 22M revenue, niche brand, founder-owned so unpublished-valuation pass does not apply. No F1 tie; HQ China not sanctioned.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) cannot be met: no valuation, revenue or verifiable company identity found. Headcount also unverified. This is an evidence failure, not a confirmed small company; re-open only if the legal entity is identified.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>HMD Global</t>
+          <t>FiiO Electronics</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -64860,14 +64764,14 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B): only published figure is USD 1B from 2018, not above the bar and not re-confirmed since; not family/foundation-owned so the no-valuation exception does not apply. Filter 3 (capacity) does NOT fail: US exit is a market refocus, no distress evidence. Filters 2, 4, 5 pass. Reopen if a current post-money above USD 1B is shown.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) failed: no published valuation, ~USD 22M revenue, niche brand, founder-owned so unpublished-valuation pass does not apply. No F1 tie; HQ China not sanctioned.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Lenbrook Industries (Bluesound/NAD)</t>
+          <t>HMD Global</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -64882,14 +64786,14 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B): private, no published valuation, est. revenue USD 26-42M, not a market leader, so the unpublished-valuation exception (revenue &gt; USD 1B or clear leader) fails. Headcount (192) passes; no distress, F1 tie or sanctions issue.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B): only published figure is USD 1B from 2018, not above the bar and not re-confirmed since; not family/foundation-owned so the no-valuation exception does not apply. Filter 3 (capacity) does NOT fail: US exit is a market refocus, no distress evidence. Filters 2, 4, 5 pass. Reopen if a current post-money above USD 1B is shown.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Native Union</t>
+          <t>Lenbrook Industries (Bluesound/NAD)</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -64904,14 +64808,14 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B): no valuation, revenue ~USD 28M, not a market leader. Headcount is also borderline (47-65, conflicting sources).</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B): private, no published valuation, est. revenue USD 26-42M, not a market leader, so the unpublished-valuation exception (revenue &gt; USD 1B or clear leader) fails. Headcount (192) passes; no distress, F1 tie or sanctions issue.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Satechi</t>
+          <t>Native Union</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -64926,14 +64830,14 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B): aggregator valuation USD 22.4M, revenue well under USD 100M, not a market leader. Headcount 70 passes.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B): no valuation, revenue ~USD 28M, not a market leader. Headcount is also borderline (47-65, conflicting sources).</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Skullcandy</t>
+          <t>Satechi</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -64948,14 +64852,14 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) failed: last mark USD 196.6M (Oct 2016 buyout), no later valuation, revenue ~USD 79M. Headcount ~327-344 passes; no current F1 tie (historic Force India deal only).</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B): aggregator valuation USD 22.4M, revenue well under USD 100M, not a market leader. Headcount 70 passes.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Teenage Engineering</t>
+          <t>Skullcandy</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -64970,14 +64874,14 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B) failed: ~SEK 1.5B (~USD 140M) valuation (Jan 2023), revenue ~USD 23-27M. Headcount ~116 passes; no distress evidence; no F1 tie.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) failed: last mark USD 196.6M (Oct 2016 buyout), no later valuation, revenue ~USD 79M. Headcount ~327-344 passes; no current F1 tie (historic Force India deal only).</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Xtorm</t>
+          <t>Teenage Engineering</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -64992,19 +64896,19 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B): unfunded private company, no valuation, revenue USD 5-8M, not a market leader. Headcount 65 passes.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B) failed: ~SEK 1.5B (~USD 140M) valuation (Jan 2023), revenue ~USD 23-27M. Headcount ~116 passes; no distress evidence; no F1 tie.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Bardahl</t>
+          <t>Xtorm</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>X16 Specialty Chemicals &amp; Coatin</t>
+          <t>X15 Consumer Electronics &amp; Audio</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -65014,14 +64918,14 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B): family-owned with no published valuation; the exception requires revenue &gt; USD 1B or clear market leader, and revenue is est. USD 22-69M. Headcount is also uncertain.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B): unfunded private company, no valuation, revenue USD 5-8M, not a market leader. Headcount 65 passes.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Master Bond Inc</t>
+          <t>Bardahl</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -65036,14 +64940,14 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 2 (headcount &gt;= 51): 21-27 employees. Hard filter 1 (valuation &gt; USD 1B) also fails: private, no valuation, small revenue.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B): family-owned with no published valuation; the exception requires revenue &gt; USD 1B or clear market leader, and revenue is est. USD 22-69M. Headcount is also uncertain.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Millers Oils</t>
+          <t>Master Bond Inc</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -65058,14 +64962,14 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 1 (valuation &gt; USD 1B): family/trust/employee-owned, no published valuation, turnover ~GBP 30.6M, not a clear market leader, so the exception fails. Headcount (~93) passes.</t>
+          <t>Hard filter 2 (headcount &gt;= 51): 21-27 employees. Hard filter 1 (valuation &gt; USD 1B) also fails: private, no valuation, small revenue.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Nippon Bee Chemical</t>
+          <t>Millers Oils</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -65080,14 +64984,14 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 4 (acquired/merged-away): Nippon Bee Chemical is a wholly owned Nippon Paint Holdings subsidiary (since 2006), now operating as Nippon Paint Automotive Coatings; acquirer is Nippon Paint Holdings. Separately, entity headcount is unverified. The parent group (market cap ~USD 15.5B, no F1 tie found) is the right unit to consider, not this entity.</t>
+          <t>Hard filter 1 (valuation &gt; USD 1B): family/trust/employee-owned, no published valuation, turnover ~GBP 30.6M, not a clear market leader, so the exception fails. Headcount (~93) passes.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Penrite Oil</t>
+          <t>Nippon Bee Chemical</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -65102,14 +65006,14 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation &gt; USD 1B) failed: family-owned, no published valuation, revenue ~USD 53-84M est (far below USD 1B) and not a clear market leader, so the no-published-valuation exemption does not apply. Headcount 96-146 passes; no F1 tie found.</t>
+          <t>Hard filter 4 (acquired/merged-away): Nippon Bee Chemical is a wholly owned Nippon Paint Holdings subsidiary (since 2006), now operating as Nippon Paint Automotive Coatings; acquirer is Nippon Paint Holdings. Separately, entity headcount is unverified. The parent group (market cap ~USD 15.5B, no F1 tie found) is the right unit to consider, not this entity.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Red Line Synthetic Oil</t>
+          <t>Penrite Oil</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -65124,19 +65028,19 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation &gt; USD 1B) failed: no standalone valuation, controlled by Phillips 66, revenue small and not &gt; USD 1B, not a clear market leader (exemption is for family/foundation/employee-owned only). Headcount ~95 passes; no F1 tie found.</t>
+          <t>Filter 1 (valuation &gt; USD 1B) failed: family-owned, no published valuation, revenue ~USD 53-84M est (far below USD 1B) and not a clear market leader, so the no-published-valuation exemption does not apply. Headcount 96-146 passes; no F1 tie found.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>GigSky</t>
+          <t>Red Line Synthetic Oil</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>X17 Private 5G &amp; Telecom Equipme</t>
+          <t>X16 Specialty Chemicals &amp; Coatin</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -65146,14 +65050,14 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation &gt; USD 1B) failed: estimated ~USD 163M (StartupHub, 2026), total funding ~USD 25-41M. Also weak on capacity to spend USD 2.5M/yr against ~USD 10M revenue (not scored as a fail). Headcount 61 passes; no F1 tie.</t>
+          <t>Filter 1 (valuation &gt; USD 1B) failed: no standalone valuation, controlled by Phillips 66, revenue small and not &gt; USD 1B, not a clear market leader (exemption is for family/foundation/employee-owned only). Headcount ~95 passes; no F1 tie found.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Highway9 Networks</t>
+          <t>GigSky</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -65168,14 +65072,14 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation &gt; USD 1B) failed: only USD 25M raised (Series B Feb 2024), no valuation near USD 1B. Capacity to spend USD 2.5M/yr also doubtful (revenue ~USD 1.5M; funding outside 24 months), and headcount is unconfirmed (20 vs 56).</t>
+          <t>Filter 1 (valuation &gt; USD 1B) failed: estimated ~USD 163M (StartupHub, 2026), total funding ~USD 25-41M. Also weak on capacity to spend USD 2.5M/yr against ~USD 10M revenue (not scored as a fail). Headcount 61 passes; no F1 tie.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Lycamobile</t>
+          <t>Highway9 Networks</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -65190,14 +65094,14 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Fails hard filter 3 (capacity to spend). PKF Littlejohn could not obtain sufficient audit evidence to sign off accounts, with going-concern doubt noted; HMRC won GBP 51M VAT tribunal and issued a winding-up petition (Aug 2024); loss-making and restructuring with up to 316 UK roles at risk, services moving to India (Dec 2024 reports, Lyca Group restructuring). Also fails filter 1 as no published valuation and no evidence of &gt;$1B revenue or clear market leadership. No F1 tie found (search 5 Oct 2026).</t>
+          <t>Filter 1 (valuation &gt; USD 1B) failed: only USD 25M raised (Series B Feb 2024), no valuation near USD 1B. Capacity to spend USD 2.5M/yr also doubtful (revenue ~USD 1.5M; funding outside 24 months), and headcount is unconfirmed (20 vs 56).</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Lynk Global</t>
+          <t>Lycamobile</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -65212,14 +65116,14 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation &gt; USD 1B) failed: no dated, sourced valuation above USD 1B found; last published USD 800-913.5M (2023-24) and Elveo terms undisclosed. Pre-revenue only passes if valued &gt; USD 1B. Headcount 87 passes; no F1 tie found. Reopen if a USD 1B+ valuation is documented for Elveo Mobile.</t>
+          <t>Fails hard filter 3 (capacity to spend). PKF Littlejohn could not obtain sufficient audit evidence to sign off accounts, with going-concern doubt noted; HMRC won GBP 51M VAT tribunal and issued a winding-up petition (Aug 2024); loss-making and restructuring with up to 316 UK roles at risk, services moving to India (Dec 2024 reports, Lyca Group restructuring). Also fails filter 1 as no published valuation and no evidence of &gt;$1B revenue or clear market leadership. No F1 tie found (search 5 Oct 2026).</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Red Pocket Mobile</t>
+          <t>Lynk Global</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -65234,14 +65138,14 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation &gt; USD 1B) failed: private, no published valuation, revenue est USD 5-50M and not a clear leader. Headcount 73-81 passes; no F1 tie found.</t>
+          <t>Filter 1 (valuation &gt; USD 1B) failed: no dated, sourced valuation above USD 1B found; last published USD 800-913.5M (2023-24) and Elveo terms undisclosed. Pre-revenue only passes if valued &gt; USD 1B. Headcount 87 passes; no F1 tie found. Reopen if a USD 1B+ valuation is documented for Elveo Mobile.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Tello Mobile</t>
+          <t>Red Pocket Mobile</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -65256,19 +65160,19 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation &gt; USD 1B) failed: private, no published valuation, revenue ~USD 15M est, not a clear leader. Filter 2 (headcount &gt;= 51) is also unconfirmed (23-51 across sources). No F1 tie.</t>
+          <t>Filter 1 (valuation &gt; USD 1B) failed: private, no published valuation, revenue est USD 5-50M and not a clear leader. Headcount 73-81 passes; no F1 tie found.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Lake Shore Cryotronics</t>
+          <t>Tello Mobile</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>X18 Quantum Computing</t>
+          <t>X17 Private 5G &amp; Telecom Equipme</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -65278,14 +65182,14 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation &gt; USD 1B) failed: no published valuation, revenue est USD 24-72M, not a clear leader, and the company is now a unit of DwyerOmega (Arcline) (acquirer named per filter 4). Headcount 157-266 passes; no F1 tie.</t>
+          <t>Filter 1 (valuation &gt; USD 1B) failed: private, no published valuation, revenue ~USD 15M est, not a clear leader. Filter 2 (headcount &gt;= 51) is also unconfirmed (23-51 across sources). No F1 tie.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Oratomic</t>
+          <t>Lake Shore Cryotronics</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -65295,76 +65199,98 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>FAILS hard filter 2 (headcount &gt;= 51): best evidence is 11-50 FTEs (Quantum Insider, Jul 2026); no source confirms &gt;= 51. Valuation (USD 1.5B, secondary source) and funding (USD 300M Jul 2026) would otherwise pass.</t>
+          <t>Filter 1 (valuation &gt; USD 1B) failed: no published valuation, revenue est USD 24-72M, not a clear leader, and the company is now a unit of DwyerOmega (Arcline) (acquirer named per filter 4). Headcount 157-266 passes; no F1 tie.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Mannai Corporation (Damas)</t>
+          <t>Oratomic</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>X21 Watches &amp; Jewellery</t>
+          <t>X18 Quantum Computing</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Filter 1 (valuation &gt; USD 1B) failed: listed company with market cap ~USD 0.64B (Oct 2026). Royal/state ownership is only a flag under v3 and was not used for the No. Headcount 21,000 and revenue ~USD 1.4B pass; no F1 tie.</t>
+          <t>FAILS hard filter 2 (headcount &gt;= 51): best evidence is 11-50 FTEs (Quantum Insider, Jul 2026); no source confirms &gt;= 51. Valuation (USD 1.5B, secondary source) and funding (USD 300M Jul 2026) would otherwise pass.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Teamworks</t>
+          <t>Mannai Corporation (Damas)</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>X35 Sports Tech &amp; Fan Engagement</t>
+          <t>X21 Watches &amp; Jewellery</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Hard filter 4 failed: confirmed partnership with the Aston Martin Aramco F1 Team (Teamworks blog, 5 Feb 2024; software supplier relationship) plus More than Equal F1 driver programme.</t>
+          <t>Filter 1 (valuation &gt; USD 1B) failed: listed company with market cap ~USD 0.64B (Oct 2026). Royal/state ownership is only a flag under v3 and was not used for the No. Headcount 21,000 and revenue ~USD 1.4B pass; no F1 tie.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
+          <t>Teamworks</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>X35 Sports Tech &amp; Fan Engagement</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Hard filter 4 failed: confirmed partnership with the Aston Martin Aramco F1 Team (Teamworks blog, 5 Feb 2024; software supplier relationship) plus More than Equal F1 driver programme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
           <t>Uzbekistan National Investment Fund (UzNIF)</t>
         </is>
       </c>
-      <c r="B86" s="2" t="inlineStr">
+      <c r="B87" s="2" t="inlineStr">
         <is>
           <t>X39 Central Asia &amp; Caucasus Champions</t>
         </is>
       </c>
-      <c r="C86" s="2" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr">
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
         <is>
           <t>Filter 2 (headcount &gt;=51) failed/unverifiable: UzNIF is a trustee-managed holding fund with minority stakes and no evidence of 51+ own employees; also state-linked with no consumer brand or marketing function. Valuation (USD 1.95B IPO, 2026) and capacity would otherwise pass; no F1 tie found.</t>
         </is>

</xml_diff>